<commit_message>
Fill the test sheet's score columns from a rater's file
The two score columns are copied from data/eval/network_test_scores.json,
one rater's reading of all 110 answers against the book, with the note
that decided each. The sheet tabs are rewritten whole on every run, so
the file, not the sheet, is where a score lives.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/eval/แบบทดสอบแชทบอทเครือข่าย.xlsx
+++ b/data/eval/แบบทดสอบแชทบอทเครือข่าย.xlsx
@@ -79,11 +79,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -93,6 +94,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -470,6 +474,7 @@
     <col width="90" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
@@ -505,42 +510,47 @@
           <t>ประเมิน RAG</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>หมายเหตุผู้ประเมิน</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>คำถามตรง ตอบตรง</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>คำถามตรง ตอบไม่ตรง</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>ระดับ</t>
         </is>
       </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>เกณฑ์</t>
         </is>
       </c>
-      <c r="N1" s="5" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>คะแนน</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>จงอธิบายความแตกต่างระหว่างการสื่อสารโทรศัพท์แบบทั่วไป กับแบบ VoIP</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>การสื่อสารโทรศัพท์แบบทั่วไปใช้ระบบ PSTN (Public Switched Telephony Network) ที่ส่งสัญญาณเสียงในรูปแบบแอนะล็อกผ่านสายทองแดง โดยใช้การเชื่อมต่อแบบเซอร์กิต (Circuit Switching) ซึ่งต้องมีการจองช่องทางการสื่อสารตลอดเวลาที่ใช้พูดคุย
 การสื่อสารแบบ VoIP (Voice Over Internet Protocol) ใช้การแปลงเสียงให้เป็นข้อมูลดิจิตอลแล้วบรรจุลงในแพ็กเก็ตข้อมูล เพื่อส่งผ่านเครือข่ายอินเทอร์เน็ตโดยใช้การส่งแบบแพ็กเก็ต (Packet Switching) ทำให้ประหยัดค่าใช้จ่าย โดยเฉพาะการโทรข้ามประเทศ (บทที่ 1 หน้า 12-13)
@@ -549,48 +559,57 @@
 การสื่อสารด้วย VoIP ต้องอาศัยอินเทอร์เน็ตที่มีความเร็วและเสถียรพอสมควร ขณะที่ระบบโทรศัพท์แบบทั่วไปไม่ต้องพึ่งพาอินเทอร์เน็ต (บทที่ 1 หน้า 28)</t>
         </is>
       </c>
-      <c r="D2" s="7" t="n"/>
-      <c r="E2" s="8" t="n"/>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="D2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>ใจความตรงกับ net-1-3 ถึง net-1-5 (หน้า 12-15) แต่เรื่อง Circuit/Packet Switching การจองช่องทาง และข้อความที่อ้างหน้า 28 ไม่มีในตำรา</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>ประเมินค่าความถูกต้อง</t>
         </is>
       </c>
-      <c r="H2" s="4">
+      <c r="H2" s="5">
         <f>COUNTIF(D2:D100,1)</f>
         <v/>
       </c>
-      <c r="I2" s="4">
+      <c r="I2" s="5">
         <f>COUNTIF(D2:D100,0)</f>
         <v/>
       </c>
-      <c r="K2" s="9" t="inlineStr">
+      <c r="K2" s="11" t="inlineStr">
         <is>
           <t>ประเมิน RAG and LLM</t>
         </is>
       </c>
-      <c r="L2" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="M2" s="10" t="inlineStr">
+      <c r="L2" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="M2" s="12" t="inlineStr">
         <is>
           <t>คำตอบถูกต้องและครบถ้วนตามเนื้อหาในตำรา</t>
         </is>
       </c>
-      <c r="N2" s="10" t="n">
+      <c r="N2" s="12" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>ระบบโทรศัพท์แบบ VoIP ช่วยลดค่าใช้จ่ายในด้านการสื่อสารระหว่างประเทศ อยากทราบว่าช่วยลดค่าใช้จ่ายได้อย่างไร จงอธิบาย</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>ระบบโทรศัพท์แบบ VoIP ช่วยลดค่าใช้จ่ายในการสื่อสารระหว่างประเทศได้ เพราะสามารถส่งข้อมูลเสียงผ่านเครือข่ายอินเทอร์เน็ตแทนการใช้เครือข่ายโทรศัพท์สาธารณะ (PSTN) ที่มีค่าบริการสูง โดยเฉพาะการโทรข้ามประเทศ (บทที่ 1 หน้า 14)
 เทคโนโลยี VoIP ใช้การบรรจุสัญญาณเสียงลงในรูปแบบของแพ็กเก็ตข้อมูลและส่งผ่านเร้าเตอร์ ทำให้ไม่ต้องพึ่งพาโครงข่ายโทรศัพท์เฉพาะทางที่มีต้นทุนสูง (บทที่ 1 หน้า 12-13)
@@ -600,30 +619,39 @@
 ระบบ VoIP ใช้โครงข่ายอินเทอร์เน็ตที่มีการแบ่งปันทรัพยากรร่วมกัน จึงไม่ต้องเสียค่าใช้จ่ายเพิ่มเติมสำหรับการเชื่อมต่อข้ามประเทศเหมือนกับระบบ PSTN ที่มีการเรียกเก็บค่าบริการตามระยะทาง</t>
         </is>
       </c>
-      <c r="D3" s="7" t="n"/>
-      <c r="E3" s="8" t="n"/>
-      <c r="L3" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M3" s="10" t="inlineStr">
+      <c r="D3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>ตรงกับ net-1-4 หน้า 14 ที่ว่า VoIP ส่งเสียงผ่านอินเทอร์เน็ตโดยไม่ต้องผ่าน PSTN ที่ค่าบริการสูงกว่า</t>
+        </is>
+      </c>
+      <c r="L3" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="12" t="inlineStr">
         <is>
           <t>คำตอบถูกต้องบางส่วน แต่ข้อมูลไม่ครบ</t>
         </is>
       </c>
-      <c r="N3" s="10" t="n">
+      <c r="N3" s="12" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>จงบอกข้อเสียของระบบ VolP</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>ข้อเสียของระบบ VoIP คือ ความสามารถในการส่งข้อมูลแบบเรียลไทม์อาจลดลง เนื่องจากแพ็กเก็ตข้อมูลที่ส่งจากต้นทางไปยังปลายทางต้องผ่านเครือข่ายอินเทอร์เน็ตที่มีจำนวนเครือข่ายมากมายมหาศาล ทำให้เกิดการดีเลย์หรือความล่าช้าในการสื่อสารได้ (บทที่ 1 หน้า 14-15)
 การสื่อสารข้อมูลด้วย VoIP อาจไม่เกิดขึ้นทันทีทันใดเหมือนการใช้โทรศัพท์แบบดั้งเดิม เนื่องจากการส่งผ่านข้อมูลผ่านเครือข่ายอินเทอร์เน็ตที่มีความซับซ้อน (บทที่ 1 หน้า 28-29)
@@ -631,30 +659,39 @@
 ข้อเสียอีกประการหนึ่งอาจเกิดจากความเสถียรของอินเทอร์เน็ต เช่น หากความเร็วหรือความหนาแน่นของเครือข่ายต่ำ อาจทำให้เสียงขาดหรือมีเสียงรบกวนได้</t>
         </is>
       </c>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="8" t="n"/>
-      <c r="L4" s="10" t="n">
+      <c r="D4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>ตรงกับ net-1-5 หน้า 14-15 ข้อเสียคือการส่งแบบเรียลไทม์อาจล่าช้าหรือดีเลย์</t>
+        </is>
+      </c>
+      <c r="L4" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="M4" s="10" t="inlineStr">
+      <c r="M4" s="12" t="inlineStr">
         <is>
           <t>คำตอบไม่ถูกต้องหรือไม่มีข้อมูลสนับสนุนจากตำรา</t>
         </is>
       </c>
-      <c r="N4" s="10" t="n">
+      <c r="N4" s="12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>จงอธิบายความหมายของเครือข่ายคอมพิวเตอร์</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>เครือข่ายคอมพิวเตอร์ หมายถึง การนำอุปกรณ์ตั้งแต่หนึ่งชิ้นขึ้นไปมาเชื่อมโยงระหว่างกัน ทำให้สามารถสื่อสารเพื่อการแลกเปลี่ยนข้อมูลระหว่างกัน โดยเฉพาะการนำคอมพิวเตอร์มาเชื่อมโยงกันเป็นเครือข่ายเพื่อใช้งานร่วมกัน (บทที่ 1 หน้า 28)
 เครือข่ายคอมพิวเตอร์ช่วยให้สามารถใช้ทรัพยากรร่วมกันได้ เช่น เครื่องพิมพ์ โปรแกรม และข้อมูล รวมถึงช่วยลดต้นทุนและเพิ่มความสะดวกในการสื่อสาร พร้อมทั้งมีระบบความปลอดภัยในการควบคุมการเข้าถึง (บทที่ 1 หน้า 18)
@@ -663,19 +700,28 @@
 เครือข่ายคอมพิวเตอร์ยังมีการใช้มาตรฐาน เช่น แบบจำลอง OSI ที่ถูกกำหนดโดยหน่วยงาน ISO เพื่อให้อุปกรณ์จากผู้ผลิตต่างๆ สามารถทำงานร่วมกันได้ (บทที่ 1 หน้า 28-29)</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="8" t="n"/>
+      <c r="D5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>ความหมายตรงกับบทสรุป net-1-26 หน้า 28 ส่วนที่เสริมมาตรงกับ net-1-8 ถึง net-1-10 และ net-1-22</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>อยากทราบว่าหน่วยงานกำหนดมาตรฐานเครือข่ายมีบทบาทหน้าที่อะไร จงยกตัวอย่างหน่วยงานดังกล่าวมา 2 ตัวอย่าง พร้อมระบุหน้าที่ของแต่ละหน่วยงานมาให้เข้าใจพอสังเขป</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>หน่วยงานกำหนดมาตรฐานมีบทบาทในการสร้างข้อกำหนดและเกณฑ์มาตรฐานสากล เพื่อให้อุปกรณ์หรือผลิตภัณฑ์จากผู้ผลิตต่างๆ สามารถทำงานร่วมกันได้อย่างมีประสิทธิภาพ โดยช่วยลดความซับซ้อนในการสื่อสารข้อมูลระหว่างระบบต่างๆ และทำให้ผู้บริโภคสามารถเลือกใช้อุปกรณ์จากค่ายต่างๆ ได้โดยไม่ต้องกังวลเรื่องความเข้ากันได้ (บทที่ 1 หน้า 18)
 ตัวอย่างหน่วยงานดังกล่าว ได้แก่
@@ -685,19 +731,28 @@
 หน่วยงานเหล่านี้ช่วยให้เกิดความเข้ากันได้ระหว่างอุปกรณ์จากผู้ผลิตต่างประเทศ และสนับสนุนการพัฒนาเทคโนโลยีเครือข่ายอย่างต่อเนื่องครับ</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="8" t="n"/>
+      <c r="D6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>บทบาทและตัวอย่าง ISO กับ IEEE ตรงกับ net-1-11 หน้า 18 และ net-1-12 หน้า 19</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>ระบบการสื่อสารข้อมูลจะสมบูรณ์ต่อเมื่อต้องมีส่วนประกอบส่วนใดบ้าง จงอธิบาย</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>ระบบการสื่อสารข้อมูลจะสมบูรณ์ต่อเมื่อมีส่วนประกอบ 5 ส่วน ได้แก่ ข้อมูล ฝ่ายส่งข้อมูล ฝ่ายรับข้อมูล สื่อกลางส่งข้อมูล และโปรโตคอล (บทที่ 1 หน้า 28-29)
 1. ข้อมูล คือ ข่าวสารหรือสารสนเทศที่ต้องการส่ง เช่น ข้อความ ภาพ วิดีโอ หรือสื่อประสม ซึ่งจะถูกเข้ารหัสแล้วส่งผ่านสายส่งข้อมูล (บทที่ 1 หน้า 15-16)
@@ -707,19 +762,28 @@
 5. โปรโตคอล คือ ภาษาหรือข้อตกลงที่ใช้ให้ฝ่ายส่งและฝ่ายรับสื่อสารกันเข้าใจได้ (บทที่ 1 หน้า 16)</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="8" t="n"/>
+      <c r="D7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>ครบ 5 ส่วนพร้อมคำอธิบายตาม net-1-6 และ net-1-7 หน้า 15-16</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="A8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>จงบอกประโยชน์ของระบบเครือข่าย</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>ระบบเครือข่ายมีประโยชน์หลายประการ ได้แก่
 1. สามารถใช้ทรัพยากรร่วมกัน เช่น เครื่องคอมพิวเตอร์ เครื่องพิมพ์ และโปรแกรมได้ แม้จะไม่ได้ต่อพ่วงกับเครื่องตนเองโดยตรง แต่สามารถเข้าถึงและใช้งานผ่านเครือข่ายได้ (บทที่ 1 หน้า 16-17)
@@ -729,19 +793,28 @@
 5. มีโปรแกรมอรรถประโยชน์ที่ช่วยเสริมประสิทธิภาพการทำงาน เช่น โปรแกรมไฟร์วอลล์ โปรแกรมสำรองข้อมูล โปรแกรมป้องกันไวรัส และโปรแกรมเข้าถึงระบบจากระยะไกล (บทที่ 2 หน้า 65)</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="8" t="n"/>
+      <c r="D8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>ประโยชน์ 4 ข้อแรกตรงกับ net-1-8 ถึง net-1-10 แต่ข้อ 5 นำโปรแกรมอรรถประโยชน์จาก net-2-29 หน้า 65 มาเพิ่ม ซึ่งตำราไม่ได้จัดเป็นประโยชน์ของเครือข่าย</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>จงสรุปหลักการทำงานของแต่ละลำดับชั้นบนแบบจำลอง OSI</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>ชั้นสื่อสารทางกายภาพ (Physical Layer) มีหน้าที่เกี่ยวข้องกับคุณลักษณะทางกายภาพด้านการสื่อสารระหว่างอุปกรณ์ โดยกำหนดวิธีควบคุมการรับส่งข้อมูลระหว่างเครื่องคอมพิวเตอร์ในระดับบิต ใช้แรงดันไฟฟ้าเท่าใด ใช้สายเคเบิลชนิดใด รูปแบบการส่งข้อมูลเป็นแบบทิศทางเดียวหรือสองทิศทาง และลักษณะการเชื่อมต่ออุปกรณ์ภายในเครือข่าย (บทที่ 1 หน้า 21-22)
 ชั้นสื่อสารเชื่อมต่อข้อมูล (Data Link Layer) มีหน้าที่จัดรูปแบบข้อมูลในรูปแบบของเฟรมข้อมูล และระบุที่อยู่ปลายทาง รวมถึงตรวจสอบความถูกต้องของข้อมูลที่ส่งผ่านช่องทางการสื่อสาร
@@ -752,19 +825,28 @@
 ชั้นสื่อสารการประยุกต์ (Application Layer) เป็นชั้นที่เกี่ยวข้องกับการทำงานของโปรแกรมประยุกต์ต่างๆ ที่ผู้ใช้สามารถใช้เข้าถึงเครือข่าย เช่น โปรแกรมอีเมล โปรโตคอล FTP หรือเทลเน็ต (บทที่ 1 หน้า 23)</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="8" t="n"/>
+      <c r="D9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>สรุปหน้าที่ครบทั้ง 7 ชั้นตรงกับ net-1-16 ถึง net-1-19 และตารางที่ 1.1 ใน net-1-21</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>เครือข่ายคอมพิวเตอร์มีอยู่กี่ประเภท อะไรบ้าง จงอธิบาย</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>เครือข่ายคอมพิวเตอร์สามารถแบ่งประเภทตามลักษณะทางภูมิศาสตร์ได้ 3 ประเภทด้วยกัน คือ
 1. เครือข่ายท้องถิ่น (Local Area Network : LAN)
@@ -775,38 +857,56 @@
 เครือข่ายระดับประเทศ (WAN) เป็นเครือข่ายที่ครอบคลุมพื้นที่กว้างมาก เช่น หลายจังหวัด หลายประเทศ หรือทั่วโลก โดยมักใช้ระบบสื่อสารผ่านดาวเทียมหรือสายเคเบิล (บทที่ 1 หน้า 24-25)</t>
         </is>
       </c>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="8" t="n"/>
+      <c r="D10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>3 ประเภทตรงกับ net-1-22 แต่ข้อความว่า LAN เหมาะกับ 10-20 เครื่องไม่มีใน net-1-23 หน้า 25 (เป็นข้อมูลเพียร์ทูเพียร์ในบทที่ 3)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>ในอนาคตจะเป็นไปได้หรือไม่ว่าระบบโทรศัพท์แบบ VoIP จะมาทดแทนระบบโทรศัพท์แบบเดิมที่ใช้งานอยู่ในปัจจุบัน จงอธิบายพร้อมเหตุผลประกอบ</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>ในอนาคต ระบบโทรศัพท์แบบ VoIP มีแนวโน้มจะมาทดแทนระบบโทรศัพท์แบบเดิมที่ใช้งานอยู่ในปัจจุบันได้ เนื่องจากเทคโนโลยี VoIP ใช้เครือข่ายอินเทอร์เน็ตในการส่งข้อมูลเสียงโดยการบรรจุเสียงลงในรูปแบบของแพ็กเก็ต และส่งผ่านเร้าเตอร์ ซึ่งช่วยลดต้นทุนด้านการสื่อสารระหว่างประเทศได้มาก (บทที่ 1 หน้า 12-13) นอกจากนี้ ระบบ VoIP ยังสามารถทำงานร่วมกับเครือข่ายดิจิตอลและระบบไร้สายได้ ทำให้เหมาะกับการใช้งานในยุคปัจจุบันที่มีการเชื่อมต่ออินเทอร์เน็ตอย่างกว้างขวาง (บทที่ 1 หน้า 14)
 อย่างไรก็ตาม ข้อจำกัดของ VoIP คืออาจเกิดความล่าช้าหรือดีเลย์ในการสื่อสาร เนื่องจากแพ็กเก็ตข้อมูลต้องผ่านเครือข่ายอินเทอร์เน็ตที่มีความซับซ้อนสูง ซึ่งอาจทำให้การพูดคุยไม่เป็นไปอย่างทันทีทันใดเท่ากับระบบโทรศัพท์แบบเดิม (บทที่ 1 หน้า 14-15) อย่างไรก็ตาม ด้วยการพัฒนาเทคโนโลยีเครือข่ายและคุณภาพการเชื่อมต่อที่ดีขึ้น ความเสี่ยงด้านความล่าช้าก็อาจลดลงได้ในอนาคต (บทที่ 1 หน้า 14)
 ดังนั้น แม้ระบบโทรศัพท์แบบเดิมยังคงใช้งานอยู่ในบางพื้นที่ โดยเฉพาะบริเวณปลายทางที่ยังใช้ระบบแอนะล็อก เช่น POTS และ PSTN (บทที่ 1 หน้า 14) แต่แนวโน้มการใช้งาน VoIP เพิ่มขึ้นเรื่อย ๆ ทั้งในองค์กรและบุคคลทั่วไป จึงเป็นไปได้ว่าในอนาคต VoIP จะกลายเป็นระบบหลักในการสื่อสารผ่านโทรศัพท์ (บทที่ 1 หน้า 12-13)</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="8" t="n"/>
+      <c r="D11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>ให้เหตุผลจากข้อดีเรื่องต้นทุนและข้อเสียเรื่องดีเลย์ตาม net-1-3 ถึง net-1-5 หน้า 12-15</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="A12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>เครือข่ายคอมพิวเตอร์คืออะไร</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>เครือข่ายคอมพิวเตอร์คือการนำเครื่องคอมพิวเตอร์มากกว่าหนึ่งเครื่องมาเชื่อมโยงเข้าด้วยกันผ่านช่องทางการสื่อสารทั้งแบบมีสายและแบบไร้สาย เพื่อให้สามารถสื่อสารและใช้ทรัพยากรร่วมกันได้
 การเชื่อมโยงดังกล่าวอาจใช้สายเคเบิล สายโทรศัพท์ สายไฟฟ้า คลื่นวิทยุ หรือคลื่นอินฟราเรด เป็นต้น รวมถึงอุปกรณ์เช่น การ์ดเครือข่ายและอุปกรณ์คอนเน็กเตอร์ (บทที่ 1 หน้า 12)
@@ -815,19 +915,28 @@
 เครือข่ายคอมพิวเตอร์จัดเป็นส่วนหนึ่งของระบบเครือข่ายที่กว้างขึ้น ซึ่งอาจประกอบด้วยอุปกรณ์อื่นๆ ได้ด้วย (บทที่ 1 หน้า 28)</t>
         </is>
       </c>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="8" t="n"/>
+      <c r="D12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>ตรงกับ net-1-2 หน้า 12 นำคอมพิวเตอร์มากกว่าหนึ่งเครื่องมาเชื่อมโยงกันผ่านช่องทางการสื่อสาร</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="A13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>แบบจำลอง OSI มีกี่ชั้น</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>แบบจำลอง OSI มีชั้นสื่อสารทั้งหมด 7 ชั้น (บทที่ 1 หน้า 21)
 ชั้นสื่อสารทั้ง 7 ได้แก่
@@ -840,38 +949,56 @@
 7. ชั้นสื่อสารการประยุกต์ (บทที่ 1 หน้า 21-22)</t>
         </is>
       </c>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="8" t="n"/>
+      <c r="D13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>7 ชั้นพร้อมชื่อครบตาม net-1-15 และ net-1-16 หน้า 21-22</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="A14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>ใครเป็นผู้ประดิษฐ์โทรศัพท์ และเมื่อปีใด</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>ผู้ประดิษฐ์โทรศัพท์คือ อเล็กซานเดอร์ แกรแฮม เบล ในปี ค.ศ. 1876
 เทคโนโลยีโทรศัพท์เริ่มแรกใช้การแปลงเสียงพูดเป็นสัญญาณแอนะล็อกส่งผ่านสาย และแปลงกลับเป็นเสียงที่ปลายทาง
 ปัจจุบันมีการพัฒนาเทคโนโลยีโทรศัพท์ให้ซับซ้อนขึ้น ทั้งระบบดิจิตอลและระบบ VoIP ที่ส่งผ่านเครือข่ายอินเทอร์เน็ต (บทที่ 1 หน้า 12-13)</t>
         </is>
       </c>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="8" t="n"/>
+      <c r="D14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>อเล็กซานเดอร์ แกรแฮม เบล ค.ศ. 1876 ตรงกับ net-1-3 หน้า 12-13</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="A15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>ข้อเสียของ VoIP คืออะไร</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>ข้อเสียของ VoIP คือ ความสามารถในการส่งข้อมูลแบบเรียลไทม์อาจลดลง เนื่องจากแพ็กเก็ตข้อมูลต้องผ่านเครือข่ายอินเทอร์เน็ตที่มีจำนวนเครือข่ายมากมาย ทำให้เกิดการดีเลย์หรือความล่าช้าในการสื่อสารได้ (บทที่ 1 หน้า 14-15)
 การสื่อสารแบบเรียลไทม์อาจไม่สมบูรณ์ตามเวลาที่ต้องการ เนื่องจากการส่งข้อมูลผ่านเครือข่ายอินเทอร์เน็ตที่มีความซับซ้อนและอาจมีปัญหาด้านความหนาแน่นของข้อมูล (บทที่ 1 หน้า 28-29)
@@ -879,37 +1006,55 @@
 ข้อเสียอีกประการหนึ่งอาจเกิดจากความเสถียรของอินเทอร์เน็ต หากความเร็วหรือความเสถียรสัญญาณต่ำ อาจทำให้เสียงพูดขาดหายหรือมีเสียงรบกวนได้</t>
         </is>
       </c>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="8" t="n"/>
+      <c r="D15" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>ข้อเสียเรื่องเรียลไทม์และดีเลย์ตรงกับ net-1-5 หน้า 14-15 และ net-1-27</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="A16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>IEEE 802.5 คือมาตรฐานอะไร</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>IEEE 802.5 คือมาตรฐานเครือข่ายโทเค็นริง
 มาตรฐานนี้ระบุเกณฑ์การสื่อสารในเครือข่ายท้องถิ่นที่ใช้โครงสร้างแบบวงแหวน โดยมีการส่งข้อมูลผ่านสัญญาณโทเค็น (Token) เพื่อควบคุมการเข้าถึงสื่อกลางอย่างมีระเบียบ (บทที่ 1 หน้า 19-20)</t>
         </is>
       </c>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="8" t="n"/>
+      <c r="D16" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>IEEE 802.5 (Token Ring) มาตรฐานเครือข่ายโทเค็นริง ตรงกับ net-1-13 หน้า 19-20</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="A17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>ส่วนประกอบของระบบการสื่อสารข้อมูลมีอะไรบ้าง</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>ส่วนประกอบของระบบการสื่อสารข้อมูลมี 5 ส่วน ได้แก่
 1. ข้อมูล ข้อมูลในที่นี้ก็คือข่าวสารหรือสารสนเทศต่างๆ ที่ต้องการส่งไปยังปลายทาง ข่าวสารเหล่านี้อาจเป็นข้อความ ภาพ วิดีโอ หรือสื่อประสม (Multimedia) ข้อมูลที่ส่งไปจะถูกเข้ารหัส และส่งผ่านสายส่งข้อมูลไปยังปลายทาง ครั้นเมื่อปลายทางได้รับข้อมูลแล้ว ก็จะดำเนินการถอดรหัสข้อมูลข่าวสารนี้ให้กลับมาอยู่ในรูปแบบข้อมูลเดิมเหมือนกับต้นฉบับที่ส่งมา (บทที่ 1 หน้า 15-16)
@@ -919,38 +1064,56 @@
 5. โปรโตคอล (Protocol) การสื่อสารระหว่างต้นทางไปยังปลายทางจะสมบูรณ์ก็ต่อเมื่อ ทั้งสองฝ่ายต่างสื่อสารกันได้อย่างเข้าใจ ดังนั้นโปรโตคอลจึงมีบทบาทหน้าที่สำคัญเพื่อการนี้ โดยโปรโตคอลจะเปรียบเสมือนภาษาที่ใช้เป็นภาษากลางเพื่อให้ฝ่ายส่งข้อมูลและฝ่ายรับข้อมูลสามารถสื่อสารกันได้อย่างเข้าใจ เพื่อนำไปสู่การปฏิบัติตามข้อตกลงได้อย่างถูกต้อง และส่งผลให้การสื่อสารทั้งสองฝ่ายเกิดผลสัมฤทธิ์ในที่สุด (บทที่ 1 หน้า 16)</t>
         </is>
       </c>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="8" t="n"/>
+      <c r="D17" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>5 ส่วนพร้อมคำอธิบายตรงกับ net-1-6 และ net-1-7 หน้า 15-16</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="A18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>เครือข่ายท้องถิ่นหรือ LAN คืออะไร</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>เครือข่ายท้องถิ่น หรือ LAN คือ เครือข่ายขนาดเล็กที่สุดในบรรดาทั้ง 3 ประเภท เนื่องจากครอบคลุมพื้นที่บนระยะทางที่จำกัด เช่น ภายในอาคาร สำนักงานห้องทำงานที่อยู่ภายในบริเวณเดียวกัน เป็นต้น
 เครือข่ายท้องถิ่นจัดเป็นเครือข่ายที่มีการนำไปติดตั้งเพื่อใช้งานมากที่สุดในกลุ่ม ไม่ว่าจะเป็นตามที่อยู่อาศัยหรือหน่วยงานทั่วไป ตัวอย่างเช่นการติดตั้งเครือข่ายท้องถิ่นตามบริษัทต่างๆ ตามสถาบันการศึกษา หรือโรงพยาบาล เป็นต้น
 เครือข่ายท้องถิ่นมีข้อจำกัดบนพื้นที่ไม่กี่กิโลเมตร ดังนั้นหากต้องการเพิ่มขยายระยะทาง ก็สามารถเพิ่มได้ด้วยการใช้อุปกรณ์ทวนสัญญาณ เพื่อให้สามารถเชื่อมโยงเครือข่ายบนระยะทางที่ไกลออกไปได้กว่าเดิม แต่ก็มีข้อจำกัดบนระยะทางยาวสูงสุด ซึ่งโดยส่วนใหญ่แล้วมักมีการเชื่อมโยงบนระยะทางโดยรวมแล้วไม่เกินกว่า 10 กิโลเมตร (บทที่ 1 หน้า 25)</t>
         </is>
       </c>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="8" t="n"/>
+      <c r="D18" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>ความหมายของ LAN ตรงกับ net-1-23 หน้า 25</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="A19" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>ช่องทางการสื่อสารถือเป็นส่วนสำคัญต่อระบบการสื่อสารข้อมูลอย่างไร</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>ช่องทางการสื่อสารถือเป็นส่วนสำคัญของระบบการสื่อสาร เพราะเป็นเส้นทางที่ใช้ลำเลียงข้อมูลหรือสารสนเทศระหว่างอุปกรณ์ที่สื่อสารกัน
 ช่องทางการสื่อสารเกี่ยวข้องกับแถบความถี่ (Bandwidth) ซึ่งถ้าช่องทางมีแถบความถี่กว้าง จะสามารถส่งข้อมูลได้เร็วขึ้น และรองรับข้อมูลที่ต้องการความเร็วสูง เช่น เสียง วิดีโอ หรือสื่อประสมได้ดีกว่า
@@ -962,38 +1125,56 @@
 การพิจารณาช่องทางการสื่อสารควรพิจารณาจากปัจจัยต่างๆ เช่น ต้นทุน ความเร็ว ความปลอดภัย และสภาพแวดล้อม (บทที่ 2 หน้า 52) (บทที่ 2 หน้า 53)</t>
         </is>
       </c>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="8" t="n"/>
+      <c r="D19" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>ตรงกับ net-2-1 หน้า 40 ช่องทางการสื่อสารเป็นเส้นทางลำเลียงข้อมูลและเกี่ยวข้องกับแถบความถี่</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="A20" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>การส่งสัญญาณแบบเบสแบนด์ต่างจากการส่งสัญญาณแบบบรอดแบนต์อย่างไร</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>การส่งสัญญาณแบบเบสแบนด์ใช้ช่องทางการสื่อสารเพียงช่องทางเดียวสำหรับส่งสัญญาณดิจิตอลในแต่ละครั้งในช่วงเวลาหนึ่ง ขณะที่การส่งสัญญาณแบบบรอดแบนด์ใช้ช่องทางการสื่อสารหลายช่องทางเพื่อส่งสัญญาณแอนะล็อก โดยข้อมูลสามารถลำเลียงบนช่วงความถี่ที่แตกต่างกันได้ในแต่ละครั้ง (บทที่ 2 หน้า 40-41)
 การส่งสัญญาณแบบเบสแบนด์มีระบบการจัดการที่ไม่ซับซ้อนและควบคุมได้ง่าย แต่การส่งสัญญาณแบบบรอดแบนด์มีระบบการจัดการที่ยุ่งยากกว่ามาก เนื่องจากต้องจัดการกับข้อมูลที่ลำเลียงอยู่บนหลายช่องความถี่พร้อมกัน (บทที่ 2 หน้า 41)
 เครือข่ายท้องถิ่นโดยทั่วไปใช้วิธีการส่งสัญญาณแบบเบสแบนด์ (บทที่ 2 หน้า 69)</t>
         </is>
       </c>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="8" t="n"/>
+      <c r="D20" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>ตรงกับ net-2-2 และ net-2-3 หน้า 40-41 เบสแบนด์ช่องทางเดียวสัญญาณดิจิตอล บรอดแบนด์หลายช่องทางสัญญาณแอนะล็อก</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="A21" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>สายคู่บิดเกลียวมีลักษณะอย่างไร และมีกี่ประเภท อะไรบ้าง</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>สายคู่บิดเกลียวเป็นสายทองแดงที่มีวัสดุห่อหุ้มด้วยพลาสติก โดยสายแต่ละคู่จะถูกบิดเกลียวเข้าหากันเพื่อลดสัญญาณรบกวน
 สายคู่บิดเกลียวแบ่งออกเป็น 2 ประเภท ได้แก่ สายยูที่พี (UTP : Unshielded Twisted-Pair Cable) ที่ไม่มีฉนวนป้องกันสัญญาณรบกวน และสายเอสทีพี (STP : Shielded Twisted-Pair Cable) ที่มีฉนวนป้องกันสัญญาณรบกวน
@@ -1002,19 +1183,28 @@
 สายคู่บิดเกลียวมีหลายประเภทตามมาตรฐาน เช่น สายยูที่พี CAT2, CAT3, และ CAT5 ซึ่งใช้หัวเชื่อมต่อแบบ RJ-11 หรือ RJ-45 ขึ้นอยู่กับรุ่น (บทที่ 2 หน้า 54-55)</t>
         </is>
       </c>
-      <c r="D21" s="7" t="n"/>
-      <c r="E21" s="8" t="n"/>
+      <c r="D21" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>ลักษณะและ 2 ประเภท (UTP, STP) ตรงกับ net-2-5 หน้า 41-43</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="A22" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>สายโคแอกเชียลมีข้อดีและข้อเสียด้านไดบ้าง</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>สายโคแอกเชียลมีข้อดีคือ เป็นสายสัญญาณที่ป้องกันสัญญาณรบกวนได้เป็นอย่างดี
 ข้อดีอีกประการคือ สามารถเชื่อมโยงได้ในระยะทางไกลกว่าสายคู่บิดเกลียว
@@ -1024,19 +1214,28 @@
 ข้อเสียสุดท้ายคือ การติดตั้งหัวเชื่อมต่อต้องใช้ความเชี่ยวชาญ (บทที่ 2 หน้า 43-44)</t>
         </is>
       </c>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="8" t="n"/>
+      <c r="D22" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>ข้อดี 3 ข้อและข้อเสีย 3 ข้อครบตาม net-2-6 หน้า 43-44</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="A23" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>สายใยแก้วนำแสงมักนำไปใช้เพื่องานใด</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>สายใยแก้วนำแสงมักนำไปใช้เป็นสายแกนหลักเพื่อเชื่อมโยงเครือข่ายต่างๆ เข้าด้วยกัน โดยเฉพาะในระยะทางหลายกิโลเมตร ซึ่งสามารถเชื่อมโยงได้โดยไม่ต้องใช้อุปกรณ์ทวนสัญญาณ (บทที่ 2 หน้า 44-45)
 เนื่องจากมีอัตราการลดทอนของสัญญาณต่ำ และรองรับความเร็วสูงได้ดี จึงเหมาะกับการใช้งานในงานที่ต้องการความเร็วและระยะทางไกล เช่น การเชื่อมโยงระหว่างตึกภายในมหาวิทยาลัยหรือการส่งข้อมูลข้ามมหาสมุทร (บทที่ 2 หน้า 54)
@@ -1044,19 +1243,28 @@
 สายใยแก้วนำแสงมักใช้ในโครงข่ายหลัก (backbone network) ขององค์กรหรือผู้ให้บริการอินเทอร์เน็ต (ISP) เพื่อรองรับปริมาณข้อมูลจำนวนมากในระยะทางไกล</t>
         </is>
       </c>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="8" t="n"/>
+      <c r="D23" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>ใช้เป็นสายแกนหลักเชื่อมโยงเครือข่ายตรงกับ net-2-7 หน้า 44-45 และ net-2-18 หน้า 54</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="A24" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>จงสรุปข้อดีและข้อเสียของคลื่นวิทยุ</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>ข้อดีของคลื่นวิทยุ
 • คลื่นวิทยุจัดเป็นคลื่นที่สามารถสร้างขึ้นมาเพื่อใช้งานได้ง่าย
@@ -1069,37 +1277,55 @@
 • สัญญาณจะถูกดูดซึมเมื่อเดินทางผ่านสายฝน (บทที่ 2 หน้า 46)</t>
         </is>
       </c>
-      <c r="D24" s="7" t="n"/>
-      <c r="E24" s="8" t="n"/>
+      <c r="D24" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>ข้อดี 4 ข้อและข้อเสีย 3 ข้อครบตาม net-2-8 หน้า 46</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="A25" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>จงบอกความแตกต่างระหว่างเซลลูลาร์ระบบ AMPS และ GSM</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>ระบบ AMPS และ GSM เป็นระบบเซลลูลาร์ที่ใช้คลื่นความถี่สูงในการสื่อสาร แต่มีความแตกต่างกันตรงที่ระบบ AMPS ส่งข้อมูลแบบแอนะล็อก ใช้คลื่นความถี่ 800 - 900 เมกะเฮิรตซ์ ในขณะที่ระบบ GSM ส่งข้อมูลแบบดิจิตอล ใช้คลื่นความถี่ 1,800 เมกะเฮิรตซ์
 • GSM รองรับการใช้งานร่วมกับบริการอื่น ๆ เช่น SMS และการเข้าถึงอินเทอร์เน็ตได้ดีกว่า (บทที่ 2 หน้า 47)</t>
         </is>
       </c>
-      <c r="D25" s="7" t="n"/>
-      <c r="E25" s="8" t="n"/>
+      <c r="D25" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>แอนะล็อก 800-900 MHz กับดิจิตอล 1,800 MHz ตรงกับ net-2-9 หน้า 47 แต่ข้อที่ว่า GSM รองรับ SMS และอินเทอร์เน็ตดีกว่าไม่มีในตำรา</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="A26" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>จงบอกส่วนที่เหมือนและส่วนต่างระหว่างไมโครเวฟและดาวเทียม</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>ส่วนที่เหมือนระหว่างไมโครเวฟและดาวเทียมคือทั้งสองระบบใช้คลื่นความถี่สูงในการส่งสัญญาณ และสามารถส่งข้อมูลได้ในระยะไกล โดยทั้งสองระบบต้องอาศัยการติดตั้งอุปกรณ์รับส่งสัญญาณที่มีความแม่นยำ เช่น จานรับส่งสัญญาณ ซึ่งต้องตั้งอยู่ในตำแหน่งที่มองเห็นกันได้โดยตรง (บทที่ 2 หน้า 47-49)
 ส่วนต่างคือ ไมโครเวฟส่งสัญญาณระหว่างสถานีภาคพื้นดินที่อยู่ใกล้กัน โดยต้องติดตั้งบนตึกสูงหรือภูเขาเพื่อหลีกเลี่ยงสิ่งกีดขวาง ขณะที่ดาวเทียมส่งสัญญาณจากสถานีภาคพื้นดินไปยังดาวเทียมที่อยู่ในอวกาศ ซึ่งห่างจากพื้นโลกประมาณ 22,000 ไมล์ และส่งกลับมายังสถานีภาคพื้นดินทั่วประเทศ (บทที่ 2 หน้า 47-49)
@@ -1107,38 +1333,56 @@
 ส่วนข้อเสียที่ต่างกันคือ ไมโครเวฟมีปัญหาจากภูมิประเทศและสภาพอากาศ แต่ดาวเทียมมีปัญหาเรื่องความปลอดภัยของข้อมูลและการรบกวนจากพายุฝนตกชุก (บทที่ 2 หน้า 47-49) (บทที่ 2 หน้า 49-50)</t>
         </is>
       </c>
-      <c r="D26" s="7" t="n"/>
-      <c r="E26" s="8" t="n"/>
+      <c r="D26" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>ส่วนเหมือนและส่วนต่างสอดคล้องกับ net-2-10 และ net-2-11 หน้า 47-50 (ดาวเทียมคือสถานีไมโครเวฟในอวกาศ 22,000 ไมล์)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="A27" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>จงสรุปการสื่อสารไร้สายด้วยบลูทูธและอินฟราเรดมาให้พอเข้าใจ</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>การสื่อสารไร้สายด้วยบลูทูธเหมาะสำหรับการใช้งานในระยะใกล้ ประมาณ 10 เมตร แต่สามารถขยายได้ถึง 100 เมตรด้วยอุปกรณ์เสริม และใช้คลื่นวิทยุ ทำให้สามารถส่งผ่านวัตถุหรือสิ่งกีดขวางได้ รองรับการเชื่อมต่อหลายอุปกรณ์พร้อมกัน เช่น คอมพิวเตอร์ โทรศัพท์มือถือ เครื่องพิมพ์ และหูฟัง พร้อมทั้งมีต้นทุนต่ำและได้รับการสนับสนุนจากบริษัทจำนวนมาก (บทที่ 2 หน้า 51)
 การสื่อสารไร้สายด้วยอินฟราเรดใช้คลื่นความถี่สั้นที่ต้องส่งผ่านแนวเส้นตรงโดยไม่สามารถทะลุผ่านวัตถุทึบแสงได้ เช่น ผนัง แต่เหมาะกับการใช้งานระยะใกล้ เช่น รีโมตคอนโทรล หรือการเชื่อมต่อระหว่างคอมพิวเตอร์ เครื่องพิมพ์ และกล้องดิจิตอลผ่านพอร์ต IrDA ข้อดีคือมีความปลอดภัยสูงเพราะสัญญาณไม่สามารถรั่วไปยังห้องข้างเคียงได้ และมีต้นทุนต่ำ
 ทั้งสองเทคโนโลยีเหมาะกับการสื่อสารระยะใกล้ โดยบลูทูธมีความยืดหยุ่นมากกว่าในเรื่องการส่งผ่านสิ่งกีดขวาง ขณะที่อินฟราเรดต้องการการจัดวางอุปกรณ์ให้เห็นกันโดยตรง (บทที่ 2 หน้า 51) (บทที่ 2 หน้า 51-52)</t>
         </is>
       </c>
-      <c r="D27" s="7" t="n"/>
-      <c r="E27" s="8" t="n"/>
+      <c r="D27" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>สรุปบลูทูธตาม net-2-12 หน้า 51 และอินฟราเรดตาม net-2-13 หน้า 51-52 ถูกต้อง</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="A28" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>จงสรุปการพิจารณาสื่อกลางส่งข้อมูลด้านต้นทุน ความเร็ว และระยะทางมาให้พอเข้าใจ</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>การพิจารณาสื่อกลางส่งข้อมูลจากด้านต้นทุน ความเร็ว และระยะทาง มีรายละเอียดดังนี้
 ต้นทุน ควรพิจารณาต้นทุนพื้นฐานของอุปกรณ์สนับสนุนสายเคเบิลชนิดนั้นๆ ต้นทุนการติดตั้งอุปกรณ์ และเปรียบเทียบประสิทธิภาพที่ได้สมกับราคาหรือไม่ โดยอาจเทียบเป็นอัตราส่วนหรือความคุ้มค่าเพียงไร (บทที่ 2 หน้า 52)
@@ -1146,38 +1390,56 @@
 ระยะทาง สื่อกลางแต่ละชนิดมีขีดความสามารถในการส่งสัญญาณได้ไกลต่างกัน สายใยแก้วนำแสงเหมาะกับการเชื่อมโยงระยะไกลหลายกิโลเมตร ในขณะที่สายคู่บิดเกลียวเชื่อมโยงได้ไกลสุดเพียง 100 เมตร แม้จะใช้เครื่องทวนสัญญาณก็ตาม แต่ก็มีข้อจำกัดด้านจำนวนเซกเมนต์ที่เชื่อมต่อ (บทที่ 2 หน้า 52-53)</t>
         </is>
       </c>
-      <c r="D28" s="7" t="n"/>
-      <c r="E28" s="8" t="n"/>
+      <c r="D28" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>ต้นทุน ความเร็ว ระยะทาง ตรงกับ net-2-14 และ net-2-15 หน้า 52-53</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="A29" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>จงสรุปการพิจารณาสื่อกลางส่งข้อมูลด้านสภาพแวดล้อมและความปลอดภัยมาให้พอเข้าใจ</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>การพิจารณาสื่อกลางส่งข้อมูลด้านสภาพแวดล้อมและความปลอดภัยมีดังนี้
 • ด้านสภาพแวดล้อม ควรเลือกใช้สื่อกลางที่ทนทานต่อสัญญาณรบกวน เช่น สายส่งข้อมูลที่มีฉนวนป้องกันสัญญาณรบกวน หรือสายใยแก้วนำแสงชนิดทนความร้อน โดยเฉพาะในสถานที่ที่มีคลื่นรบกวนมาก เช่น โรงงานอุตสาหกรรม และควรหลีกเลี่ยงการใช้สื่อกลางแบบไร้สายในพื้นที่ดังกล่าวเพื่อป้องกันการรบกวนของคลื่น
 • ด้านความปลอดภัย ควรเลือกใช้สื่อกลางที่ยากต่อการดักจับสัญญาณข้อมูล เช่น สายใยแก้วนำแสง หรือใช้ซอฟต์แวร์เข้ารหัสข้อมูลก่อนส่งผ่านสื่อกลาง เพื่อป้องกันการลักลอบหรือจารกรรมข้อมูลบนเครือข่าย (บทที่ 2 หน้า 53)</t>
         </is>
       </c>
-      <c r="D29" s="7" t="n"/>
-      <c r="E29" s="8" t="n"/>
+      <c r="D29" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>สภาพแวดล้อมและความปลอดภัยตรงกับ net-2-16 หน้า 53</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="A30" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>ส่วนประกอบเครือข่ายประกอบด้วยส่วนใดบ้าง จงอธิบายแต่ละส่วนมาให้เข้าใจพอสังเขป</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>ส่วนประกอบของเครือข่ายประกอบด้วย 6 ส่วน ได้แก่
 1. สายเคเบิล ใช้สำหรับขนส่งสัญญาณข้อมูลไปยังปลายทาง ทั้งในระยะใกล้และไกล เช่น สายคู่บิดเกลียว (UTP), สายโคแอกเชียล, สายใยแก้วนำแสง (บทที่ 2 หน้า 54)
@@ -1188,19 +1450,28 @@
 6. โปรโตคอล เป็นภาษาหรือข้อตกลงที่ใช้ในการสื่อสารระหว่างฝ่ายส่งและฝ่ายรับให้เข้าใจกันได้ (บทที่ 1 หน้า 16)</t>
         </is>
       </c>
-      <c r="D30" s="7" t="n"/>
-      <c r="E30" s="8" t="n"/>
+      <c r="D30" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>ครบ 6 ส่วนตาม net-2-18 ถึง net-2-30 และบทสรุป net-2-37</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="A31" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>เกณฑ์วัดประสิทธิภาพเครือข่ายด้านสมรรถนะประกอบด้วยส่วนใดบ้าง จงอธิบาย</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>เกณฑ์วัดประสิทธิภาพเครือข่ายด้านสมรรถนะประกอบด้วยเวลาที่ใช้ในการขนส่งข้อมูล และเวลาตอบสนอง ซึ่งเวลาที่ใช้ในการขนส่งข้อมูลคือช่วงเวลาที่ใช้ส่งข้อมูลจากต้นทางไปยังปลายทาง ส่วนเวลาตอบสนองคือช่วงระยะเวลาระหว่างที่มีการร้องขอข้อมูลจนได้รับข้อมูลกลับมา (บทที่ 2 หน้า 66-67)
 สมรรถนะของเครือข่ายขึ้นอยู่กับปัจจัยหลายด้าน ได้แก่
@@ -1210,55 +1481,82 @@
 4. ซอฟต์แวร์ ซอฟต์แวร์จัดเป็นส่วนสำคัญที่ส่งผลต่อสมรรถนะโดยรวมของเครือช่าย เช่น ระบบปฏิบัติการเครือข่ายที่มีประสิทธิภาพ ย่อมมีระบบการทำงานและควบคุมอุปกรณ์ฮาร์ดแวร์ให้ทำงานได้อย่างมีประสิทธิภาพและรวดเร็ว (บทที่ 2 หน้า 67)</t>
         </is>
       </c>
-      <c r="D31" s="7" t="n"/>
-      <c r="E31" s="8" t="n"/>
+      <c r="D31" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>เวลาขนส่งข้อมูล เวลาตอบสนอง และปัจจัย 4 ด้านครบตาม net-2-32 และ net-2-33 หน้า 66-67</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="A32" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>เกณฑ์วัดประสิทธิภาพเครือข่ายด้านความน่าเชื่อถือและด้านความปลอดภัย ประกอบด้วยส่วนใดบ้าง จงอธิบาย</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>เกณฑ์วัดประสิทธิภาพเครือข่ายด้านความน่าเชื่อถือประกอบด้วย ความถี่ของความล้มเหลว ระยะเวลาในการกู้คืน และความคงทนต่อความล้มเหลว (บทที่ 2 หน้า 67-68)
 ด้านความปลอดภัยประกอบด้วยการป้องกันการลักลอบหรือจารกรรมข้อมูล โดยเฉพาะการดักจับสัญญาณบนเครือข่าย ซึ่งสามารถลดความเสี่ยงได้ด้วยการเลือกใช้สื่อกลางที่ยากต่อการดักจับ เช่น สายใยแก้วนำแสง หรือใช้ซอฟต์แวร์เข้ารหัสข้อมูลก่อนส่ง (บทที่ 2 หน้า 53)</t>
         </is>
       </c>
-      <c r="D32" s="7" t="n"/>
-      <c r="E32" s="8" t="n"/>
+      <c r="D32" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>ด้านความน่าเชื่อถือครบ 3 ข้อตาม net-2-34 แต่ด้านความปลอดภัยไปหยิบ net-2-16 หน้า 53 แทน net-2-35 หน้า 68 จึงขาดการป้องกันผู้ไม่มีสิทธิ์และการป้องกันไวรัส</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="A33" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>อยากทราบว่านักเรียนมีมาตรการป้องกันความปลอดภัยจากการใช้งานคอมพิวเตอร์มิให้ติดไวรัสไต้อย่างไร</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>นักเรียนสามารถป้องกันความปลอดภัยจากการใช้งานคอมพิวเตอร์ไม่ให้ติดไวรัสได้โดยการติดตั้งโปรแกรมป้องกันไวรัส และต้องอัปเดตโปรแกรมไวรัสอยู่เสมอ
 นอกจากนี้ ควรมีการกำหนดยูสเซอร์พร้อมรหัสผ่าน การกำหนดสิทธิ์การใช้งาน และการติดตั้งไฟร์วอลล์เพื่อป้องกันผู้บุกรุกจากเครือข่ายภายนอก (บทที่ 2 หน้า 68)</t>
         </is>
       </c>
-      <c r="D33" s="7" t="n"/>
-      <c r="E33" s="8" t="n"/>
+      <c r="D33" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>ติดตั้งและอัปเดตโปรแกรมป้องกันไวรัสตรงกับ net-2-35 หน้า 68</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="A34" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
         <is>
           <t>สายคู่บิดเกลียวคืออะไร มีข้อดีข้อเสียอย่างไร</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>สายคู่บิดเกลียวคือสายทองแดงที่มีฉนวนพลาสติกห่อหุ้ม โดยสายแต่ละคู่จะถูกบิดเกลียวเข้าหากันเพื่อลดสัญญาณรบกวน ซึ่งสามารถแบ่งเป็นสายยูทีพี (UTP) ที่ไม่มีฉนวนป้องกัน และสายเอสทีพี (STP) ที่มีฉนวนป้องกันสัญญาณรบกวน (บทที่ 2 หน้า 41-43)
 ข้อดีของสายคู่บิดเกลียว ได้แก่
@@ -1272,19 +1570,28 @@
 • มีความเร็วค่อนข้างจำกัด (บทที่ 2 หน้า 41-43)</t>
         </is>
       </c>
-      <c r="D34" s="7" t="n"/>
-      <c r="E34" s="8" t="n"/>
+      <c r="D34" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>ความหมาย ข้อดี 4 ข้อ ข้อเสีย 3 ข้อครบตาม net-2-5 หน้า 41-43</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="A35" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>สายใยแก้วนำแสงมีข้อเสียอะไรบ้าง</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>สายใยแก้วนำแสงมีข้อเสียดังนี้
 • มีราคาแพงที่สุดเมื่อเปรียบเทียบกับสายชนิดอื่นๆ
@@ -1292,19 +1599,28 @@
 • ตัวสายไม่สามารถโค้งงอได้มาก (บทที่ 2 หน้า 44-45)</t>
         </is>
       </c>
-      <c r="D35" s="7" t="n"/>
-      <c r="E35" s="8" t="n"/>
+      <c r="D35" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>ข้อเสีย 3 ข้อครบตาม net-2-7 หน้า 44-45</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="A36" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
         <is>
           <t>สายโคแอกเชียลมีข้อดีอะไร</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C36" s="7" t="inlineStr">
         <is>
           <t>สายโคแอกเชียลมีข้อดีดังนี้
 • เป็นสายสัญญาณที่ป้องกันสัญญาณรบกวนได้เป็นอย่างดี
@@ -1312,38 +1628,56 @@
 • ความเร็วในการส่งข้อมูลสูง (บทที่ 2 หน้า 43-44)</t>
         </is>
       </c>
-      <c r="D36" s="7" t="n"/>
-      <c r="E36" s="8" t="n"/>
+      <c r="D36" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>ข้อดี 3 ข้อครบตาม net-2-6 หน้า 43-44</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="A37" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>บลูทูธส่งสัญญาณได้ไกลประมาณกี่เมตร</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>บลูทูธส่งสัญญาณได้ไกลประมาณ 10 เมตร สำหรับการใช้งานทั่วไปในสำนักงานขนาดเล็กและบ้านพักอาศัย แต่สามารถขยายระยะทางได้ไกลถึง 100 เมตร หากมีอุปกรณ์เพิ่มเติมสนับสนุนระบบ (บทที่ 2 หน้า 51)
 💡 เสริมจากความรู้ทั่วไปของ AI (ส่วนนี้ไม่ได้มาจากหนังสือ ควรตรวจกับครูผู้สอนหรือแหล่งอื่นประกอบ)
 ระยะทางที่กล่าวถึงขึ้นอยู่กับรุ่นของบลูทูธและสภาพแวดล้อม เช่น ไม่มีสิ่งกีดขวางหรือสัญญาณรบกวน</t>
         </is>
       </c>
-      <c r="D37" s="7" t="n"/>
-      <c r="E37" s="8" t="n"/>
+      <c r="D37" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>ประมาณ 10 เมตร ขยายได้ถึง 100 เมตร ตรงกับ net-2-12 หน้า 51</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="A38" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>ฮับทำงานอยู่ในชั้นสื่อสารใดของแบบจำลอง OSI</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>ฮับทำงานอยู่ในชั้นสื่อสารทางกายภาพของแบบจำลอง OSI (บทที่ 2 หน้า 53-54)
 ชั้นสื่อสารทางกายภาพมีหน้าที่เกี่ยวข้องกับคุณลักษณะทางกายภาพด้านการสื่อสารระหว่างอุปกรณ์ โดยการกำหนดวิธีควบคุมการรับส่งข้อมูลระหว่างเครื่องคอมพิวเตอร์ในระดับบิต (บทที่ 1 หน้า 21-22)
@@ -1351,38 +1685,56 @@
 การเชื่อมต่อระหว่างอุปกรณ์ด้วยฮับทำให้เครือข่ายทั้งหมดถือเป็นเครือข่ายเดียวกัน (บทที่ 2 หน้า 59)</t>
         </is>
       </c>
-      <c r="D38" s="7" t="n"/>
-      <c r="E38" s="8" t="n"/>
+      <c r="D38" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>ฮับทำงานในชั้นสื่อสารทางกายภาพ ตรงกับตารางที่ 2.2 ใน net-2-17 หน้า 53-54 และ net-2-21</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="A39" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
         <is>
           <t>เร้าเตอร์ทำงานอยู่ในชั้นสื่อสารใด</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>เร้าเตอร์ทำงานอยู่ในชั้นสื่อสารควบคุมเครือข่าย ซึ่งเป็นชั้นที่ 3 ของแบบจำลอง OSI (บทที่ 2 หน้า 53-54)
 นอกจากนี้ เร้าเตอร์ยังทำงานในชั้นสื่อสารทางกายภาพและชั้นสื่อสารเชื่อมต่อข้อมูลด้วย ตามลำดับชั้นแรกสามชั้นของแบบจำลอง OSI (บทที่ 2 หน้า 60)
 การจัดการเส้นทางข้อมูลและการส่งแพ็กเก็ตไปยังปลายทางที่เหมาะสมเป็นหน้าที่หลักของเร้าเตอร์ในชั้นสื่อสารควบคุมเครือข่าย (บทที่ 1 หน้า 22-23)</t>
         </is>
       </c>
-      <c r="D39" s="7" t="n"/>
-      <c r="E39" s="8" t="n"/>
+      <c r="D39" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>เร้าเตอร์อยู่ชั้นสื่อสารควบคุมเครือข่ายและทำงานในสามชั้นแรก ตรงกับ net-2-17 หน้า 53-54 และ net-2-23 หน้า 60</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
+      <c r="A40" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>เกณฑ์วัดประสิทธิภาพเครือข่ายมีอะไรบ้าง</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>เกณฑ์วัดประสิทธิภาพเครือข่ายมี 3 ประการ ได้แก่
 1. สมรรถนะ
@@ -1395,36 +1747,54 @@
 ความปลอดภัยหมายถึงการป้องกันข้อมูลจากการเข้าถึงโดยไม่ได้รับอนุญาตหรือการโจมตีจากภายนอก (บทที่ 2 หน้า 66)</t>
         </is>
       </c>
-      <c r="D40" s="7" t="n"/>
-      <c r="E40" s="8" t="n"/>
+      <c r="D40" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>3 เกณฑ์ สมรรถนะ ความน่าเชื่อถือ ความปลอดภัย ตรงกับ net-2-31 หน้า 66</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B41" s="6" t="inlineStr">
+      <c r="A41" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>สายยูทีพี CAT3 ภายในมีสายทองแดงกี่คู่</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>สายยูทีพี CAT3 ภายในมีสายทองแดงอยู่ 4 คู่ (8 เส้น) ด้วยกัน (บทที่ 2 หน้า 54-55)</t>
         </is>
       </c>
-      <c r="D41" s="7" t="n"/>
-      <c r="E41" s="8" t="n"/>
+      <c r="D41" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>4 คู่ (8 เส้น) ตรงกับ net-2-19 หน้า 54-55</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="n">
+      <c r="A42" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B42" s="7" t="inlineStr">
         <is>
           <t>ลักษณะการเชื่อมโยงเครือข่ายมีกี่ลักษณะ อะไรบ้าง จงอธิบาย</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C42" s="7" t="inlineStr">
         <is>
           <t>ลักษณะการเชื่อมโยงเครือข่ายมี 2 ลักษณะ ได้แก่ การเชื่อมโยงแบบจุดต่อจุด (Point-to-Point) และการเชื่อมโยงแบบหลายจุด (Multi-Point) (บทที่ 3 หน้า 82)
 1. การเชื่อมโยงเครือข่ายแบบจุดต่อจุด (Point-to-Point) เป็นการเชื่อมต่อระหว่างอุปกรณ์ 2 อุปกรณ์ที่เชื่อมโยงถึงกันเท่านั้น โดยช่องทางการสื่อสารจะถูกจับจองสำหรับอุปกรณ์ 2 อุปกรณ์เพื่อใช้สื่อสารระหว่างกัน อย่างไรก็ตาม หากโหนดคู่ใดที่ไม่มีสายส่งถึงกัน ก็สามารถสื่อสารผ่านโหนดที่อยู่ติดกันเพื่อส่งทอดต่อไปเรื่อยๆ จนถึงโหนดปลายทางที่ต้องการ (บทที่ 3 หน้า 82)
@@ -1445,19 +1815,28 @@
   • ไม่เหมาะกับการส่งข้อมูลแบบต่อเนื่องที่มีข้อมูลคราวละมากๆ (บทที่ 3 หน้า 83)</t>
         </is>
       </c>
-      <c r="D42" s="7" t="n"/>
-      <c r="E42" s="8" t="n"/>
+      <c r="D42" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>2 ลักษณะพร้อมคำอธิบายตรงกับ net-3-2 หน้า 82 และ net-3-3 หน้า 83</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="n">
+      <c r="A43" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B43" s="6" t="inlineStr">
+      <c r="B43" s="7" t="inlineStr">
         <is>
           <t>จงบอกข้อดีและข้อเสียของการเชื่อมโยงเครือข่ายแต่ละลักษณะ</t>
         </is>
       </c>
-      <c r="C43" s="6" t="inlineStr">
+      <c r="C43" s="7" t="inlineStr">
         <is>
           <t>ข้อดีและข้อเสียของการเชื่อมโยงเครือข่ายแบบจุดต่อจุด (Point-to-Point)
 ข้อดี
@@ -1476,19 +1855,28 @@
 - ไม่เหมาะกับการส่งข้อมูลแบบต่อเนื่องที่มีข้อมูลคราวละมากๆ (บทที่ 3 หน้า 83)</t>
         </is>
       </c>
-      <c r="D43" s="7" t="n"/>
-      <c r="E43" s="8" t="n"/>
+      <c r="D43" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>ข้อดีข้อเสียของแบบจุดต่อจุดและหลายจุดครบตาม net-3-2 และ net-3-3</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="n">
+      <c r="A44" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B44" s="6" t="inlineStr">
+      <c r="B44" s="7" t="inlineStr">
         <is>
           <t>เพราะเหตุใด ทำไมระบบเครือข่ายคอมพิวเตอร์โดยทั่วไปจึงมักนิยมเชื่อมโยงเครือข่าย ในลักษณะแบบหลายจุด</t>
         </is>
       </c>
-      <c r="C44" s="6" t="inlineStr">
+      <c r="C44" s="7" t="inlineStr">
         <is>
           <t>ระบบเครือข่ายคอมพิวเตอร์โดยทั่วไปมักนิยมเชื่อมโยงเครือข่ายในลักษณะแบบหลายจุด เพราะช่วยประหยัดสายส่งข้อมูล และสามารถเพิ่มโหนดใหม่เข้าสู่เครือข่ายได้ง่ายด้วยการเชื่อมต่อเข้ากับสายส่งที่ใช้งานร่วมกันได้ทันที (บทที่ 3 หน้า 83)
 • ประหยัดสายส่งข้อมูล
@@ -1496,19 +1884,28 @@
 ระบบเครือข่ายคอมพิวเตอร์ส่วนใหญ่แล้วจะใช้วิธีการเชื่อมโยงแบบหลายจุด (บทที่ 3 หน้า 83)</t>
         </is>
       </c>
-      <c r="D44" s="7" t="n"/>
-      <c r="E44" s="8" t="n"/>
+      <c r="D44" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" s="10" t="inlineStr">
+        <is>
+          <t>ประหยัดสายและเพิ่มโหนดง่ายตรงกับ net-3-3 หน้า 83</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="n">
+      <c r="A45" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B45" s="6" t="inlineStr">
+      <c r="B45" s="7" t="inlineStr">
         <is>
           <t>จงวาดแผนภาพการเชื่อมโยงเครือข่ายตามมาตรฐานโทโปโลยีแบบบัส พร้อมระบุข้อดีและข้อเสีย</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C45" s="7" t="inlineStr">
         <is>
           <t>แผนภาพการเชื่อมโยงเครือข่ายตามมาตรฐานโทโปโลยีแบบบัส แสดงให้เห็นถึงสายเคเบิลเส้นหนึ่งเป็นสายแกนหลักที่เชื่อมต่ออุปกรณ์ทั้งหมด โดยแต่ละอุปกรณ์เชื่อมต่อผ่านตัวทีคอนเน็กเตอร์ (T-Connector) ที่ติดตั้งบนสายเคเบิล และปลายทั้งสองฝั่งของสายเคเบิลต้องมีเทอร์มิเนเตอร์ (Terminator) ปิดไว้เพื่อดูดซับสัญญาณและป้องกันการสะท้อนกลับของสัญญาณ (บทที่ 3 หน้า 84-86)
 • ข้อดีของโทโปโลยีแบบบัส
@@ -1521,19 +1918,28 @@
 - แต่ละโหนดที่เชื่อมต่อบนเครือข่ายจะต้องอยู่ห่างกันตามข้อกำหนด (บทที่ 3 หน้า 84-86)</t>
         </is>
       </c>
-      <c r="D45" s="7" t="n"/>
-      <c r="E45" s="8" t="n"/>
+      <c r="D45" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F45" s="10" t="inlineStr">
+        <is>
+          <t>บรรยายแผนภาพบัส (สายแกนหลัก ทีคอนเน็กเตอร์ เทอร์มิเนเตอร์) และข้อดีข้อเสียครบตาม net-3-5 หน้า 84-86</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="n">
+      <c r="A46" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B46" s="6" t="inlineStr">
+      <c r="B46" s="7" t="inlineStr">
         <is>
           <t>จงวาดแผนภาพการเชื่อมโยงเครือข่ายตามมาตรฐานโทโปโลยีแบบดาว พร้อมระบุข้อดีและข้อเสีย</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C46" s="7" t="inlineStr">
         <is>
           <t>แผนภาพการเชื่อมโยงเครือข่ายตามมาตรฐานโทโปโลยีแบบดาว แสดงให้เห็นว่ามีอุปกรณ์ฮับ (Hub) เป็นศูนย์กลาง โดยคอมพิวเตอร์ทุกโหนดจะเชื่อมต่อกับฮับผ่านสายเคเบิลแยกต่างหาก ทำให้รูปทรงดูคล้ายดาว มีลำแสงยื่นออกไปจากจุดศูนย์กลาง (บทที่ 3 หน้า 87-88)
 ข้อดีของโทโปโลยีแบบดาว:
@@ -1545,19 +1951,28 @@
 • หากอุปกรณ์ฮับเสียหาย เครือข่ายจะหยุดการทำงานทันที (บทที่ 3 หน้า 87-88)</t>
         </is>
       </c>
-      <c r="D46" s="7" t="n"/>
-      <c r="E46" s="8" t="n"/>
+      <c r="D46" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F46" s="10" t="inlineStr">
+        <is>
+          <t>ฮับเป็นศูนย์กลาง ข้อดี 2 ข้อ ข้อเสีย 3 ข้อครบตาม net-3-6 หน้า 87-88</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="n">
+      <c r="A47" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B47" s="6" t="inlineStr">
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>จงวาดแผนภาพการเชื่อมโยงเครือข่ายตามมาตรฐานโทโปโลยีแบบวงแหวน พร้อมระบุข้อดีและข้อเสีย</t>
         </is>
       </c>
-      <c r="C47" s="6" t="inlineStr">
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t>แผนภาพการเชื่อมโยงเครือข่ายตามมาตรฐานโทโปโลยีแบบวงแหวน แสดงให้เห็นว่าโหนดแรกและโหนดสุดท้ายเชื่อมต่อกันเป็นวงกลม ทำให้เกิดรูปแบบทางกายภาพเป็นวงแหวน โดยแต่ละโหนดจะส่งสัญญาณไปยังโหนดถัดไปในทิศทางเดียว และแต่ละโหนดทำหน้าที่เป็นเครื่องทวนสัญญาณ (repeater) ด้วยตัวเอง (บทที่ 3 หน้า 89-90)
 ข้อดีของโทโปโลยีแบบวงแหวน
@@ -1569,19 +1984,28 @@
 • หากมีบางโหนดบนเครือข่ายเกิดขัดข้อง จะยากต่อการตรวจสอบและค้นหาโหนดที่เสีย (บทที่ 3 หน้า 89-90)</t>
         </is>
       </c>
-      <c r="D47" s="7" t="n"/>
-      <c r="E47" s="8" t="n"/>
+      <c r="D47" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F47" s="10" t="inlineStr">
+        <is>
+          <t>ลักษณะวงแหวน ข้อดี 3 ข้อ ข้อเสีย 2 ข้อครบตาม net-3-7 หน้า 89-90</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="n">
+      <c r="A48" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B48" s="6" t="inlineStr">
+      <c r="B48" s="7" t="inlineStr">
         <is>
           <t>จงอธิบายสถาปัตยกรรมเครือข่ายแบบเพียร์ทูเพียร์มาให้พอเข้าใจ พร้อมระบุข้อดีและข้อเสีย</t>
         </is>
       </c>
-      <c r="C48" s="6" t="inlineStr">
+      <c r="C48" s="7" t="inlineStr">
         <is>
           <t>สถาปัตยกรรมเครือข่ายแบบเพียร์ทูเพียร์ (Peer-to-Peer Network) คือ รูปแบบเครือข่ายที่ทุกเครื่องมีสิทธิเท่าเทียมกัน โดยไม่มีเครื่องใดทำหน้าที่เป็นเซิร์ฟเวอร์เฉพาะ แต่สามารถทำหน้าที่ทั้งผู้ให้บริการ (Server) และผู้รับบริการ (Client) ได้ในเวลาเดียวกัน ขึ้นอยู่กับการตั้งค่าการใช้งาน (บทที่ 3 หน้า 90-91)
 ข้อดีของเครือข่ายแบบเพียร์ทูเพียร์ ได้แก่
@@ -1597,19 +2021,28 @@
 จุดประสงค์หลักของเครือข่ายเพียร์ทูเพียร์คือการแชร์ข้อมูลภายในเครือข่ายเป็นหลัก ไม่ได้มุ่งเน้นด้านความปลอดภัยเท่ากับเครือข่ายแบบไคลเอนต์/เซิร์ฟเวอร์ (บทที่ 3 หน้า 90-91)</t>
         </is>
       </c>
-      <c r="D48" s="7" t="n"/>
-      <c r="E48" s="8" t="n"/>
+      <c r="D48" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F48" s="10" t="inlineStr">
+        <is>
+          <t>คำอธิบายและข้อดีข้อเสียตรงกับ net-3-9 และ net-3-10 หน้า 90-92</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="n">
+      <c r="A49" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B49" s="6" t="inlineStr">
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>จงอธิบายสถาปัตยกรรมเครือข่ายแบบโคลเอนต์/เชิร์ฟเวอร์มาให้พอเข้าใจ พร้อมระบุข้อดีและข้อเสีย</t>
         </is>
       </c>
-      <c r="C49" s="6" t="inlineStr">
+      <c r="C49" s="7" t="inlineStr">
         <is>
           <t>สถาปัตยกรรมเครือข่ายแบบไคลเอนต์/เซิร์ฟเวอร์ (Client/Server) เป็นรูปแบบที่มีเครื่องเซิร์ฟเวอร์เป็นศูนย์กลางในการให้บริการทรัพยากรต่าง ๆ เช่น ไฟล์ งานพิมพ์ ฐานข้อมูล และเว็บไซต์ ให้กับเครื่องลูกข่าย (ไคลเอนต์) ที่ต้องการใช้งาน โดยเครื่องเซิร์ฟเวอร์จะทำหน้าที่รับคำขอจากไคลเอนต์และส่งข้อมูลหรือบริการกลับไปยังเครื่องนั้น
 ข้อดีของเครือข่ายแบบไคลเอนต์/เซิร์ฟเวอร์คือ มีความปลอดภัยสูง มีประสิทธิภาพสูง สามารถเชื่อมต่อเครื่องลูกข่ายได้จำนวนมาก สำรองข้อมูลได้ง่ายเนื่องจากข้อมูลจัดเก็บอยู่ที่เครื่องเซิร์ฟเวอร์เพียงเครื่องเดียว และมีความน่าเชื่อถือสูง
@@ -1618,19 +2051,28 @@
 รูปแบบนี้เหมาะกับองค์กรขนาดใหญ่หรือธุรกิจที่ต้องการควบคุมข้อมูลและสิทธิ์การเข้าถึงอย่างเข้มงวด ซึ่งต่างจากเครือข่ายเพียร์ทูเพียร์ที่เน้นความง่ายและต้นทุนต่ำแต่จำกัดในเรื่องความปลอดภัยและความสามารถในการขยายระบบ</t>
         </is>
       </c>
-      <c r="D49" s="7" t="n"/>
-      <c r="E49" s="8" t="n"/>
+      <c r="D49" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F49" s="10" t="inlineStr">
+        <is>
+          <t>คำอธิบาย ข้อดี 4 ข้อ ข้อเสีย 2 ข้อตรงกับ net-3-11 หน้า 92-93</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="n">
+      <c r="A50" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B50" s="6" t="inlineStr">
+      <c r="B50" s="7" t="inlineStr">
         <is>
           <t>หากนักเรียนมีความต้องการสร้างระบบเครือข่ายขึ้นมาใช้งานเอง อยากทราบว่าจะสร้างเครือข่ายแบบเพียร์ทูเพียร์หรือไคลเอนต์/เซิร์ฟเวอร์ จงอธิบายเหตุผลประกอบ</t>
         </is>
       </c>
-      <c r="C50" s="6" t="inlineStr">
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>หากนักเรียนต้องการสร้างระบบเครือข่ายขึ้นมาใช้งานเอง โดยพิจารณาจากความต้องการทั่วไปของผู้เรียนระดับ ปวช. ควรเลือกใช้เครือข่ายแบบเพียร์ทูเพียร์ เนื่องจากสามารถติดตั้งได้ง่ายและมีต้นทุนต่ำกว่า (บทที่ 3 หน้า 90-91)
 เครือข่ายแบบเพียร์ทูเพียร์เหมาะสำหรับเครือข่ายขนาดเล็ก จำนวน 10–20 เครื่อง โดยไม่จำเป็นต้องใช้ระบบปฏิบัติการเครือข่ายพิเศษ เพราะสามารถตั้งค่าได้จาก Windows ทั่วไป เช่น Windows 7 หรือ Windows 8
@@ -1641,38 +2083,56 @@
 ข้อเสียของเครือข่ายแบบเพียร์ทูเพียร์คือการจัดการบัญชีผู้ใช้ต้องทำแยกตามแต่ละเครื่อง ทำให้ยุ่งยากเมื่อเครือข่ายมีขนาดใหญ่ขึ้น</t>
         </is>
       </c>
-      <c r="D50" s="7" t="n"/>
-      <c r="E50" s="8" t="n"/>
+      <c r="D50" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F50" s="10" t="inlineStr">
+        <is>
+          <t>เลือกเพียร์ทูเพียร์โดยอ้างข้อดีข้อเสียจาก net-3-9 และ net-3-10 หน้า 90-92 ได้ถูกต้อง</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="n">
+      <c r="A51" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="B51" s="7" t="inlineStr">
         <is>
           <t>กลไกการส่งข้อมูลแบบ CSMA/CD ประกอบด้วยกลไกใดบ้าง แต่ละกลไกมีวิธีการทำงานอย่างไร</t>
         </is>
       </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="C51" s="7" t="inlineStr">
         <is>
           <t>กลไกที่ 1 การตรวจฟังสัญญาณ (Carrier Sense) เป็นกลไกสำหรับตรวจฟังสัญญาณในสื่อกลาง หรือสายส่งข้อมูลในขณะนั้นว่าว่างหรือไม่ หากสายสัญญาณในขณะนั้นว่าง จึงจะสามารถส่งข้อมูลได้ แต่ต้องเข้าใจว่าในช่วงเวลานั้นเครื่องลูกข่ายเครื่องอื่นอาจกำลังต้องการส่งข้อมูลพอดี และได้มีการตรวจฟังสัญญาณในขณะนั้นว่าว่างเช่นเดียวกัน ดังนั้นเหตุการณ์นี้เอง จึงจัดเป็นเหตุการณ์หนึ่งที่นำไปสู่การชนกันของกลุ่มข้อมูลได้ในเวลาต่อมารูปที่ 3.16 แสดงถึงเครื่องคอมพิวเตอร์โหนด A ต้องการส่งข้อมูลภายในเครือข่าย และมีการตรวจฟังสัญญาณในขณะนั้นแล้วว่าว่าง จึงดำเนินการส่งข้อมูลผ่านสายส่งไปโดยทันที (บทที่ 3 หน้า 94)
 กลไกที่ 2 การเข้าถึงสื่อกลางร่วมกัน (Multiple Access) เครือข่ายท้องถิ่น โดยเฉพาะเครือข่ายอีเทอร์เน็ต เครื่องลูกข่ายทุกเครื่องจะมีสิทธิเท่าเทียมกันในการส่งข้อมูลบนสื่อกลางกล่าวคือ ทุกๆ เครื่องบนเครือข่ายจะใช้สายส่งเดียวกันเพื่อส่งข้อมูลร่วมกันอย่างเสมอภาคเท่าเทียมกัน ดังนั้นหากมีการตรวจฟังสัญญาณในสายว่าว่าง ก็สามารถส่งได้ทันที ในรูปที่ 3.17 ในช่วงเวลาขณะนั้นเอง เครื่องคอมพิวเตอร์โหนด B ก็ต้องการส่งข้อมูลแล้วมีการตรวจฟังสัญญาณในขณะนั้นว่าว่าง จึงส่งข้อมูลออกมาโดยทันทีเช่นเดียวกัน ครั้นเมื่อทั้งโหนด A และโหนด B ได้ส่งข้อมูลผ่านสายส่งพร้อมกัน ในเวลาต่อมา ข้อมูลของโหนด A และโหนด B ก็ได้เกิดเหตุการณ์การชนกันของกลุ่มข้อมูลขึ้น ทำให้ข้อมูลที่ชนกันเกิดความเสียหาย ข้อมูลที่ส่งไปจึงใช้การไม่ได้อีกต่อไป รูปที่ 3.18 แสดงถึงเหตุการณ์การชนกันของกลุ่มข้อมูลบนสายส่ง (บทที่ 3 หน้า 94-95)
 กลไกที่ 3 การตรวจจับการชนกัน (Collision Detection) หากภายในสายส่งข้อมูลเกิดเหตุการณ์การชนกันของกลุ่มข้อมูลขึ้น นั่นหมายความว่าข้อมูลที่ส่งไปในขณะนั้นใช้การไม่ได้อีกต่อไป ดังนั้นกลไกของวิธีนี้ก็คือ จะรายงานผลว่ามีการชนกันของกลุ่มข้อมูลขึ้นภายในสายส่ง ครั้นเมื่อเครือข่ายได้รับทราบรายงานแล้ว ก็จะให้เครื่องลูกข่ายที่ส่งข้อมูลในขณะนั้นรอสักครู่หนึ่ง เพื่อสุ่มเวลาในการส่งข้อมูลรอบใหม่บนช่วงเวลาที่แตกต่างกัน ดังนั้นโอกาสที่จะเกิดการชนกันในรอบใหม่จึงลดน้อยลง รูปที่ 3.19 ได้มีการตรวจจับพบสัญญาณข้อมูลชนกัน ดังนั้นจึงมีการรายงานให้เครือข่ายรับทราบ รูปที่ 3.20 แต่ละโหนตจะสุ่มเวลาส่งข้อมูลรอบใหม่ เพื่อไม่ให้เกิดการชนกันของข้อมูลอีกโดยจากรูป โหนด A ได้มีการส่งข้อมูลรอบใหม่อย่างสมบูรณ์ โดยปราศจากการชนกันของกลุ่มข้อมูลภายในสายส่ง (บทที่ 3 หน้า 95-96)</t>
         </is>
       </c>
-      <c r="D51" s="7" t="n"/>
-      <c r="E51" s="8" t="n"/>
+      <c r="D51" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F51" s="10" t="inlineStr">
+        <is>
+          <t>3 กลไกของ CSMA/CD พร้อมวิธีทำงานตรงกับ net-3-13 ถึง net-3-15 หน้า 94-96</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="n">
+      <c r="A52" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="B52" s="7" t="inlineStr">
         <is>
           <t>มาตรฐานเครือข่ายอีเทอร์เน็ตแบบดั้งเติมสามารถเชื่อมโยงเครือข่ายในรูปแบบใดได้บ้าง</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C52" s="7" t="inlineStr">
         <is>
           <t>มาตรฐานเครือข่ายอีเทอร์เน็ตแบบดั้งเดิมสามารถเชื่อมโยงเครือข่ายในรูปแบบ 10Base5, 10Base2 และ 10BaseT ได้ (บทที่ 3 หน้า 96)
 • รูปแบบ 10Base5 ใช้สายโคแอกเซียลแบบหนา (RG-8) รูปแบบบัส ระยะทางสูงสุดต่อเซกเมนต์ 500 เมตร ใช้การ์ดเครือข่ายช็อกเก็ตแบบ AUI และมีการติดตั้งทรานซีฟเวอร์ที่ห่างกัน 2.5 เมตร (บทที่ 3 หน้า 98-99)
@@ -1680,19 +2140,28 @@
 • รูปแบบ 10BaseT ใช้สายยูทีพี (CAT-3 หรือ CAT-5) รูปแบบดาว ระยะทางสูงสุดจากฮับถึงโหนด 100 เมตร ใช้การ์ดเครือข่ายช็อกเก็ตแบบ RJ-45 และมีฮับเป็นศูนย์กลาง (บทที่ 3 หน้า 101-104)</t>
         </is>
       </c>
-      <c r="D52" s="7" t="n"/>
-      <c r="E52" s="8" t="n"/>
+      <c r="D52" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F52" s="10" t="inlineStr">
+        <is>
+          <t>3 รูปแบบ 10Base5, 10Base2, 10BaseT ตรงกับ net-3-17 หน้า 96 และรายละเอียดใน net-3-18 ถึง net-3-21</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="n">
+      <c r="A53" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B53" s="7" t="inlineStr">
         <is>
           <t>จงสรุปข้อกำหนดมาตรฐานอีเทอร์เน็ตแบบ 10Base5</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C53" s="7" t="inlineStr">
         <is>
           <t>ข้อกำหนดมาตรฐานอีเทอร์เน็ตแบบ 10Base5 คือ
 1. ส่งข้อมูลแบบเบสแบนด์
@@ -1705,19 +2174,28 @@
 8. ใช้เทอร์มิเนเตอร์แบบ N-Series ที่มีความต้านทานทางไฟฟ้า 50 โอห์ม (บทที่ 3 หน้า 98-99)</t>
         </is>
       </c>
-      <c r="D53" s="7" t="n"/>
-      <c r="E53" s="8" t="n"/>
+      <c r="D53" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F53" s="10" t="inlineStr">
+        <is>
+          <t>ข้อกำหนด 8 ข้อครบตามบทสรุปใน net-3-19 หน้า 98-99</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="n">
+      <c r="A54" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B54" s="7" t="inlineStr">
         <is>
           <t>จงสรุปข้อกำหนดมาตรฐานอีเทอร์เน็ตแบบ 10Base2</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C54" s="7" t="inlineStr">
         <is>
           <t>ข้อกำหนดมาตรฐานอีเทอร์เน็ตแบบ 10Base2 คือ
 1. ส่งข้อมูลแบบเบสแบนด์
@@ -1730,19 +2208,28 @@
 8. ใช้เทอร์มิเนเตอร์ที่มีความต้านทานทางไฟฟ้า 50 โอห์ม ปิดปลายสายเคเบิลทั้งสองฝั่ง (บทที่ 3 หน้า 99-101)</t>
         </is>
       </c>
-      <c r="D54" s="7" t="n"/>
-      <c r="E54" s="8" t="n"/>
+      <c r="D54" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F54" s="10" t="inlineStr">
+        <is>
+          <t>ข้อกำหนด 8 ข้อครบตาม net-3-20 และ net-3-21 หน้า 99-101</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="n">
+      <c r="A55" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B55" s="6" t="inlineStr">
+      <c r="B55" s="7" t="inlineStr">
         <is>
           <t>จงสรุปข้อกำหนดมาตรฐานอีเทอร์เน็ตแบบ 10BaseT</t>
         </is>
       </c>
-      <c r="C55" s="6" t="inlineStr">
+      <c r="C55" s="7" t="inlineStr">
         <is>
           <t>ข้อกำหนดมาตรฐานอีเทอร์เน็ตแบบ 10BaseT คือ
 1. ส่งข้อมูลแบบเบสแบนด์
@@ -1754,19 +2241,28 @@
 7. ใช้การ์ดเครือข่ายที่มีช็อกเก็ตแบบ RJ-45 (บทที่ 3 หน้า 104)</t>
         </is>
       </c>
-      <c r="D55" s="7" t="n"/>
-      <c r="E55" s="8" t="n"/>
+      <c r="D55" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F55" s="10" t="inlineStr">
+        <is>
+          <t>ข้อกำหนด 7 ข้อครบตาม net-3-22 หน้า 104</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="n">
+      <c r="A56" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B56" s="6" t="inlineStr">
+      <c r="B56" s="7" t="inlineStr">
         <is>
           <t>สาเหตุใดที่เครือข่ายแบบ 10Base5 และ 10Base2 ในปัจจุบันไม่นิยมใช้แล้ว</t>
         </is>
       </c>
-      <c r="C56" s="6" t="inlineStr">
+      <c r="C56" s="7" t="inlineStr">
         <is>
           <t>เครือข่ายแบบ 10Base5 และ 10Base2 ไม่นิยมใช้แล้วเนื่องจากมีข้อจำกัดด้านการติดตั้งและการบำรุงรักษาที่สูง ทั้งสองรูปแบบใช้สายโคแอกเชียลที่มีขนาดหนา (10Base5) หรือบาง (10Base2) ซึ่งต้องติดตั้งโดยการเจาะสายเพื่อต่อทรานซีฟเวอร์หรือทีคอนเน็กเตอร์ ทำให้เสี่ยงต่อการเสียหายของสายและยากต่อการตรวจสอบจุดขัดข้อง (บทที่ 3 หน้า 97-98)
 นอกจากนี้ ระยะทางการเชื่อมต่อสูงสุดของแต่ละเซกเมนต์มีข้อจำกัด เช่น 10Base5 ใช้ระยะ 500 เมตร และ 10Base2 ใช้ระยะ 185 เมตร พร้อมกับข้อกำหนดเรื่องระยะห่างระหว่างโหนดที่ต้องห่างกันอย่างน้อย 2.5 เมตร (10Base5) หรือ 0.5 เมตร (10Base2) ทำให้การวางสายและจัดการเครือข่ายซับซ้อน (บทที่ 3 หน้า 98-99)
@@ -1774,19 +2270,28 @@
 ในปัจจุบัน 10BaseT ที่ใช้สายยูทีพีและเชื่อมต่อแบบดาวด้วยฮับ จึงได้รับความนิยมมากกว่า เพราะติดตั้งง่าย บำรุงรักษาง่าย และรองรับการขยายเครือข่ายได้ดีกว่า (บทที่ 3 หน้า 101-104)</t>
         </is>
       </c>
-      <c r="D56" s="7" t="n"/>
-      <c r="E56" s="8" t="n"/>
+      <c r="D56" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" s="10" t="inlineStr">
+        <is>
+          <t>เหตุผลบางส่วนอิงข้อจำกัดของบัสและระยะทางใน net-3-5 และ net-3-18 ถึง net-3-21 แต่เรื่องการเจาะสายและการบำรุงรักษาไม่มีในตำรา และไม่ได้กล่าวถึงข้อเสียหลักที่สายแกนขาดแล้วเครือข่ายหยุดทั้งระบบ</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="n">
+      <c r="A57" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B57" s="6" t="inlineStr">
+      <c r="B57" s="7" t="inlineStr">
         <is>
           <t>สวิตซ์อีเทอร์เน็ตมีความคล้ายและแตกต่างจาก 10BaseT อย่างไร จงอธิบาย</t>
         </is>
       </c>
-      <c r="C57" s="6" t="inlineStr">
+      <c r="C57" s="7" t="inlineStr">
         <is>
           <t>สวิตซ์อีเทอร์เน็ตมีความคล้ายกับ 10BaseT ตรงที่ทั้งสองใช้มาตรฐานเครือข่าย 802.3 และส่งข้อมูลด้วยความเร็ว 10 เมกะบิตต่อวินาที ใช้สายยูทีพี (UTP) รหัส CAT-3 หรือ CAT-5 และใช้การ์ดเครือข่ายที่มีช็อกเก็ตแบบ RJ-45
 ความแตกต่างคือ 10BaseT ใช้อุปกรณ์ฮับ (Hub) เป็นศูนย์กลางในการกระจายข้อมูลไปยังทุกพอร์ต ทำให้เกิดการแพร่สัญญาณไปยังทุกโหนด แม้จะไม่ได้ต้องการ (บทที่ 3 หน้า 104) ส่วนสวิตซ์อีเทอร์เน็ตใช้อุปกรณ์สวิตช์แทนฮับ ซึ่งสามารถส่งข้อมูลไปยังพอร์ตที่ต้องการได้เฉพาะจุด ทำให้การส่งข้อมูลมีประสิทธิภาพและรวดเร็วขึ้น (บทที่ 3 หน้า 104)
@@ -1794,19 +2299,28 @@
 สวิตซ์อีเทอร์เน็ตสามารถจัดการการสื่อสารได้ดีกว่าฮับ เพราะไม่ส่งข้อมูลไปยังทุกพอร์ตโดยไม่จำเป็น ลดการชนกันของแพ็กเก็ตและเพิ่มประสิทธิภาพการใช้แบนด์วิธ</t>
         </is>
       </c>
-      <c r="D57" s="7" t="n"/>
-      <c r="E57" s="8" t="n"/>
+      <c r="D57" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F57" s="10" t="inlineStr">
+        <is>
+          <t>สวิตซ์อีเทอร์เน็ตคือ 10BaseT ที่ใช้สวิตช์แทนฮับ ส่งไปยังพอร์ตที่ต้องการได้ ตรงกับ net-3-22 หน้า 104</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="n">
+      <c r="A58" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B58" s="6" t="inlineStr">
+      <c r="B58" s="7" t="inlineStr">
         <is>
           <t>อีเทอร์เน็ตความเร็วสูงรับส่งข้อมูลด้วยความเร็วเท่าใด และมีความแตกต่างจาก 10BaseT อย่างไร จงอธิบาย</t>
         </is>
       </c>
-      <c r="C58" s="6" t="inlineStr">
+      <c r="C58" s="7" t="inlineStr">
         <is>
           <t>อีเทอร์เน็ตความเร็วสูงสามารถรับส่งข้อมูลได้สูงสุดถึง 100 เมกะบิตต่อวินาทีในรูปแบบ Fast Ethernet และสูงสุดถึง 1,000 เมกะบิตต่อวินาทีหรือ 1 กิกะบิตต่อวินาทีในรูปแบบ Gigabit Ethernet
 ความแตกต่างจาก 10BaseT คือ 10BaseT ส่งข้อมูลด้วยความเร็ว 10 เมกะบิตต่อวินาที ใช้สายยูทีพี (CAT-3 หรือ CAT-5) และเชื่อมต่อผ่านฮับ ในขณะที่อีเทอร์เน็ตความเร็วสูงใช้การ์ดเครือข่ายความเร็วสูง ใช้สวิตช์แทนฮับ และสามารถใช้สายใยแก้วนำแสงได้ (บทที่ 3 หน้า 104)
@@ -1816,19 +2330,28 @@
 อีเทอร์เน็ตความเร็วสูงจึงเร็วกว่า 10BaseT หลายเท่า และใช้เทคโนโลยีที่ทันสมัยกว่า เช่น การใช้สวิตช์แทนฮับ ทำให้การส่งข้อมูลมีประสิทธิภาพมากขึ้น (บทที่ 3 หน้า 104)</t>
         </is>
       </c>
-      <c r="D58" s="7" t="n"/>
-      <c r="E58" s="8" t="n"/>
+      <c r="D58" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F58" s="10" t="inlineStr">
+        <is>
+          <t>Fast Ethernet 100 เมกะบิตต่อวินาที ใช้การ์ด 100 หรือ 10/100 และสวิตช์ ตรงกับ net-3-22 หน้า 104</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="n">
+      <c r="A59" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B59" s="6" t="inlineStr">
+      <c r="B59" s="7" t="inlineStr">
         <is>
           <t>จงอธิบายกลไกการส่งข้อมูลด้วย Token Passing มาให้พอเข้าใจ</t>
         </is>
       </c>
-      <c r="C59" s="6" t="inlineStr">
+      <c r="C59" s="7" t="inlineStr">
         <is>
           <t>กลไกการส่งข้อมูลด้วย Token Passing คือการที่ในช่วงเวลาหนึ่งจะมีเพียงโหนดเดียวที่สามารถส่งข้อมูลได้ ซึ่งก็คือโหนดที่ครอบครองโทเค็น
 โทเค็นจะวิ่งไปตามวงแหวนของเครือข่าย และโหนดใดได้รับโทเค็นก่อนก็จะสามารถส่งข้อมูลได้ทันที
@@ -1843,19 +2366,28 @@
 การใช้สองวงแหวนช่วยให้เครือข่ายยังคงดำเนินการได้ตามปกติแม้เกิดความเสียหาย (บทที่ 3 หน้า 107-108)</t>
         </is>
       </c>
-      <c r="D59" s="7" t="n"/>
-      <c r="E59" s="8" t="n"/>
+      <c r="D59" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F59" s="10" t="inlineStr">
+        <is>
+          <t>กลไก Token Passing ตรงกับ net-3-23 และ net-3-24 หน้า 105-107</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="n">
+      <c r="A60" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="B60" s="7" t="inlineStr">
         <is>
           <t>วงแหวนปฐมภูมิและวงแหวนทุติยภูมิบนเครือข่ายเอฟดีดีไอมีไว้เพื่ออะไร</t>
         </is>
       </c>
-      <c r="C60" s="6" t="inlineStr">
+      <c r="C60" s="7" t="inlineStr">
         <is>
           <t>วงแหวนปฐมภูมิ (Primary Ring) คือวงแหวนหลักด้านนอกที่ใช้เป็นสายส่งข้อมูลหลักภายในเครือข่ายเอฟดีดีไอ โดยรหัสโทเค็นจะวิ่งรอบวงแหวนทิศทางใดทิศทางหนึ่ง
 วงแหวนทุติยภูมิ (Secondary Ring) คือวงแหวนสำรองที่อยู่ด้านใน โทเค็นที่อยู่วงแหวนด้านในจะวิ่งในทิศทางตรงกันข้ามกับวงแหวนด้านนอก และจะถูกใช้งานเมื่อวงแหวนปฐมภูมิเกิดปัญหา เช่น สายเคเบิลขาด ทำให้เครือข่ายยังคงทำงานต่อไปได้ (บทที่ 3 หน้า 106-107)
@@ -1863,19 +2395,28 @@
 การมีทั้งสองวงแหวนช่วยให้เครือข่ายเอฟดีดีไอสามารถทนต่อความเสียหายของสายเคเบิลได้ และยังคงรักษาการสื่อสารข้อมูลต่อเนื่อง (บทที่ 3 หน้า 106-107)</t>
         </is>
       </c>
-      <c r="D60" s="7" t="n"/>
-      <c r="E60" s="8" t="n"/>
+      <c r="D60" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F60" s="10" t="inlineStr">
+        <is>
+          <t>วงแหวนหลักส่งข้อมูลและวงแหวนสำรองใช้เมื่อวงหลักมีปัญหา ตรงกับ net-3-24 หน้า 106-107</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="6" t="n">
+      <c r="A61" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B61" s="6" t="inlineStr">
+      <c r="B61" s="7" t="inlineStr">
         <is>
           <t>กลไกการทำงานของวงแหวนทุติยภูมิจะทำงานอย่างไร เมื่อวงแหวนปฐมภูมิเกิดขาดหรือเสียหายขึ้นมา จงอธิบาย</t>
         </is>
       </c>
-      <c r="C61" s="6" t="inlineStr">
+      <c r="C61" s="7" t="inlineStr">
         <is>
           <t>เมื่อวงแหวนปฐมภูมิเกิดขาดหรือเสียหาย วงแหวนทุติยภูมิจะทำงานเป็นวงแหวนสำรอง โดยเริ่มเชื่อมต่อกับวงแหวนปฐมภูมิทันทีเพื่อให้เกิดวงรอบใหม่ ทำให้โทเค็นสามารถวิ่งรอบภายในวงแหวนได้เช่นเดิม ซึ่งช่วยให้เครือข่ายยังคงดำเนินการได้ตามปกติ
 วงแหวนทุติยภูมิจะวิ่งในทิศทางตรงกันข้ามกับวงแหวนปฐมภูมิ และเมื่อเกิดเหตุการณ์ขาดสายในวงแหวนปฐมภูมิ ระบบจะสลับไปใช้วงแหวนทุติยภูมิทันที ทำให้การส่งข้อมูลยังคงดำเนินต่อไปได้ (บทที่ 3 หน้า 106-107)
@@ -1884,57 +2425,84 @@
 ระบบดังกล่าวช่วยเพิ่มความทนทานต่อความเสียหายของสายเคเบิล โดยเฉพาะในเครือข่ายเอฟดีดีไอที่ออกแบบมาให้รองรับความเสียหายได้</t>
         </is>
       </c>
-      <c r="D61" s="7" t="n"/>
-      <c r="E61" s="8" t="n"/>
+      <c r="D61" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F61" s="10" t="inlineStr">
+        <is>
+          <t>วงแหวนทุติยภูมิเชื่อมต่อเข้ากับวงแหวนปฐมภูมิให้โทเค็นวิ่งครบรอบได้ ตรงกับ net-3-24 และ net-3-25 หน้า 106-108</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="n">
+      <c r="A62" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B62" s="6" t="inlineStr">
+      <c r="B62" s="7" t="inlineStr">
         <is>
           <t>โทโปโลยีแบบดาวใช้อุปกรณ์อะไรเป็นศูนย์กลาง</t>
         </is>
       </c>
-      <c r="C62" s="6" t="inlineStr">
+      <c r="C62" s="7" t="inlineStr">
         <is>
           <t>โทโปโลยีแบบดาวใช้อุปกรณ์ฮับ (Hub) เป็นศูนย์กลางการเชื่อมต่อของเครือข่ายทั้งหมด
 ฮับทำหน้าที่เป็นจุดรวมสายเคเบิลจากคอมพิวเตอร์ทุกโหนดในเครือข่าย
 หากฮับเสียหาย เครือข่ายทั้งระบบจะหยุดทำงานทันที (บทที่ 3 หน้า 87-88)</t>
         </is>
       </c>
-      <c r="D62" s="7" t="n"/>
-      <c r="E62" s="8" t="n"/>
+      <c r="D62" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F62" s="10" t="inlineStr">
+        <is>
+          <t>ฮับเป็นศูนย์กลาง ตรงกับ net-3-6 หน้า 87-88</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="6" t="n">
+      <c r="A63" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B63" s="6" t="inlineStr">
+      <c r="B63" s="7" t="inlineStr">
         <is>
           <t>โทโปโลยีแบบวงแหวนมีข้อเสียอย่างไร</t>
         </is>
       </c>
-      <c r="C63" s="6" t="inlineStr">
+      <c r="C63" s="7" t="inlineStr">
         <is>
           <t>โทโปโลยีแบบวงแหวนมีข้อเสียดังนี้
 • สายเคเบิลที่ใช้เป็นวงแหวน หากเกิดชำรุดเสียหาย เครือข่ายจะหยุดการทำงานลง
 • หากมีบางโหนดบนเครือข่ายเกิดขัดข้อง จะยากต่อการตรวจสอบและค้นหาโหนดที่เสีย (บทที่ 3 หน้า 89-90)</t>
         </is>
       </c>
-      <c r="D63" s="7" t="n"/>
-      <c r="E63" s="8" t="n"/>
+      <c r="D63" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F63" s="10" t="inlineStr">
+        <is>
+          <t>ข้อเสีย 2 ข้อครบตาม net-3-7 หน้า 89-90</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="n">
+      <c r="A64" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B64" s="6" t="inlineStr">
+      <c r="B64" s="7" t="inlineStr">
         <is>
           <t>จงสรุปคุณสมบัติของเครือข่ายแบบเวิร์กกรุ๊ป</t>
         </is>
       </c>
-      <c r="C64" s="6" t="inlineStr">
+      <c r="C64" s="7" t="inlineStr">
         <is>
           <t>เครือข่ายแบบเวิร์กกรุ๊ปมีคุณสมบัติดังนี้
 - ต้นทุนในการจัดการต่ำ ไม่จำเป็นต้องพึ่งพาผู้เชี่ยวชาญ ก็สามารถทำได้
@@ -1946,19 +2514,28 @@
 - คอมพิวเตอร์บนเวิร์กกรุ๊ปจะต้องอยู่ภายในเครือข่ายเดียวกัน (บทที่ 4 หน้า 130-131)</t>
         </is>
       </c>
-      <c r="D64" s="7" t="n"/>
-      <c r="E64" s="8" t="n"/>
+      <c r="D64" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F64" s="10" t="inlineStr">
+        <is>
+          <t>คุณสมบัติ 7 ข้อครบตาม net-4-6 หน้า 130-131</t>
+        </is>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="n">
+      <c r="A65" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B65" s="6" t="inlineStr">
+      <c r="B65" s="7" t="inlineStr">
         <is>
           <t>จงสรุปคุณสมบัติของเครือข่ายแบบโดเมน</t>
         </is>
       </c>
-      <c r="C65" s="6" t="inlineStr">
+      <c r="C65" s="7" t="inlineStr">
         <is>
           <t>คุณสมบัติของเครือข่ายแบบโดเมน ได้แก่
 - ต้นทุนในการจัดการสูง ต้องพึ่งพาผู้เชี่ยวชาญด้านเครือข่าย
@@ -1970,19 +2547,28 @@
 - คอมพิวเตอร์ที่ใช้งานบนเครือข่ายสามารถอยู่คนละเครือข่ายกันได้ (บทที่ 4 หน้า 131-132)</t>
         </is>
       </c>
-      <c r="D65" s="7" t="n"/>
-      <c r="E65" s="8" t="n"/>
+      <c r="D65" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F65" s="10" t="inlineStr">
+        <is>
+          <t>คุณสมบัติ 7 ข้อครบตาม net-4-7 และ net-4-8 หน้า 131-132</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="n">
+      <c r="A66" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B66" s="6" t="inlineStr">
+      <c r="B66" s="7" t="inlineStr">
         <is>
           <t>หากต้องการสร้างสายแลนชนิด RJ-45 แบบเชื่อมต่อตรง สามารถเชื่อมต่อด้วยการเรียงสีสายสัญญาณตามมาตรฐานใด</t>
         </is>
       </c>
-      <c r="C66" s="6" t="inlineStr">
+      <c r="C66" s="7" t="inlineStr">
         <is>
           <t>หากต้องการสร้างสายแลนชนิด RJ-45 แบบเชื่อมต่อตรง สามารถเชื่อมต่อด้วยการเรียงสีสายสัญญาณตามมาตรฐาน T568A หรือ T568B ก็ได้ แต่ต้องใช้มาตรฐานเดียวกันทั้งสองปลายของสาย
 การจัดเรียงสีตามมาตรฐาน T568A คือ ขาวเขียว/เขียว, ขาวส้ม/น้ำเงิน, ขาวน้ำเงิน/ส้ม, ขาวน้ำตาล/น้ำตาล
@@ -1992,19 +2578,28 @@
 ทั้งสองมาตรฐานนี้ใช้ได้กับสายต่อตรง (Straight Through) ซึ่งเหมาะสำหรับการเชื่อมต่อระหว่างคอมพิวเตอร์กับฮับหรือสวิตช์ โดยไม่ต้องสลับสาย</t>
         </is>
       </c>
-      <c r="D66" s="7" t="n"/>
-      <c r="E66" s="8" t="n"/>
+      <c r="D66" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F66" s="10" t="inlineStr">
+        <is>
+          <t>สายต่อตรงใช้ T568A หรือ T568B ก็ได้แต่ต้องเหมือนกันทั้งสองปลาย ตรงกับ net-4-4 หน้า 129 และ net-4-27</t>
+        </is>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="6" t="n">
+      <c r="A67" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B67" s="6" t="inlineStr">
+      <c r="B67" s="7" t="inlineStr">
         <is>
           <t>หากต้องการสร้างสายแลนชนิด RJ-45 แบบไขว้ จะต้องเรียงสีที่ปลายสายทั้งสองฝั่งด้วยมาตรฐานใด</t>
         </is>
       </c>
-      <c r="C67" s="6" t="inlineStr">
+      <c r="C67" s="7" t="inlineStr">
         <is>
           <t>หากต้องการสร้างสายแลนชนิด RJ-45 แบบไขว้ จะต้องเรียงสีที่ปลายสายทั้งสองฝั่งด้วยมาตรฐาน T568A และ T568B
 ปลายสายหนึ่งต้องใช้มาตรฐาน T568A ส่วนอีกปลายต้องใช้มาตรฐาน T568B (บทที่ 4 หน้า 129)
@@ -2013,19 +2608,28 @@
 การใช้มาตรฐานทั้งสองฝั่งนี้จะทำให้สายแลนทำงานในรูปแบบไขว้ (Crossover) ตามที่ต้องการ (บทที่ 4 หน้า 129)</t>
         </is>
       </c>
-      <c r="D67" s="7" t="n"/>
-      <c r="E67" s="8" t="n"/>
+      <c r="D67" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F67" s="10" t="inlineStr">
+        <is>
+          <t>สายไขว้ปลายหนึ่ง T568A อีกปลาย T568B ตรงกับ net-4-4 หน้า 129</t>
+        </is>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" s="6" t="n">
+      <c r="A68" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B68" s="6" t="inlineStr">
+      <c r="B68" s="7" t="inlineStr">
         <is>
           <t>ในระบบปฏิบัติการ Windows 7 หากกำหนดเงื่อนไขการแชร์ตรงส่วนของ Public Folder Sharing ด้วยการตั้งค่าเป็น Turn On หมายความว่าอย่างไร แล้วผลที่ได้จากการตั้งค่าในครั้งนี้ คืออะไร จงอธิบาย</t>
         </is>
       </c>
-      <c r="C68" s="6" t="inlineStr">
+      <c r="C68" s="7" t="inlineStr">
         <is>
           <t>การตั้งค่า Turn on Public folder sharing ในระบบปฏิบัติการ Windows 7 หมายความว่า เปิดการแชร์โฟลเดอร์ Public บนเครื่องนั้นให้สามารถเข้าถึงได้จากเครื่องอื่นในเวิร์กกรุ๊ปโดยไม่ต้องใช้รหัสผ่าน (บทที่ 4 หน้า 139-141)
 ผลที่ได้จากการตั้งค่านี้คือ เครื่องอื่นในเครือข่ายเดียวกันสามารถเข้าถึงโฟลเดอร์ Public บนเครื่องนั้นได้ทั้งในการอ่านและเขียนไฟล์ รวมถึงสามารถเข้าถึงโฟลเดอร์ย่อยต่างๆ เช่น Public Documents, Public Music, Public Pictures ฯลฯ ได้ทันที (บทที่ 4 หน้า 165-166)
@@ -2034,19 +2638,28 @@
 การตั้งค่า Turn on ทำให้ไม่ต้องพิมพ์ชื่อผู้ใช้และรหัสผ่านเมื่อเข้าถึงไฟล์จากเครื่องอื่น แต่ลดระดับความปลอดภัยลง</t>
         </is>
       </c>
-      <c r="D68" s="7" t="n"/>
-      <c r="E68" s="8" t="n"/>
+      <c r="D68" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F68" s="10" t="inlineStr">
+        <is>
+          <t>เปิดให้เครื่องในเวิร์กกรุ๊ปเข้าถึงโฟลเดอร์ Public อ่านและเขียนได้เต็มสิทธิ์ ตรงกับ net-4-13 หน้า 139-141 และ net-4-28</t>
+        </is>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="6" t="n">
+      <c r="A69" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B69" s="6" t="inlineStr">
+      <c r="B69" s="7" t="inlineStr">
         <is>
           <t>หมายเลขไอพี (IP Address) คืออะไร มีส่วนสำคัญอย่างไร จงอธิบาย</t>
         </is>
       </c>
-      <c r="C69" s="6" t="inlineStr">
+      <c r="C69" s="7" t="inlineStr">
         <is>
           <t>หมายเลขไอพี (IP Address) คือชุดหมายเลขที่ใช้อ้างอิงตำแหน่งที่อยู่ของคอมพิวเตอร์และอุปกรณ์บนเครือข่ายอินเทอร์เน็ตที่ใช้โปรโตคอล TCP/IP (บทที่ 4 หน้า 166)
 หมายเลขไอพีมีส่วนสำคัญในการระบุตำแหน่งของอุปกรณ์ในเครือข่าย เพื่อให้สามารถส่งข้อมูลไปยังอุปกรณ์ปลายทางได้อย่างถูกต้อง โดยต้องไม่ซ้ำกันในเครือข่ายเดียวกัน (บทที่ 4 หน้า 141-142)
@@ -2063,19 +2676,28 @@
 หลังตั้งค่าแล้ว สามารถทดสอบการสื่อสารระหว่างเครื่องในเครือข่ายได้โดยใช้คำสั่ง ping พร้อมระบุหมายเลขไอพีของเครื่องปลายทาง หากได้รับการตอบกลับ แสดงว่าเครื่องทั้งสองสามารถสื่อสารกันได้ (บทที่ 4 หน้า 166-167)</t>
         </is>
       </c>
-      <c r="D69" s="7" t="n"/>
-      <c r="E69" s="8" t="n"/>
+      <c r="D69" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E69" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F69" s="10" t="inlineStr">
+        <is>
+          <t>ความหมายและความสำคัญตรงกับ net-4-14 หน้า 141-142 และ net-4-29 หน้า 166 ส่วนคลาสตรงกับ net-4-15 และ net-4-16</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="6" t="n">
+      <c r="A70" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B70" s="6" t="inlineStr">
+      <c r="B70" s="7" t="inlineStr">
         <is>
           <t>ฟิลด์หลักๆ ภายในหมายเลขไอพีประกอบด้วยฟิลด์อะไรบ้าง จงอธิบาย</t>
         </is>
       </c>
-      <c r="C70" s="6" t="inlineStr">
+      <c r="C70" s="7" t="inlineStr">
         <is>
           <t>ฟิลด์หลักๆ ภายในหมายเลขไอพีประกอบด้วย 3 ฟิลด์ ได้แก่
 1. ประเภทของคลาส — เป็นคลาสที่ใช้ระบุหมายเลขไอพี เพื่อให้รู้ว่าหมายเลขไอพีแอดเดรสนี้อยู่ในคลาสใด
@@ -2083,19 +2705,28 @@
 3. หมายเลขโฮสต์ (HostID) — เป็นส่วนที่ใช้ระบุตำแหน่งของอุปกรณ์หรือโฮสต์บนเครือข่าย (บทที่ 4 หน้า 141-142)</t>
         </is>
       </c>
-      <c r="D70" s="7" t="n"/>
-      <c r="E70" s="8" t="n"/>
+      <c r="D70" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F70" s="10" t="inlineStr">
+        <is>
+          <t>3 ฟิลด์ (ประเภทของคลาส NetID HostID) พร้อมคำอธิบายตรงกับ net-4-14 หน้า 141-142</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="6" t="n">
+      <c r="A71" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B71" s="6" t="inlineStr">
+      <c r="B71" s="7" t="inlineStr">
         <is>
           <t>จงระบุช่วงแอดเดรสของหมายเลขไอพีคลาส A, B และ C พร้อมชุดหมายเลขไอพีแบบภายใน</t>
         </is>
       </c>
-      <c r="C71" s="6" t="inlineStr">
+      <c r="C71" s="7" t="inlineStr">
         <is>
           <t>ช่วงแอดเดรสของหมายเลขไอพีคลาส A คือ 0.0.0.0 ถึง 127.255.255.255
 ช่วงแอดเดรสของหมายเลขไอพีคลาส B คือ 128.0.0.0 ถึง 191.255.255.255
@@ -2106,19 +2737,28 @@
 • คลาส C 192.168.0.0 ถึง 192.168.255.255 (บทที่ 4 หน้า 143-144)</t>
         </is>
       </c>
-      <c r="D71" s="7" t="n"/>
-      <c r="E71" s="8" t="n"/>
+      <c r="D71" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F71" s="10" t="inlineStr">
+        <is>
+          <t>ช่วงแอดเดรสคลาส A B C และไอพีภายในตรงกับ net-4-15 และ net-4-16 หน้า 142-144</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="6" t="n">
+      <c r="A72" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B72" s="6" t="inlineStr">
+      <c r="B72" s="7" t="inlineStr">
         <is>
           <t>การกำหนดชื่อเวิร์กกรุ๊ปบนเครือข่าย ทำไมจึงต้องกำหนดชื่อให้ตรงกัน</t>
         </is>
       </c>
-      <c r="C72" s="6" t="inlineStr">
+      <c r="C72" s="7" t="inlineStr">
         <is>
           <t>การกำหนดชื่อเวิร์กกรุ๊ปบนเครือข่ายต้องกำหนดให้ตรงกัน เพื่อให้คอมพิวเตอร์ทุกเครื่องในเครือข่ายสามารถรับรู้และเชื่อมต่อกันได้อย่างถูกต้อง ซึ่งเป็นข้อกำหนดสำคัญในการจัดการเครือข่ายเวิร์กกรุ๊ปให้ทำงานร่วมกันได้
 หากชื่อเวิร์กกรุ๊ปไม่ตรงกัน เครื่องคอมพิวเตอร์จะไม่สามารถมองเห็นหรือเชื่อมต่อกันได้ในเครือข่ายเดียวกัน
@@ -2127,19 +2767,28 @@
 การตั้งชื่อเวิร์กกรุ๊ปให้ตรงกันเป็นสิ่งจำเป็นในเครือข่ายแบบเพียร์ทูเพียร์ (Peer-to-Peer) เพื่อให้ระบบสามารถจัดกลุ่มเครื่องคอมพิวเตอร์ที่ต้องการใช้งานร่วมกันได้อย่างถูกต้อง</t>
         </is>
       </c>
-      <c r="D72" s="7" t="n"/>
-      <c r="E72" s="8" t="n"/>
+      <c r="D72" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" s="10" t="inlineStr">
+        <is>
+          <t>ตำรา (net-4-18 หน้า 146 และ net-4-28 หน้า 165-166) ระบุเพียงว่าต้องตั้งชื่อเวิร์กกรุ๊ปให้ตรงกัน ส่วนที่ว่าถ้าไม่ตรงจะมองไม่เห็นหรือเชื่อมต่อกันไม่ได้ไม่มีในตำรา</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="6" t="n">
+      <c r="A73" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B73" s="6" t="inlineStr">
+      <c r="B73" s="7" t="inlineStr">
         <is>
           <t>จะทราบได้อย่างไรว่า บนเครือข่ายเวิร์กกรุ๊ปในขณะนั้น มีเครื่องใดบ้างที่เชื่อมต่ออยู่</t>
         </is>
       </c>
-      <c r="C73" s="6" t="inlineStr">
+      <c r="C73" s="7" t="inlineStr">
         <is>
           <t>สามารถทราบได้ว่ามีเครื่องใดบ้างที่เชื่อมต่ออยู่บนเครือข่ายเวิร์กกรุ๊ป โดยการใช้โปรแกรมประยุกต์ที่แสดงรายชื่อเครื่องคอมพิวเตอร์บนเครือข่าย ซึ่งจะแสดงเครื่องที่อยู่ในเครือข่ายเดียวกัน เช่น COMPUTER1, COMPUTER2, COMPUTER3 เป็นต้น
 เมื่อเปิดโปรแกรมดังกล่าว จะปรากฏรายการเครื่องคอมพิวเตอร์ที่เชื่อมต่ออยู่ในเฟรมด้านซ้าย ซึ่งสามารถคลิกที่ชื่อเครื่องเพื่อดูรายละเอียดต่างๆ ได้
@@ -2147,19 +2796,28 @@
 หากต้องการจัดเรียงลำดับชื่อเครื่อง ให้คลิกขวาที่โฟลเดอร์ ALL COMPUTERS แล้วเลือก ALL COMPUTER® รายการ Sort Items (บทที่ 7 หน้า 280-281)</t>
         </is>
       </c>
-      <c r="D73" s="7" t="n"/>
-      <c r="E73" s="8" t="n"/>
+      <c r="D73" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="10" t="inlineStr">
+        <is>
+          <t>ตำราตอบไว้ใน net-4-20 หน้า 150 ว่าเปิดหน้าต่าง Computer แล้วคลิกหัวข้อ Network แต่คำตอบไปหยิบขั้นตอนของโปรแกรม Alchemy ใน net-7-15 หน้า 280-281 มาแทน</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="6" t="n">
+      <c r="A74" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B74" s="6" t="inlineStr">
+      <c r="B74" s="7" t="inlineStr">
         <is>
           <t>สาเหตุใดที่เครือข่ายแบบเวิร์กกรุ๊ป ไม่เหมาะกับการเชื่อมต่อเครื่องลูกข่ายจำนวนมากๆ</t>
         </is>
       </c>
-      <c r="C74" s="6" t="inlineStr">
+      <c r="C74" s="7" t="inlineStr">
         <is>
           <t>เครือข่ายแบบเวิร์กกรุ๊ปไม่เหมาะกับการเชื่อมต่อเครื่องลูกข่ายจำนวนมากมายนั้น เพราะมีจำนวนเครื่องที่เชื่อมต่อมีจำนวนจำกัด (ไม่ควรเกินกว่า 20 เครื่อง) (บทที่ 4 หน้า 130-131)
 นอกจากนี้ ระบบความปลอดภัยของเครือข่ายเวิร์กกรุ๊ปมีข้อจำกัดและค่อนข้างต่ำ ทำให้ควบคุมการเข้าถึงทรัพยากรได้ยากเมื่อจำนวนเครื่องเพิ่มขึ้น (บทที่ 4 หน้า 130)
@@ -2169,19 +2827,28 @@
 เครือข่ายแบบเวิร์กกรุ๊ปไม่มีศูนย์กลางในการจัดการข้อมูล ทำให้การควบคุมและตรวจสอบระบบทำได้ยากเมื่อขยายขนาดเครือข่าย</t>
         </is>
       </c>
-      <c r="D74" s="7" t="n"/>
-      <c r="E74" s="8" t="n"/>
+      <c r="D74" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F74" s="10" t="inlineStr">
+        <is>
+          <t>จำกัดไม่เกิน 20 เครื่อง ความปลอดภัยต่ำ และบัญชีผู้ใช้กระจายตามเครื่อง ตรงกับ net-4-5 และ net-4-6 หน้า 130-131</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="6" t="n">
+      <c r="A75" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B75" s="6" t="inlineStr">
+      <c r="B75" s="7" t="inlineStr">
         <is>
           <t>การที่เวิร์กกรุ๊ปหรือเครือข่ายเพียร์ทูเพียร์นั้น ทุกๆ เครื่องมีสิทธิ์เท่าเทียมกันทั้งหมดนั่นหมายความว่าอย่างไร</t>
         </is>
       </c>
-      <c r="C75" s="6" t="inlineStr">
+      <c r="C75" s="7" t="inlineStr">
         <is>
           <t>การที่เวิร์กกรุ๊ปหรือเครือข่ายเพียร์ทูเพียร์มีเครื่องทุกเครื่องมีสิทธิ์เท่าเทียมกัน หมายความว่า ไม่มีเครื่องใดเป็นศูนย์กลางหรือควบคุมเครื่องอื่นๆ โดยทุกเครื่องสามารถทำหน้าที่เป็นทั้งผู้ให้บริการ (Server) และผู้รับบริการ (Client) ได้ในเวลาเดียวกัน (บทที่ 3 หน้า 90-91)
 ทุกเครื่องมีสิทธิ์เท่าเทียมกันทั้งหมด ไม่มีเครื่องใดควบคุมคอมพิวเตอร์เครื่องอื่นๆ
@@ -2190,19 +2857,28 @@
 เครือข่ายประเภทนี้เหมาะกับการแชร์ไฟล์และทรัพยากรในกลุ่มเล็กๆ โดยไม่ต้องใช้ผู้ดูแลระบบหรือเครื่องเชิร์ฟเวอร์เฉพาะ (บทที่ 3 หน้า 91-92)</t>
         </is>
       </c>
-      <c r="D75" s="7" t="n"/>
-      <c r="E75" s="8" t="n"/>
+      <c r="D75" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E75" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F75" s="10" t="inlineStr">
+        <is>
+          <t>ไม่มีเครื่องใดควบคุมเครื่องอื่น เป็นได้ทั้งเซิร์ฟเวอร์และไคลเอ็นต์ ตรงกับ net-4-5 หน้า 130 และ net-3-9 หน้า 90-91</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="6" t="n">
+      <c r="A76" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B76" s="6" t="inlineStr">
+      <c r="B76" s="7" t="inlineStr">
         <is>
           <t>ทำไมการจัดการบัญชีผู้ใช้บนเครือข่ายแบบโดเมน มีความสะดวกกว่าแบบเวิร์กกรุ๊ป</t>
         </is>
       </c>
-      <c r="C76" s="6" t="inlineStr">
+      <c r="C76" s="7" t="inlineStr">
         <is>
           <t>การจัดการบัญชีผู้ใช้บนเครือข่ายแบบโดเมนสะดวกกว่าแบบเวิร์กกรุ๊ปเพราะบัญชีผู้ใช้จะถูกจัดเก็บไว้ในศูนย์กลางที่เรียกว่า โดเมนคอนโทรลเลอร์ (Domain Controller) ทำให้ผู้ดูแลระบบสามารถจัดการและควบคุมบัญชีผู้ใช้ทั้งหมดได้จากเครื่องเซิร์ฟเวอร์เพียงเครื่องเดียว (บทที่ 4 หน้า 131)
 ในขณะที่เครือข่ายแบบเวิร์กกรุ๊ปต้องสร้างบัญชีผู้ใช้กระจายอยู่ตามเครื่องต่างๆ ทำให้ต้องจัดการทีละเครื่อง ซึ่งยุ่งยากและเสี่ยงต่อความผิดพลาด (บทที่ 5 หน้า 176)
@@ -2211,19 +2887,28 @@
 ดังนั้น การจัดการบัญชีผู้ใช้ในเครือข่ายแบบโดเมนจึงมีประสิทธิภาพและควบคุมได้ง่ายกว่า (บทที่ 4 หน้า 131)</t>
         </is>
       </c>
-      <c r="D76" s="7" t="n"/>
-      <c r="E76" s="8" t="n"/>
+      <c r="D76" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E76" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F76" s="10" t="inlineStr">
+        <is>
+          <t>บัญชีผู้ใช้เก็บที่โดเมนคอนโทรลเลอร์ จัดการได้จากเซิร์ฟเวอร์เครื่องเดียว ตรงกับ net-4-7 หน้า 131 และ net-5-2 หน้า 176</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" s="6" t="n">
+      <c r="A77" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B77" s="6" t="inlineStr">
+      <c r="B77" s="7" t="inlineStr">
         <is>
           <t>คำสั่ง ping เป็นคำสั่งที่นำมาใช้เพื่อทดสอบอะไรบนเครือข่าย</t>
         </is>
       </c>
-      <c r="C77" s="6" t="inlineStr">
+      <c r="C77" s="7" t="inlineStr">
         <is>
           <t>คำสั่ง ping เป็นคำสั่งที่นำมาใช้เพื่อทดสอบการสื่อสารระหว่างเครื่องบนเครือข่าย ภายหลังจากการกำหนดโปรโตคอล TCP/IP พร้อมกำหนดหมายเลขไอพีให้กับเครื่องต่างๆ บนเครือข่ายแล้ว หากต้องการทดสอบว่าเครื่องบนเครือข่ายสามารถสื่อสารกันได้หรือไม่ ก็ให้ใช้คำสั่งนี้พร้อมระบุที่อยู่/หมายเลขไอพีของเครื่องปลายทาง หากเครื่องปลายทางตอบรับกลับมา นั่นหมายความว่าเครื่องทั้งสองสามารถสื่อสารกันได้แล้ว (บทที่ 4 หน้า 166-167)
 การทดสอบการสื่อสารกับเครื่องอื่นๆ บนเครือข่ายด้วยคำสั่ง ping เมื่อได้ดำเนินการมาถึง ณ จุดนี้ สิ่งที่ได้ดำเนินกับเครื่องทั้งสองคือ
@@ -2243,19 +2928,28 @@
 ขณะเดียวกัน ที่เครื่อง COMPUTER2 ก็สามารถติดต่อกับเครื่อง COMPUTER1 ได้เช่นกัน (บทที่ 4 หน้า 149-150)</t>
         </is>
       </c>
-      <c r="D77" s="7" t="n"/>
-      <c r="E77" s="8" t="n"/>
+      <c r="D77" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F77" s="10" t="inlineStr">
+        <is>
+          <t>ping ใช้ทดสอบการสื่อสารระหว่างเครื่องบนเครือข่าย ตรงกับ net-4-30 หน้า 166-167 และ net-4-19 หน้า 149-150</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="6" t="n">
+      <c r="A78" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B78" s="6" t="inlineStr">
+      <c r="B78" s="7" t="inlineStr">
         <is>
           <t>เครื่องพิมพ์แบบระยะไกลหรือ Remote Printer หมายถึงเครื่องพิมพ์แบบใด จงอธิบาย</t>
         </is>
       </c>
-      <c r="C78" s="6" t="inlineStr">
+      <c r="C78" s="7" t="inlineStr">
         <is>
           <t>ผมยืนยันคำตอบเรื่องนี้กับหนังสือคู่มือเรียนเครือข่ายคอมพิวเตอร์เบื้องต้นไม่ได้ คำตอบต่อไปนี้มาจากความรู้ทั่วไปของ AI ไม่ได้มาจากหนังสือ ควรตรวจกับครูผู้สอนหรือเปิดหนังสือตามหัวข้อท้ายคำตอบประกอบ
 เครื่องพิมพ์แบบระยะไกลต้องมีการตั้งค่าการแชร์บนเครื่องโฮสต์ และต้องมีการติดตั้งไดรเวอร์ที่เหมาะสมบนเครื่องผู้ใช้ปลายทางด้วย
@@ -2265,19 +2959,28 @@
 • บทที่ 4 การเชื่อมต่อเครือข่ายเวิร์กกรุ๊ปด้วย Windows 7 — หัวข้อ การแชร์เครื่องพิมพ์บนเครือข่าย (หน้า 158-162)</t>
         </is>
       </c>
-      <c r="D78" s="7" t="n"/>
-      <c r="E78" s="8" t="n"/>
+      <c r="D78" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" s="10" t="inlineStr">
+        <is>
+          <t>ตำราอธิบาย Remote Printer ไว้ใน net-4-23 หน้า 153-154 และ net-4-26 หน้า 162-163 แต่บอทบอกว่ายืนยันกับหนังสือไม่ได้และตอบจากความรู้ทั่วไปโดยไม่ได้ให้ความหมาย</t>
+        </is>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" s="6" t="n">
+      <c r="A79" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B79" s="6" t="inlineStr">
+      <c r="B79" s="7" t="inlineStr">
         <is>
           <t>การเข้าหัวสายแลนตามมาตรฐาน T568B เรียงสีอย่างไร</t>
         </is>
       </c>
-      <c r="C79" s="6" t="inlineStr">
+      <c r="C79" s="7" t="inlineStr">
         <is>
           <t>การเข้าหัวสายแลนตามมาตรฐาน T568B เรียงสีดังนี้
 • ขาวส้ม/ส้ม
@@ -2286,38 +2989,56 @@
 • ขาวน้ำตาล/น้ำตาล (บทที่ 4 หน้า 126-129) (บทที่ 4 หน้า 164-165)</t>
         </is>
       </c>
-      <c r="D79" s="7" t="n"/>
-      <c r="E79" s="8" t="n"/>
+      <c r="D79" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E79" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F79" s="10" t="inlineStr">
+        <is>
+          <t>ลำดับสี T568B ตรงกับ net-4-3 หน้า 126-129 และ net-4-27</t>
+        </is>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" s="6" t="n">
+      <c r="A80" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B80" s="6" t="inlineStr">
+      <c r="B80" s="7" t="inlineStr">
         <is>
           <t>เครือข่ายแบบเวิร์กกรุ๊ปเหมาะกับคอมพิวเตอร์กี่เครื่อง</t>
         </is>
       </c>
-      <c r="C80" s="6" t="inlineStr">
+      <c r="C80" s="7" t="inlineStr">
         <is>
           <t>เครือข่ายแบบเวิร์กกรุ๊ปเหมาะกับการใช้งานกับคอมพิวเตอร์จำนวนประมาณ 10 - 20 เครื่อง (บทที่ 4 หน้า 130)
 ไม่ควรเกิน 20 เครื่องเพื่อให้ประสิทธิภาพการทำงานบนเครือข่ายไม่ลดลง (บทที่ 4 หน้า 124)
 จำนวนเครื่องที่เชื่อมต่อไม่ควรเกินกว่า 20 เครื่อง (บทที่ 4 หน้า 164-165)</t>
         </is>
       </c>
-      <c r="D80" s="7" t="n"/>
-      <c r="E80" s="8" t="n"/>
+      <c r="D80" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F80" s="10" t="inlineStr">
+        <is>
+          <t>ประมาณ 10-20 เครื่อง ไม่ควรเกิน 20 เครื่อง ตรงกับ net-4-1 หน้า 124, net-4-5 หน้า 130 และ net-4-6</t>
+        </is>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="6" t="n">
+      <c r="A81" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B81" s="6" t="inlineStr">
+      <c r="B81" s="7" t="inlineStr">
         <is>
           <t>เครือข่ายแบบเวิร์กกรุ๊ปต่างจากแบบโดเมนอย่างไร</t>
         </is>
       </c>
-      <c r="C81" s="6" t="inlineStr">
+      <c r="C81" s="7" t="inlineStr">
         <is>
           <t>เครือข่ายแบบเวิร์กกรุ๊ปต่างจากแบบโดเมนในหลายด้าน โดยเครือข่ายแบบเวิร์กกรุ๊ปเป็นเครือข่ายแบบเพียร์ทูเพียร์ ที่ทุกเครื่องมีสิทธิ์เท่าเทียมกัน ไม่มีเครื่องใดควบคุมเครื่องอื่น และบัญชีผู้ใช้ถูกจัดเก็บกระจายอยู่ตามเครื่องต่างๆ ทำให้ต้องสร้างบัญชีผู้ใช้ทีละเครื่องเมื่อต้องการเข้าถึงทรัพยากรของอีกเครื่องหนึ่ง (บทที่ 4 หน้า 130)
 ในขณะที่เครือข่ายแบบโดเมนเป็นเครือข่ายแบบไคลเอ็นต์เชิร์ฟเวอร์ ที่มีเครื่องเชิร์ฟเวอร์ทำหน้าที่เป็นศูนย์กลางในการจัดการบัญชีผู้ใช้และสิทธิ์การเข้าถึงทรัพยากร โดยข้อมูลจะถูกเก็บไว้ในโดเมนคอนโทรลเลอร์ ทำให้ผู้ใช้สามารถเข้าถึงทรัพยากรบนเครื่องใดก็ได้ด้วยบัญชีเดียว และมีระบบความปลอดภัยที่เข้มงวดกว่า (บทที่ 4 หน้า 131)
@@ -2327,38 +3048,56 @@
 • เครือข่ายเวิร์กกรุ๊ปมีระบบความปลอดภัยต่ำ แต่เครือข่ายโดเมนมีการควบคุมสิทธิ์อย่างเข้มงวด เช่น กำหนดเวลาเข้าระบบ หรือจำกัดการล็อกออนเฉพาะเครื่องที่กำหนด (บทที่ 4 หน้า 131-132)</t>
         </is>
       </c>
-      <c r="D81" s="7" t="n"/>
-      <c r="E81" s="8" t="n"/>
+      <c r="D81" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E81" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F81" s="10" t="inlineStr">
+        <is>
+          <t>ข้อแตกต่างตรงกับ net-4-5 ถึง net-4-8 หน้า 130-132</t>
+        </is>
+      </c>
     </row>
     <row r="82">
-      <c r="A82" s="6" t="n">
+      <c r="A82" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B82" s="6" t="inlineStr">
+      <c r="B82" s="7" t="inlineStr">
         <is>
           <t>หมายเลขไอพีคลาส C สำหรับเครือข่ายส่วนตัวอยู่ในช่วงใด</t>
         </is>
       </c>
-      <c r="C82" s="6" t="inlineStr">
+      <c r="C82" s="7" t="inlineStr">
         <is>
           <t>หมายเลขไอพีคลาส C สำหรับเครือข่ายส่วนตัวอยู่ในช่วง 192.168.0.0 ถึง 192.168.255.255 (บทที่ 4 หน้า 166-167)
 💡 เสริมจากความรู้ทั่วไปของ AI (ส่วนนี้ไม่ได้มาจากหนังสือ ควรตรวจกับครูผู้สอนหรือแหล่งอื่นประกอบ)
 ช่วงหมายเลขไอพีนี้ถูกออกแบบมาเพื่อใช้ในเครือข่ายภายใน (Private IP) โดยเฉพาะเครือข่ายขนาดเล็ก เช่น บ้านหรือสำนักงานเล็ก ๆ ซึ่งไม่ต้องเชื่อมต่อกับอินเทอร์เน็ตโดยตรง และสามารถใช้ซ้ำได้ในหลายเครือข่ายโดยไม่เกิดความขัดแย้ง</t>
         </is>
       </c>
-      <c r="D82" s="7" t="n"/>
-      <c r="E82" s="8" t="n"/>
+      <c r="D82" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F82" s="10" t="inlineStr">
+        <is>
+          <t>192.168.0.0 ถึง 192.168.255.255 ตรงกับ net-4-16 หน้า 143-144 และ net-4-30</t>
+        </is>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" s="6" t="n">
+      <c r="A83" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B83" s="6" t="inlineStr">
+      <c r="B83" s="7" t="inlineStr">
         <is>
           <t>สร้างสายแลนแบบไขว้ต้องเรียงสีแบบไหน</t>
         </is>
       </c>
-      <c r="C83" s="6" t="inlineStr">
+      <c r="C83" s="7" t="inlineStr">
         <is>
           <t>สายแลนแบบไขว้ (Crossover) ต้องเรียงสีปลายหนึ่งตามมาตรฐาน T568A และอีกปลายหนึ่งตามมาตรฐาน T568B
 ปลายที่เรียงตามมาตรฐาน T568A คือ ขาวเขียว/เขียว, ขาวส้ม/น้ำเงิน, ขาวน้ำเงิน/ส้ม, ขาวน้ำตาล/น้ำตาล (บทที่ 4 หน้า 129)
@@ -2368,19 +3107,28 @@
 สายแบบไขว้ใช้เชื่อมต่อระหว่างคอมพิวเตอร์ 2 เครื่องโดยตรง หรือเชื่อมต่อฮับกับฮับ โดยต้องเรียงสีต่างกันทั้งสองปลาย</t>
         </is>
       </c>
-      <c r="D83" s="7" t="n"/>
-      <c r="E83" s="8" t="n"/>
+      <c r="D83" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E83" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F83" s="10" t="inlineStr">
+        <is>
+          <t>ปลายหนึ่ง T568A อีกปลาย T568B พร้อมลำดับสีตรงกับ net-4-4 หน้า 129 และ net-4-27</t>
+        </is>
+      </c>
     </row>
     <row r="84">
-      <c r="A84" s="6" t="n">
+      <c r="A84" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B84" s="6" t="inlineStr">
+      <c r="B84" s="7" t="inlineStr">
         <is>
           <t>เครือข่ายเวิร์กกรุ๊ปที่อนุญาตให้เฉพาะผู้มีบัญชีผู้ใช้เท่านั้น สามารถเข้าถึงทรัพยากรที่เปิดแชร์ได้ คิดว่ามีข้อดีกว่าการเปิดแชร์แบบ Public อย่างไร จงอธิบาย</t>
         </is>
       </c>
-      <c r="C84" s="6" t="inlineStr">
+      <c r="C84" s="7" t="inlineStr">
         <is>
           <t>การที่เครือข่ายเวิร์กกรุ๊ปอนุญาตให้เฉพาะผู้มีบัญชีผู้ใช้เท่านั้นเข้าถึงทรัพยากรที่เปิดแชร์ได้ มีข้อดีกว่าการเปิดแชร์แบบ Public ตรงที่สามารถควบคุมสิทธิ์การเข้าถึงได้อย่างแม่นยำ ทำให้ข้อมูลมีความปลอดภัยมากขึ้น (บทที่ 5 หน้า 175-176)
 โดยสามารถกำหนดสิทธิ์ให้ผู้ใช้แต่ละรายได้เฉพาะสิทธิ์ที่เหมาะสม เช่น อนุญาตให้ "อ่าน" เท่านั้น หรือ "อ่านและเขียน" ได้ตามความจำเป็น ซึ่งช่วยป้องกันการแก้ไขหรือลบไฟล์โดยไม่ได้รับอนุญาต (บทที่ 5 หน้า 220-221)
@@ -2389,36 +3137,54 @@
 การตั้งค่าดังกล่าวจึงช่วยเพิ่มความปลอดภัยและความเป็นระเบียบในเครือข่ายเวิร์กกรุ๊ปได้อย่างมีประสิทธิภาพ (บทที่ 5 หน้า 175-176)</t>
         </is>
       </c>
-      <c r="D84" s="7" t="n"/>
-      <c r="E84" s="8" t="n"/>
+      <c r="D84" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E84" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F84" s="10" t="inlineStr">
+        <is>
+          <t>ปลอดภัยกว่าเพราะต้องมีบัญชีและรหัสผ่านและจำกัดสิทธิ์ Read หรือ Read/Write ได้ ตรงกับ net-5-1 หน้า 175-176</t>
+        </is>
+      </c>
     </row>
     <row r="85">
-      <c r="A85" s="6" t="n">
+      <c r="A85" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B85" s="6" t="inlineStr">
+      <c r="B85" s="7" t="inlineStr">
         <is>
           <t>แนวทางที่ดีสำหรับการสร้างบัญชีผู้ใช้บนเครือข่าย ประกอบด้วยอะไรบ้าง</t>
         </is>
       </c>
-      <c r="C85" s="6" t="inlineStr">
+      <c r="C85" s="7" t="inlineStr">
         <is>
           <t>แนวทางที่ดีสำหรับการสร้างบัญชีผู้ใช้บนเครือข่าย ประกอบด้วยการวางแผนอย่างมีระบบ โดยเริ่มจากการกำหนดกลุ่มหรือแผนกที่ต้องการ แล้วจัดทำรายชื่อผู้ใช้และแผนกที่สังกัด สร้างบัญชีผู้ใช้และกลุ่มขึ้นมา นำบัญชีผู้ใช้แต่ละคนสังกัดเข้ากลุ่มที่ต้องการ สร้างโฟลเดอร์ที่ต้องการแชร์ ทั้งโฟลเดอร์เฉพาะแผนกและโฟลเดอร์ที่เปิดให้ทุกแผนกเข้าถึงได้ แล้วกำหนดสิทธิ์ (Permission) ในการเข้าถึงโฟลเดอร์ให้กับกลุ่มต่างๆ ตามความเหมาะสม (บทที่ 5 หน้า 220)</t>
         </is>
       </c>
-      <c r="D85" s="7" t="n"/>
-      <c r="E85" s="8" t="n"/>
+      <c r="D85" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E85" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" s="10" t="inlineStr">
+        <is>
+          <t>แนวทาง 6 ข้อครบตาม net-5-4 หน้า 179 และ net-5-23 หน้า 220</t>
+        </is>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" s="6" t="n">
+      <c r="A86" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B86" s="6" t="inlineStr">
+      <c r="B86" s="7" t="inlineStr">
         <is>
           <t>จงสรุปขั้นตอนการสร้างบัญชีผู้ใช้ (User Account) มาให้เข้าใจพอสังเขป</t>
         </is>
       </c>
-      <c r="C86" s="6" t="inlineStr">
+      <c r="C86" s="7" t="inlineStr">
         <is>
           <t>ขั้นตอนการสร้างบัญชีผู้ใช้ (User Account) มีดังนี้
 1. วางแผนกลุ่มหรือแผนกที่ต้องการสร้าง เช่น แผนกคอมพิวเตอร์ และแผนกการตลาด
@@ -2435,19 +3201,28 @@
 12. สำหรับเครื่องอื่นๆ บนเครือข่าย ต้องสร้างบัญชีผู้ใช้เดียวกันทั้งหมดเพื่อให้เข้าถึงทรัพยากรได้ (บทที่ 5 หน้า 202-203)</t>
         </is>
       </c>
-      <c r="D86" s="7" t="n"/>
-      <c r="E86" s="8" t="n"/>
+      <c r="D86" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E86" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F86" s="10" t="inlineStr">
+        <is>
+          <t>ขั้นตอน Manage &gt; Local Users and Groups &gt; Users &gt; New User &gt; Create ตรงกับ net-5-6 และ net-5-7 หน้า 180-184</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" s="6" t="n">
+      <c r="A87" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B87" s="6" t="inlineStr">
+      <c r="B87" s="7" t="inlineStr">
         <is>
           <t>จงสรุปขั้นตอนการสร้างกลุ่ม (Group) มาให้เข้าใจพอสังเขป</t>
         </is>
       </c>
-      <c r="C87" s="6" t="inlineStr">
+      <c r="C87" s="7" t="inlineStr">
         <is>
           <t>ขั้นตอนการสร้างกลุ่ม (Group) มีดังนี้
 1. ที่หน้าต่าง Computer Management ตรงหัวข้อ Local Users and Groups ให้คลิกที่ Groups
@@ -2459,19 +3234,28 @@
 7. ท้ายสุด กลุ่มแผนกคอมพิวเตอร์และแผนกการตลาด ได้ถูกสร้างขึ้นมาเป็นที่เรียบร้อย (บทที่ 5 หน้า 185-186)</t>
         </is>
       </c>
-      <c r="D87" s="7" t="n"/>
-      <c r="E87" s="8" t="n"/>
+      <c r="D87" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E87" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F87" s="10" t="inlineStr">
+        <is>
+          <t>ขั้นตอนสร้างกลุ่ม 7 ข้อตรงกับ net-5-8 หน้า 185-186</t>
+        </is>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" s="6" t="n">
+      <c r="A88" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B88" s="6" t="inlineStr">
+      <c r="B88" s="7" t="inlineStr">
         <is>
           <t>การนำสมาชิกเข้าสังกัดกลุ่ม อยากทราบว่ามีข้อดีอย่างไร จงอธิบาย</t>
         </is>
       </c>
-      <c r="C88" s="6" t="inlineStr">
+      <c r="C88" s="7" t="inlineStr">
         <is>
           <t>การนำสมาชิกเข้าสังกัดกลุ่มช่วยให้การจัดการสิทธิ์การเข้าถึงทรัพยากรในเครือข่ายทำได้ง่ายและมีประสิทธิภาพ เพราะเมื่อยูสเซอร์ถูกเพิ่มเข้าสู่กลุ่มแล้ว จะได้รับสิทธิ์ (Permission) ตามที่กำหนดไว้กับกลุ่มนั้นโดยอัตโนมัติ ทำให้ผู้ดูแลระบบไม่ต้องตั้งค่าสิทธิ์ให้แต่ละบุคคลทีละราย (บทที่ 5 หน้า 179)
 การจัดกลุ่มช่วยให้สามารถควบคุมการเข้าถึงโฟลเดอร์หรือทรัพยากรต่างๆ ได้ตามแผนก เช่น แผนกคอมพิวเตอร์จะมีสิทธิ์เต็มรูปแบบ (Read/Write) ต่อโฟลเดอร์ job_computer ขณะที่แผนกการตลาดจะเข้าถึงโฟลเดอร์ job_marketing ได้เท่านั้น (บทที่ 5 หน้า 180)
@@ -2482,19 +3266,28 @@
 การใช้กลุ่มช่วยให้การจัดการเครือข่ายมีระบบและลดความผิดพลาดจากการตั้งค่าสิทธิ์ผิดพลาดได้</t>
         </is>
       </c>
-      <c r="D88" s="7" t="n"/>
-      <c r="E88" s="8" t="n"/>
+      <c r="D88" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E88" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F88" s="10" t="inlineStr">
+        <is>
+          <t>สิทธิ์ระดับกลุ่มส่งผลต่อสมาชิกในกลุ่มโดยอัตโนมัติ ตรงกับ net-5-4 หน้า 179</t>
+        </is>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" s="6" t="n">
+      <c r="A89" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B89" s="6" t="inlineStr">
+      <c r="B89" s="7" t="inlineStr">
         <is>
           <t>สิทธิ์หรือ Permissions ประกอบไปด้วยระดับใดบ้าง จงอธิบาย</t>
         </is>
       </c>
-      <c r="C89" s="6" t="inlineStr">
+      <c r="C89" s="7" t="inlineStr">
         <is>
           <t>สิทธิ์หรือ Permissions ประกอบไปด้วยระดับต่อไปนี้
 - Full Control เป็นสิทธิ์เต็มรูปแบบที่อนุญาตให้ผู้ใช้สามารถดำเนินการใดๆ ได้ทั้งหมดที่ปรากฏอยู่ในลิสต์ รวมถึงความสามารถในการเปลี่ยนแปลงสิทธิ์
@@ -2505,19 +3298,28 @@
 ระดับสิทธิ์ทั้งหลายเหล่านี้ สามารถคลิกเพื่อกำหนดสิทธิ์ได้หลายๆ ค่ารวมกัน (บทที่ 5 หน้า 193-197)</t>
         </is>
       </c>
-      <c r="D89" s="7" t="n"/>
-      <c r="E89" s="8" t="n"/>
+      <c r="D89" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E89" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F89" s="10" t="inlineStr">
+        <is>
+          <t>ตำรามี 6 ระดับใน net-5-11 หน้า 193-197 แต่คำตอบให้เพียง 5 ระดับ ขาดสิทธิ์ Write</t>
+        </is>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" s="6" t="n">
+      <c r="A90" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B90" s="6" t="inlineStr">
+      <c r="B90" s="7" t="inlineStr">
         <is>
           <t>จงสรุปขั้นตอนการแชร์ไฟล์เฉพาะผู้ได้รับอนุญาต มาให้เข้าใจพอสังเขป</t>
         </is>
       </c>
-      <c r="C90" s="6" t="inlineStr">
+      <c r="C90" s="7" t="inlineStr">
         <is>
           <t>1. ปิดการแชร์โฟลเดอร์แบบ Public ก่อน เพื่อจำกัดการเข้าถึงเฉพาะผู้ที่มีบัญชีผู้ใช้ที่ได้รับอนุญาต
 3. สร้างโฟลเดอร์ย่อยในโฟลเดอร์หลัก เช่น job_computer, job_marketing และ notice
@@ -2525,19 +3327,28 @@
 7. ผู้ใช้ที่ต้องการเข้าถึงต้องล็อกออนด้วยบัญชีผู้ใช้ที่มีอยู่ในเครื่องโฮสต์ และเครื่องไคลเอ็นต์ต้องมีบัญชีผู้ใช้นั้นด้วย (บทที่ 5 หน้า 220) (บทที่ 5 หน้า 220-221)</t>
         </is>
       </c>
-      <c r="D90" s="7" t="n"/>
-      <c r="E90" s="8" t="n"/>
+      <c r="D90" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E90" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F90" s="10" t="inlineStr">
+        <is>
+          <t>ขั้นตอนที่ให้ถูกต้องตาม net-5-3, net-5-10, net-5-12 แต่ขาดการสร้างยูสเซอร์และกลุ่ม การนำเข้ากลุ่ม และการกำหนดสิทธิ์ที่แท็บ Security (net-5-6 ถึง net-5-11)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" s="6" t="n">
+      <c r="A91" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B91" s="6" t="inlineStr">
+      <c r="B91" s="7" t="inlineStr">
         <is>
           <t>การแมปไดรฟ์ คืออะไร มีประโยชน์อย่างไร จงอธิบาย</t>
         </is>
       </c>
-      <c r="C91" s="6" t="inlineStr">
+      <c r="C91" s="7" t="inlineStr">
         <is>
           <t>การแมปไดรฟ์ คือการจำลองโฟลเดอร์ให้เป็นเสมือนไดรฟ์หนึ่งบนเครื่องของตนเอง ช่วยให้การเข้าถึงโฟลเดอร์ที่แชร์บนเครือข่ายทำได้ง่ายและรวดเร็วขึ้น เพราะสามารถคลิกเข้าไปยังไดรฟ์ที่แมปไว้ได้ทันทีโดยไม่ต้องผ่านหลายชั้นโฟลเดอร์ย่อย (บทที่ 5 หน้า 221)
 ประโยชน์ของ การแมปไดรฟ์ คือ ทำให้การเข้าถึงข้อมูลที่แชร์บนเครือข่ายสะดวกและรวดเร็วขึ้น โดยไม่ต้องคลิกผ่านโฟลเดอร์ย่อยหลายชั้น ซึ่งช่วยประหยัดเวลาในการทำงาน (บทที่ 5 หน้า 209-211)
@@ -2545,19 +3356,28 @@
 การแมปไดรฟ์ช่วยให้ผู้ใช้สามารถเข้าถึงข้อมูลที่ต้องใช้บ่อยได้อย่างต่อเนื่อง โดยไม่ต้องจำเส้นทางการเข้าถึงซ้ำ ๆ ซึ่งเหมาะกับการทำงานร่วมกันในองค์กรที่มีการแชร์ข้อมูลบ่อยครั้ง</t>
         </is>
       </c>
-      <c r="D91" s="7" t="n"/>
-      <c r="E91" s="8" t="n"/>
+      <c r="D91" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E91" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F91" s="10" t="inlineStr">
+        <is>
+          <t>ความหมายและประโยชน์ของการแมปไดรฟ์ตรงกับ net-5-19 หน้า 209 และ net-5-25 หน้า 221</t>
+        </is>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" s="6" t="n">
+      <c r="A92" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B92" s="6" t="inlineStr">
+      <c r="B92" s="7" t="inlineStr">
         <is>
           <t>จงสรุปขั้นตอนการแมปไดรฟ์ มาให้พอเข้าใจ</t>
         </is>
       </c>
-      <c r="C92" s="6" t="inlineStr">
+      <c r="C92" s="7" t="inlineStr">
         <is>
           <t>การแมปไดรฟ์คือการจำลองโฟลเดอร์ที่แชร์บนเครือข่ายให้กลายเป็นไดรฟ์เสมือนในเครื่องผู้ใช้ เพื่อให้เข้าถึงข้อมูลได้สะดวกและรวดเร็วโดยไม่ต้องคลิกผ่านหลายชั้นโฟลเดอร์ (บทที่ 5 หน้า 209-211)
 ขั้นตอนการแมปไดรฟ์มีดังนี้
@@ -2569,19 +3389,28 @@
 6. จะปรากฏไดรฟ์ S: ซึ่งแทนโฟลเดอร์ของสมศรี (COMPUTER1\\job_computer\somsri_work) สามารถดับเบิลคลิกเข้าไปใช้งานได้ทันที (บทที่ 5 หน้า 209-211)</t>
         </is>
       </c>
-      <c r="D92" s="7" t="n"/>
-      <c r="E92" s="8" t="n"/>
+      <c r="D92" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F92" s="10" t="inlineStr">
+        <is>
+          <t>ขั้นตอน 6 ข้อตรงกับ net-5-19 หน้า 209-211</t>
+        </is>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="6" t="n">
+      <c r="A93" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B93" s="6" t="inlineStr">
+      <c r="B93" s="7" t="inlineStr">
         <is>
           <t>การแชร์เครื่องพิมพ์บนเครือข่าย มีหลักการติดตั้งอย่างไร และกรณีที่เปิดแชร์เครื่องพิมพ์มากกว่าหนึ่งเครื่อง เวลาสั่งพิมพ์งานจะต้องปฏิบัติอย่างโร</t>
         </is>
       </c>
-      <c r="C93" s="6" t="inlineStr">
+      <c r="C93" s="7" t="inlineStr">
         <is>
           <t>การแชร์เครื่องพิมพ์บนเครือข่ายมีหลักการติดตั้งดังนี้
 1. ติดตั้งไดรเวอร์เครื่องพิมพ์บนเครื่องโฮสต์ (COMPUTER1) โดยใช้แผ่นไดรเวอร์จากซีดี/ดีวีดี แล้วเลือกรุ่นเครื่องพิมพ์ที่ถูกต้อง เช่น Brother รุ่น HL-2140 คลิก Next แล้วเลือกการเชื่อมต่อแบบ Local Printer ตามขั้นตอน (บทที่ 4 หน้า 153-154)
@@ -2592,38 +3421,56 @@
 หากมีหลายเครื่องพิมพ์ที่แชร์ไว้ ให้ตรวจสอบชื่อเครื่องพิมพ์ในรายการเครื่องพิมพ์ระยะไกล (Remote Printer) บนเครื่องปลายทางก่อนสั่งพิมพ์ (บทที่ 4 หน้า 158-162)</t>
         </is>
       </c>
-      <c r="D93" s="7" t="n"/>
-      <c r="E93" s="8" t="n"/>
+      <c r="D93" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E93" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F93" s="10" t="inlineStr">
+        <is>
+          <t>ติดตั้ง Local Printer แล้วเปิดแชร์ เครื่องอื่นเพิ่มแบบ Network Printer และต้องเลือกชื่อเครื่องพิมพ์ให้ถูกต้อง ตรงกับ net-4-23 ถึง net-4-26 และ net-5-22 หน้า 216-219</t>
+        </is>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" s="6" t="n">
+      <c r="A94" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B94" s="6" t="inlineStr">
+      <c r="B94" s="7" t="inlineStr">
         <is>
           <t>การแมปไดรฟ์คืออะไร</t>
         </is>
       </c>
-      <c r="C94" s="6" t="inlineStr">
+      <c r="C94" s="7" t="inlineStr">
         <is>
           <t>การแมปไดรฟ์ คือการจำลองโฟลเดอร์ให้มาเป็นเสมือนไดรฟ์หนึ่งบนเครื่องของตนเอง ช่วยสร้างความสะดวกต่อการเข้าถึง เนื่องจากสามารถคลิกเข้าไปเพื่อเข้าถึงตำแหน่งโฟลเดอร์ที่แมปไว้ได้ทันที (บทที่ 5 หน้า 221)
 • การแมปไดรฟ์ช่วยให้การเข้าถึงโฟลเดอร์ที่แชร์บนเครือข่ายสะดวกขึ้น โดยไม่ต้องคลิกผ่านโฟลเดอร์ย่อยหลายชั้น
 • หลังจากแมปแล้ว ไดรฟ์ที่สร้างขึ้นจะปรากฏในหน้าต่าง Computer ทำให้สามารถดับเบิลคลิกเข้าไปใช้งานได้ทันที (บทที่ 5 หน้า 209-211)</t>
         </is>
       </c>
-      <c r="D94" s="7" t="n"/>
-      <c r="E94" s="8" t="n"/>
+      <c r="D94" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F94" s="10" t="inlineStr">
+        <is>
+          <t>จำลองโฟลเดอร์เป็นเสมือนไดรฟ์หนึ่ง ตรงกับ net-5-25 หน้า 221 และ net-5-19</t>
+        </is>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="6" t="n">
+      <c r="A95" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B95" s="6" t="inlineStr">
+      <c r="B95" s="7" t="inlineStr">
         <is>
           <t>แนวทางในการติดตั้งโปรแกรมประยุกต์บนเครือข่าย มีอะไรบ้าง จงสรุปมาให้เข้าใจพอสังเขป</t>
         </is>
       </c>
-      <c r="C95" s="6" t="inlineStr">
+      <c r="C95" s="7" t="inlineStr">
         <is>
           <t>แนวทางในการติดตั้งโปรแกรมประยุกต์บนเครือข่ายมี 3 วิธี ได้แก่
 1. เลือกใช้โปรแกรมประยุกต์แบบชุดสำเร็จรูป (Full Packaged) เพื่อนำมาติดตั้งในคอมพิวเตอร์แต่ละเครื่อง วิธีนี้เหมาะกับการใช้งานส่วนตัว หรือหน่วยงานที่มีจำนวนคอมพิวเตอร์ไม่เกิน 5 เครื่อง
@@ -2631,19 +3478,28 @@
 3. ติดตั้งโปรแกรมประยุกต์ที่เครื่องเชิร์ฟเวอร์เพียงเครื่องเดียว แล้วเปิดแชร์ใช้งานให้กับเครื่องลูกข่ายต่างๆ บนเครือข่าย (บทที่ 7 หน้า 288)</t>
         </is>
       </c>
-      <c r="D95" s="7" t="n"/>
-      <c r="E95" s="8" t="n"/>
+      <c r="D95" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F95" s="10" t="inlineStr">
+        <is>
+          <t>แนวทาง 3 ข้อครบตาม net-7-1, net-7-2 และ net-7-18 หน้า 288</t>
+        </is>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" s="6" t="n">
+      <c r="A96" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B96" s="6" t="inlineStr">
+      <c r="B96" s="7" t="inlineStr">
         <is>
           <t>หากมีคอมพิวเตอร์บนเครือข่ายมากกว่าหนึ่งเครื่อง ได้ใช้โปรแกรมประยุกต์ เช่น MS-Word เรียกไฟล์เอกสารชุดเดียวกันขึ้นมา ซึ่งหนึ่งในนั้นได้มีเครื่องใดเครื่องหนึ่งโหลดไฟล์ชุดนั้นไปใช้งานอยู่ก่อนแล้ว (ระบบได้มีการล็อกไฟล์) ดังนั้น เครื่องในลำดับถัดมา จะมีทางเลือกในการจัดการกับข้อมูลชุดเดียวกันนี้อย่างไร จงอธิบาย</t>
         </is>
       </c>
-      <c r="C96" s="6" t="inlineStr">
+      <c r="C96" s="7" t="inlineStr">
         <is>
           <t>เมื่อเครื่องใดเครื่องหนึ่งได้โหลดไฟล์ข้อมูลชุดเดียวกันขึ้นมาใช้งานและมีการล็อกไฟล์ไว้แล้ว เครื่องอื่นที่ต้องการใช้งานไฟล์ชุดเดียวกันนี้จะมีทางเลือกในการจัดการกับข้อมูลนั้นอยู่ 3 ทาง ดังนี้
 • ทางเลือกที่ 1 : เปิดไฟล์ดังกล่าวขึ้นมาแบบอ่านได้อย่างเดียว โดยสังเกตจากคำว่า Read-Only ที่ต่อท้ายชื่อไฟล์ และปุ่มเมนูต่างๆ จะถูก Disable ไว้ ไม่สามารถใช้งานใดๆ ได้ (บทที่ 7 หน้า 264-265)
@@ -2652,19 +3508,28 @@
 แนวทางในการจัดการกับไฟล์ข้อมูลชุดเดียวกันนี้มีอยู่ 3 ทางเลือกด้วยกันคือ เปิดไฟล์แบบอ่านได้อย่างเดียว (บทที่ 7 หน้า 288)</t>
         </is>
       </c>
-      <c r="D96" s="7" t="n"/>
-      <c r="E96" s="8" t="n"/>
+      <c r="D96" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E96" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F96" s="10" t="inlineStr">
+        <is>
+          <t>ทางเลือก 3 ทางพร้อมคำอธิบายตรงกับ net-7-6 ถึง net-7-8 หน้า 264-268</t>
+        </is>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="6" t="n">
+      <c r="A97" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B97" s="6" t="inlineStr">
+      <c r="B97" s="7" t="inlineStr">
         <is>
           <t>จากข้อที่ 2 อยากทราบว่า หากไม่มีกระบวนการล็อกไฟล์เข้ามาจัดการกับการเข้าถึงข้อมูลชุดเดียวกันบนเครือข่าย คิดว่าจะก่อให้เกิดปัญหาใดตามมา</t>
         </is>
       </c>
-      <c r="C97" s="6" t="inlineStr">
+      <c r="C97" s="7" t="inlineStr">
         <is>
           <t>หากไม่มีกระบวนการล็อกไฟล์เข้ามาจัดการกับการเข้าถึงข้อมูลชุดเดียวกันบนเครือข่าย อาจก่อให้เกิดปัญหาการแก้ไขข้อมูลพร้อมกันจากผู้ใช้หลายคน ทำให้ข้อมูลสูญหายหรือขัดแย้งกันได้
 เนื่องจากผู้ใช้ที่เข้าถึงไฟล์เดียวกันพร้อมกันอาจบันทึกข้อมูลทับซ้อนกัน จนเกิดความขัดแย้งในเนื้อหาไฟล์
@@ -2672,19 +3537,28 @@
 ดังนั้น กระบวนการล็อกไฟล์จึงจำเป็นเพื่อป้องกันไม่ให้เกิดการแก้ไขข้อมูลพร้อมกันโดยไม่ควบคุม (บทที่ 7 หน้า 262-263)</t>
         </is>
       </c>
-      <c r="D97" s="7" t="n"/>
-      <c r="E97" s="8" t="n"/>
+      <c r="D97" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E97" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F97" s="10" t="inlineStr">
+        <is>
+          <t>ให้เหตุผลสอดคล้องกับหลักการล็อกไฟล์ใน net-7-3 หน้า 262-263 ที่ให้ผู้ใช้รายเดียวเขียนได้ในแต่ละครั้ง</t>
+        </is>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="6" t="n">
+      <c r="A98" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B98" s="6" t="inlineStr">
+      <c r="B98" s="7" t="inlineStr">
         <is>
           <t>โปรแกรมยูทิลิตี้ คืออะไร จงอธิบาย</t>
         </is>
       </c>
-      <c r="C98" s="6" t="inlineStr">
+      <c r="C98" s="7" t="inlineStr">
         <is>
           <t>โปรแกรมยูทิลิตี้ หรือโปรแกรมอรรถประโยชน์ เป็นโปรแกรมที่ถูกจัดอยู่ในประเภทหนึ่งของซอฟต์แวร์ระบบ ถูกออกแบบมาเพื่อทำหน้าที่เฉพาะอย่าง เช่น การวิเคราะห์ การปรับปรุงให้ระบบคอมพิวเตอร์ทำงานได้ดีขึ้น รวมถึงการบำรุงรักษาคอมพิวเตอร์ โดยปกติ โปรแกรมยูทิลิตี้จะมุ่งประเด็นในเรื่องวิธีการที่เกี่ยวข้องกับโครงสร้างพื้นฐานของคอมพิวเตอร์เป็นหลัก อันประกอบด้วย อุปกรณ์ฮาร์ดแวร์ ระบบปฏิบัติการ โปรแกรมประยุกต์ และการจัดเก็บข้อมูล (บทที่ 7 หน้า 288)
 • โปรแกรมยูทิลิตี้มักใช้เพื่อช่วยในการจัดการและดูแลระบบคอมพิวเตอร์ เช่น การจัดทำสต็อกเครื่องคอมพิวเตอร์ในองค์กร ซึ่งอาจทำได้โดยใช้โปรแกรมอย่าง Alchemy Network Inventory ที่ช่วยเก็บข้อมูลสเปกฮาร์ดแวร์ ระบบปฏิบัติการ และสามารถพิมพ์รายงานได้
@@ -2692,19 +3566,28 @@
 โปรแกรมยูทิลิตี้จึงเป็นเครื่องมือที่ช่วยให้การดูแลระบบคอมพิวเตอร์มีประสิทธิภาพมากขึ้น โดยเฉพาะในองค์กรที่มีเครื่องคอมพิวเตอร์จำนวนมาก (บทที่ 7 หน้า 269)</t>
         </is>
       </c>
-      <c r="D98" s="7" t="n"/>
-      <c r="E98" s="8" t="n"/>
+      <c r="D98" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E98" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F98" s="10" t="inlineStr">
+        <is>
+          <t>ความหมายของโปรแกรมยูทิลิตี้ตรงกับ net-7-10 หน้า 269 และ net-7-19 หน้า 288</t>
+        </is>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" s="6" t="n">
+      <c r="A99" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B99" s="6" t="inlineStr">
+      <c r="B99" s="7" t="inlineStr">
         <is>
           <t>ทำไมการจัดสต็อกเครื่องคอมพิวเตอร์ตามองค์กรขนาดใหญ่ที่มีเครื่องคอมพิวเตอร์จำนวนมาก จึงเป็นเรื่องที่ยุ่งยาก แล้วคิดว่าโปรแกรม Alchemy Network Inventory ช่วยลดภาระงานนี้ได้อย่างไร</t>
         </is>
       </c>
-      <c r="C99" s="6" t="inlineStr">
+      <c r="C99" s="7" t="inlineStr">
         <is>
           <t>การจัดสต็อกเครื่องคอมพิวเตอร์ในองค์กรขนาดใหญ่ที่มีเครื่องคอมพิวเตอร์จำนวนมากจึงเป็นเรื่องที่ยุ่งยาก เพราะต้องเก็บข้อมูลรายละเอียดของฮาร์ดแวร์ ระบบปฏิบัติการ และโปรแกรมต่างๆ ของแต่ละเครื่องด้วยมือ ซึ่งใช้เวลานานและมีโอกาสผิดพลาดสูง (บทที่ 7 หน้า 269)
 โปรแกรม Alchemy Network Inventory ช่วยลดภาระงานนี้ได้โดยสามารถสแกนและเก็บข้อมูลรายละเอียดฮาร์ดแวร์ ระบบปฏิบัติการ และโปรแกรมต่างๆ ของเครื่องคอมพิวเตอร์ที่เชื่อมต่อในเครือข่ายอัตโนมัติ พร้อมจัดเก็บข้อมูลไว้ในศูนย์กลางเดียวกัน (บทที่ 7 หน้า 269-270)
@@ -2717,19 +3600,28 @@
 โปรแกรม Alchemy Network Inventory ช่วยให้การจัดการทรัพยากรเครือข่ายมีประสิทธิภาพ โดยเฉพาะในองค์กรที่ต้องควบคุมฮาร์ดแวร์และซอฟต์แวร์จำนวนมาก ซึ่งช่วยลดความผิดพลาดจากการจัดทำสต็อกด้วยมือและประหยัดเวลาในการตรวจสอบระบบ</t>
         </is>
       </c>
-      <c r="D99" s="7" t="n"/>
-      <c r="E99" s="8" t="n"/>
+      <c r="D99" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E99" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F99" s="10" t="inlineStr">
+        <is>
+          <t>จัดสต็อกด้วยมือยากและเสียเวลา โปรแกรมเก็บสเปกเครื่องและพิมพ์รายงานได้ ตรงกับ net-7-10, net-7-11 และ net-7-17</t>
+        </is>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" s="6" t="n">
+      <c r="A100" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B100" s="6" t="inlineStr">
+      <c r="B100" s="7" t="inlineStr">
         <is>
           <t>โปรแกรม Alchemy Network Inventory ใช้ทำอะไร</t>
         </is>
       </c>
-      <c r="C100" s="6" t="inlineStr">
+      <c r="C100" s="7" t="inlineStr">
         <is>
           <t>โปรแกรม Alchemy Network Inventory ใช้จัดเก็บสต็อกเครื่องคอมพิวเตอร์ที่เชื่อมต่ออยู่บนเครือข่าย โดยเก็บรายละเอียดข้อมูลสเปกฮาร์ดแวร์ ระบบปฏิบัติการ และสามารถสั่งพิมพ์รายงานต่างๆ ได้ตามต้องการ
 โปรแกรมนี้รองรับการใช้งานทั้งเครือข่ายแบบเวิร์กกรุ๊ปและแบบไคลเอ็นต์/เชิร์ฟเวอร์ (บทที่ 7 หน้า 269-270)
@@ -2741,8 +3633,17 @@
 โปรแกรมช่วยให้การจัดการสต็อกเครื่องคอมพิวเตอร์ในองค์กรกลายเป็นเรื่องง่ายขึ้น (บทที่ 7 หน้า 269-270)</t>
         </is>
       </c>
-      <c r="D100" s="7" t="n"/>
-      <c r="E100" s="8" t="n"/>
+      <c r="D100" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E100" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F100" s="10" t="inlineStr">
+        <is>
+          <t>ใช้จัดเก็บสต็อกเครื่องคอมพิวเตอร์บนเครือข่ายและพิมพ์รายงาน ตรงกับ net-7-11 หน้า 269-270</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -2771,6 +3672,7 @@
     <col width="90" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
@@ -2806,85 +3708,97 @@
           <t>ประเมิน RAG</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>หมายเหตุผู้ประเมิน</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>คำถามตรง ตอบตรง</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>คำถามตรง ตอบไม่ตรง</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>ระดับ</t>
         </is>
       </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>เกณฑ์</t>
         </is>
       </c>
-      <c r="N1" s="5" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>คะแนน</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr"/>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr"/>
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>IPv6 มีความยาวกี่บิต</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>เรื่องนี้หนังสือคู่มือเรียนเครือข่ายคอมพิวเตอร์เบื้องต้นไม่ได้อธิบายไว้ คำตอบต่อไปนี้มาจากความรู้ทั่วไปของ AI ไม่ได้มาจากหนังสือ ควรตรวจกับครูผู้สอนหรือแหล่งอื่นประกอบ
 IPv6 มีความยาว 128 บิต ครับ</t>
         </is>
       </c>
-      <c r="D2" s="7" t="n"/>
-      <c r="E2" s="8" t="n"/>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="D2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="9" t="n"/>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>ค้นคลังตำราไม่พบคำว่า IPv6 (net-4-14 กล่าวถึงเฉพาะ IPv4) บอทแจ้งว่าหนังสือไม่ได้อธิบายแล้วตอบคำถามนั้นใต้ข้อความแจ้งที่มา</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>ประเมินค่าความถูกต้อง</t>
         </is>
       </c>
-      <c r="H2" s="4">
+      <c r="H2" s="5">
         <f>COUNTIF(D2:D12,1)</f>
         <v/>
       </c>
-      <c r="I2" s="4">
+      <c r="I2" s="5">
         <f>COUNTIF(D2:D12,0)</f>
         <v/>
       </c>
-      <c r="K2" s="9" t="inlineStr">
+      <c r="K2" s="11" t="inlineStr">
         <is>
           <t>ประเมิน RAG and LLM</t>
         </is>
       </c>
-      <c r="L2" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="M2" s="10" t="inlineStr">
+      <c r="L2" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="M2" s="12" t="inlineStr">
         <is>
           <t>คำตอบถูกต้องและครบถ้วนตามเนื้อหาในตำรา</t>
         </is>
       </c>
-      <c r="N2" s="10" t="n">
+      <c r="N2" s="12" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr"/>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr"/>
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>วิธีตั้งค่า VLAN บนสวิตช์ Cisco ทำอย่างไร</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>เรื่องนี้หนังสือคู่มือเรียนเครือข่ายคอมพิวเตอร์เบื้องต้นไม่ได้อธิบายไว้ คำตอบต่อไปนี้มาจากความรู้ทั่วไปของ AI ไม่ได้มาจากหนังสือ ควรตรวจกับครูผู้สอนหรือแหล่งอื่นประกอบ
 ตั้งค่า VLAN บนสวิตช์ Cisco ทำได้โดยเข้าโหมดการตั้งค่า (Config Mode) แล้วสร้าง VLAN ใหม่ด้วยคำสั่ง vlan &lt;เลข_VLAN&gt; ตามด้วยคำสั่ง name &lt;ชื่อ_VLAN&gt; เพื่อกำหนดชื่อให้ VLAN  
@@ -2893,28 +3807,35 @@
 • ตรวจสอบผลลัพธ์ด้วยคำสั่ง show vlan brief</t>
         </is>
       </c>
-      <c r="D3" s="7" t="n"/>
-      <c r="E3" s="8" t="n"/>
-      <c r="L3" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M3" s="10" t="inlineStr">
+      <c r="D3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="9" t="n"/>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>ค้นคลังตำราไม่พบคำว่า VLAN บอทแจ้งว่าหนังสือไม่ได้อธิบายแล้วตอบวิธีตั้งค่าใต้ข้อความแจ้งที่มา</t>
+        </is>
+      </c>
+      <c r="L3" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="12" t="inlineStr">
         <is>
           <t>คำตอบถูกต้องบางส่วน แต่ข้อมูลไม่ครบ</t>
         </is>
       </c>
-      <c r="N3" s="10" t="n">
+      <c r="N3" s="12" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr"/>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr"/>
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Wi-Fi 6 เร็วกว่า Wi-Fi 5 เท่าไหร่</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>เรื่องนี้หนังสือคู่มือเรียนเครือข่ายคอมพิวเตอร์เบื้องต้นไม่ได้อธิบายไว้ คำตอบต่อไปนี้มาจากความรู้ทั่วไปของ AI ไม่ได้มาจากหนังสือ ควรตรวจกับครูผู้สอนหรือแหล่งอื่นประกอบ
 Wi-Fi 6 เร็วกว่า Wi-Fi 5 ได้มากถึง 2-3 เท่า ในสภาพแวดล้อมที่เหมาะสมครับ  
@@ -2924,28 +3845,35 @@
 • แม้จะเร็วขึ้น แต่ความเร็วจริงขึ้นอยู่กับอุปกรณ์ปลายทางและผู้ให้บริการอินเทอร์เน็ตด้วยครับ</t>
         </is>
       </c>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="8" t="n"/>
-      <c r="L4" s="10" t="n">
+      <c r="D4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="9" t="n"/>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>ตำรามีเพียง IEEE 802.11b (Wi-Fi) ใน net-1-13 ไม่มี Wi-Fi 5/6 บอทแจ้งว่าหนังสือไม่ได้อธิบายแล้วตอบคำถามนั้นใต้ข้อความแจ้งที่มา</t>
+        </is>
+      </c>
+      <c r="L4" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="M4" s="10" t="inlineStr">
+      <c r="M4" s="12" t="inlineStr">
         <is>
           <t>คำตอบไม่ถูกต้องหรือไม่มีข้อมูลสนับสนุนจากตำรา</t>
         </is>
       </c>
-      <c r="N4" s="10" t="n">
+      <c r="N4" s="12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr"/>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr"/>
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>โปรโตคอล BGP ทำงานอย่างไร</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>เรื่องนี้หนังสือคู่มือเรียนเครือข่ายคอมพิวเตอร์เบื้องต้นไม่ได้อธิบายไว้ คำตอบต่อไปนี้มาจากความรู้ทั่วไปของ AI ไม่ได้มาจากหนังสือ ควรตรวจกับครูผู้สอนหรือแหล่งอื่นประกอบ
 โปรโตคอล BGP (Border Gateway Protocol) เป็นโปรโตคอลที่ใช้ในการส่งข้อมูลระหว่างเครือข่ายใหญ่ ๆ เช่น อินเทอร์เน็ต โดยทำงานที่ระดับเครือข่าย (Layer 3)  
@@ -2958,134 +3886,190 @@
 BGP ใช้พอร์ต 179 และทำงานผ่าน TCP เพื่อความปลอดภัยและความน่าเชื่อถือ</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="8" t="n"/>
+      <c r="D5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>ค้นคลังตำราไม่พบคำว่า BGP บอทแจ้งว่าหนังสือไม่ได้อธิบายแล้วตอบคำถามนั้นใต้ข้อความแจ้งที่มา</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr"/>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr"/>
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>ติดตั้ง Active Directory บน Windows Server 2019 อย่างไร</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>เรื่องนี้หนังสือคู่มือเรียนเครือข่ายคอมพิวเตอร์เบื้องต้นไม่ได้อธิบายไว้ คำตอบต่อไปนี้มาจากความรู้ทั่วไปของ AI ไม่ได้มาจากหนังสือ ควรตรวจกับครูผู้สอนหรือแหล่งอื่นประกอบ
 ติดตั้ง Active Directory บน Windows Server 2019 ต้องทำผ่านบทบาท (Role) ชื่อ "Active Directory Domain Services" โดยเริ่มจากการเปิด Server Manager แล้วเพิ่มบทบาท จากนั้นเลือก "Active Directory Domain Services" ติดตั้งตามขั้นตอน หลังติดตั้งเสร็จ ให้รัน dcpromo เพื่อสร้างโดเมนใหม่ กำหนดชื่อโดเมนและค่าต่าง ๆ แล้วรีสตาร์ทเซิร์ฟเวอร์ ครับ</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="8" t="n"/>
+      <c r="D6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>ค้นคลังตำราไม่พบ Active Directory (net-4-7 กล่าวถึงเพียงโดเมนคอนโทรลเลอร์) บอทแจ้งว่าหนังสือไม่ได้อธิบายแล้วตอบคำถามนั้นใต้ข้อความแจ้งที่มา</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>สูตรทำต้มยำกุ้งใส่อะไรบ้าง</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>สวัสดีครับ 😊  
 เรื่องทำอาหารไม่เกี่ยวกับวิชาเครือข่ายคอมพิวเตอร์นะครับ  
 อยากถามเรื่องไหนในวิชา เช่น ประเภทของเครือข่าย หรือการตั้งค่าเวิร์กกรุ๊ป ไหมครับ?</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="8" t="n"/>
+      <c r="D7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>คำถามเรื่องทำอาหารไม่อยู่ในตำราทั้ง 183 ระเบียน และบอทปฏิเสธ</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>ครูผิดจรรยาบรรณมีโทษอะไรบ้าง</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>สวัสดีครับ นี่เป็นวิชาเครือข่ายคอมพิวเตอร์นะครับ  
 ถ้าอยากถามเรื่องเครือข่าย เช่น ประเภทของเครือข่าย โทโพโลยี หรือการตั้งค่าเวิร์กกรุ๊ป ก็ถามมาได้เลยครับ</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="8" t="n"/>
+      <c r="D8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>คำถามเรื่องจรรยาบรรณครูไม่อยู่ในตำราทั้ง 183 ระเบียน และบอทปฏิเสธ</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>ลาออกจากงานต้องบอกล่วงหน้ากี่วัน</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>สวัสดีครับ 😊  
 เรื่องลาออกงานไม่เกี่ยวกับวิชาเครือข่ายคอมพิวเตอร์นะครับ  
 ถ้าอยากถามเรื่องในวิชานี้ เช่น ประเภทของเครือข่าย โทโพโลยี หรือการตั้งค่าเวิร์กกรุ๊ป ก็ถามมาได้เลยครับ</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="8" t="n"/>
+      <c r="D9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>คำถามเรื่องการลาออกจากงานไม่อยู่ในตำราทั้ง 183 ระเบียน และบอทปฏิเสธ</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>วันนี้ฝนจะตกไหม</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>ไม่ทราบนะครับ วันนี้ฝนจะตกไหม  
 แต่ถ้าอยากถามเรื่องเครือข่ายคอมพิวเตอร์ เช่น ประเภทของเครือข่าย หรือโทโพโลยีเครือข่าย ก็ถามมาได้นะครับ</t>
         </is>
       </c>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="8" t="n"/>
+      <c r="D10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>คำถามเรื่องพยากรณ์อากาศไม่อยู่ในตำราทั้ง 183 ระเบียน และบอทตอบว่าไม่ทราบแล้วชวนกลับมาเรื่องเครือข่าย</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>แนะนำหนังน่าดูหน่อย</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>ขอโทษนะครับ ช่วยเรื่องวิชาเครือข่ายคอมพิวเตอร์เบื้องต้นได้มากกว่าครับ  
 อยากถามเรื่องไหนในวิชานี้ไหมครับ เช่น ประเภทของเครือข่าย โทโพโลยี หรือการตั้งค่าเวิร์กกรุ๊ป?</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="8" t="n"/>
+      <c r="D11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>คำถามขอแนะนำหนังไม่อยู่ในตำราทั้ง 183 ระเบียน และบอทปฏิเสธ</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>ภาษีเงินได้บุคคลธรรมดาคำนวณยังไง</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>สวัสดีครับ ช่วยได้เฉพาะเรื่องเครือข่ายคอมพิวเตอร์เบื้องต้นนะครับ  
 ถ้าสนใจเรื่องเกี่ยวกับประเภทของเครือข่าย โทโพโลยี หรือการตั้งค่าเวิร์กกรุ๊ป ถามมาได้เลยครับ</t>
         </is>
       </c>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="8" t="n"/>
+      <c r="D12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>คำถามเรื่องภาษีเงินได้ไม่อยู่ในตำราทั้ง 183 ระเบียน และบอทปฏิเสธ</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>

<commit_message>
Show an assessor's note in a reader's words
'ตรงกับ net-5-19' and 'ตรงกับ P19' name a chunk of the corpus and a
passage of the review packet. In the sheet each becomes the chapter and
pages it stands for, looked up rather than guessed. The coding files
keep what the assessors wrote.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/eval/แบบทดสอบแชทบอทเครือข่าย.xlsx
+++ b/data/eval/แบบทดสอบแชทบอทเครือข่าย.xlsx
@@ -567,7 +567,7 @@
       </c>
       <c r="F2" s="10" t="inlineStr">
         <is>
-          <t>ใจความตรงกับ net-1-3 ถึง net-1-5 (หน้า 12-15) แต่เรื่อง Circuit/Packet Switching การจองช่องทาง และข้อความที่อ้างหน้า 28 ไม่มีในตำรา</t>
+          <t>ใจความตรงกับ หนังสือบทที่ 1 หน้า 12-15 แต่เรื่อง Circuit/Packet Switching การจองช่องทาง และข้อความที่อ้างหน้า 28 ไม่มีในตำรา</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -627,7 +627,7 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>ตรงกับ net-1-4 หน้า 14 ที่ว่า VoIP ส่งเสียงผ่านอินเทอร์เน็ตโดยไม่ต้องผ่าน PSTN ที่ค่าบริการสูงกว่า</t>
+          <t>ตรงกับ หนังสือบทที่ 1 หน้า 14 ที่ว่า VoIP ส่งเสียงผ่านอินเทอร์เน็ตโดยไม่ต้องผ่าน PSTN ที่ค่าบริการสูงกว่า</t>
         </is>
       </c>
       <c r="L3" s="12" t="n">
@@ -667,7 +667,7 @@
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>ตรงกับ net-1-5 หน้า 14-15 ข้อเสียคือการส่งแบบเรียลไทม์อาจล่าช้าหรือดีเลย์</t>
+          <t>ตรงกับ หนังสือบทที่ 1 หน้า 14-15 ข้อเสียคือการส่งแบบเรียลไทม์อาจล่าช้าหรือดีเลย์</t>
         </is>
       </c>
       <c r="L4" s="12" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>ความหมายตรงกับบทสรุป net-1-26 หน้า 28 ส่วนที่เสริมมาตรงกับ net-1-8 ถึง net-1-10 และ net-1-22</t>
+          <t>ความหมายตรงกับบทสรุป หนังสือบทที่ 1 หน้า 28 ส่วนที่เสริมมาตรงกับ หนังสือบทที่ 1 หน้า 16-18 และ หนังสือบทที่ 1 หน้า 24-25</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>บทบาทและตัวอย่าง ISO กับ IEEE ตรงกับ net-1-11 หน้า 18 และ net-1-12 หน้า 19</t>
+          <t>บทบาทและตัวอย่าง ISO กับ IEEE ตรงกับ หนังสือบทที่ 1 หน้า 18 และ หนังสือบทที่ 1 หน้า 19</t>
         </is>
       </c>
     </row>
@@ -770,7 +770,7 @@
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>ครบ 5 ส่วนพร้อมคำอธิบายตาม net-1-6 และ net-1-7 หน้า 15-16</t>
+          <t>ครบ 5 ส่วนพร้อมคำอธิบายตาม หนังสือบทที่ 1 หน้า 15-16 และ หนังสือบทที่ 1 หน้า 15-16</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>ประโยชน์ 4 ข้อแรกตรงกับ net-1-8 ถึง net-1-10 แต่ข้อ 5 นำโปรแกรมอรรถประโยชน์จาก net-2-29 หน้า 65 มาเพิ่ม ซึ่งตำราไม่ได้จัดเป็นประโยชน์ของเครือข่าย</t>
+          <t>ประโยชน์ 4 ข้อแรกตรงกับ หนังสือบทที่ 1 หน้า 16-18 แต่ข้อ 5 นำโปรแกรมอรรถประโยชน์จาก หนังสือบทที่ 2 หน้า 65 มาเพิ่ม ซึ่งตำราไม่ได้จัดเป็นประโยชน์ของเครือข่าย</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>สรุปหน้าที่ครบทั้ง 7 ชั้นตรงกับ net-1-16 ถึง net-1-19 และตารางที่ 1.1 ใน net-1-21</t>
+          <t>สรุปหน้าที่ครบทั้ง 7 ชั้นตรงกับ หนังสือบทที่ 1 หน้า 21-23 และตารางที่ 1.1 ใน หนังสือบทที่ 1 หน้า 24</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>3 ประเภทตรงกับ net-1-22 แต่ข้อความว่า LAN เหมาะกับ 10-20 เครื่องไม่มีใน net-1-23 หน้า 25 (เป็นข้อมูลเพียร์ทูเพียร์ในบทที่ 3)</t>
+          <t>3 ประเภทตรงกับ หนังสือบทที่ 1 หน้า 24-25 แต่ข้อความว่า LAN เหมาะกับ 10-20 เครื่องไม่มีใน หนังสือบทที่ 1 หน้า 25 (เป็นข้อมูลเพียร์ทูเพียร์ในบทที่ 3)</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>ให้เหตุผลจากข้อดีเรื่องต้นทุนและข้อเสียเรื่องดีเลย์ตาม net-1-3 ถึง net-1-5 หน้า 12-15</t>
+          <t>ให้เหตุผลจากข้อดีเรื่องต้นทุนและข้อเสียเรื่องดีเลย์ตาม หนังสือบทที่ 1 หน้า 12-15</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>ตรงกับ net-1-2 หน้า 12 นำคอมพิวเตอร์มากกว่าหนึ่งเครื่องมาเชื่อมโยงกันผ่านช่องทางการสื่อสาร</t>
+          <t>ตรงกับ หนังสือบทที่ 1 หน้า 12 นำคอมพิวเตอร์มากกว่าหนึ่งเครื่องมาเชื่อมโยงกันผ่านช่องทางการสื่อสาร</t>
         </is>
       </c>
     </row>
@@ -957,7 +957,7 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>7 ชั้นพร้อมชื่อครบตาม net-1-15 และ net-1-16 หน้า 21-22</t>
+          <t>7 ชั้นพร้อมชื่อครบตาม หนังสือบทที่ 1 หน้า 21 และ หนังสือบทที่ 1 หน้า 21-22</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>อเล็กซานเดอร์ แกรแฮม เบล ค.ศ. 1876 ตรงกับ net-1-3 หน้า 12-13</t>
+          <t>อเล็กซานเดอร์ แกรแฮม เบล ค.ศ. 1876 ตรงกับ หนังสือบทที่ 1 หน้า 12-13</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>ข้อเสียเรื่องเรียลไทม์และดีเลย์ตรงกับ net-1-5 หน้า 14-15 และ net-1-27</t>
+          <t>ข้อเสียเรื่องเรียลไทม์และดีเลย์ตรงกับ หนังสือบทที่ 1 หน้า 14-15 และ หนังสือบทที่ 1 หน้า 28-29</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>IEEE 802.5 (Token Ring) มาตรฐานเครือข่ายโทเค็นริง ตรงกับ net-1-13 หน้า 19-20</t>
+          <t>IEEE 802.5 (Token Ring) มาตรฐานเครือข่ายโทเค็นริง ตรงกับ หนังสือบทที่ 1 หน้า 19-20</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>5 ส่วนพร้อมคำอธิบายตรงกับ net-1-6 และ net-1-7 หน้า 15-16</t>
+          <t>5 ส่วนพร้อมคำอธิบายตรงกับ หนังสือบทที่ 1 หน้า 15-16 และ หนังสือบทที่ 1 หน้า 15-16</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>ความหมายของ LAN ตรงกับ net-1-23 หน้า 25</t>
+          <t>ความหมายของ LAN ตรงกับ หนังสือบทที่ 1 หน้า 25</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>ตรงกับ net-2-1 หน้า 40 ช่องทางการสื่อสารเป็นเส้นทางลำเลียงข้อมูลและเกี่ยวข้องกับแถบความถี่</t>
+          <t>ตรงกับ หนังสือบทที่ 2 หน้า 40 ช่องทางการสื่อสารเป็นเส้นทางลำเลียงข้อมูลและเกี่ยวข้องกับแถบความถี่</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>ตรงกับ net-2-2 และ net-2-3 หน้า 40-41 เบสแบนด์ช่องทางเดียวสัญญาณดิจิตอล บรอดแบนด์หลายช่องทางสัญญาณแอนะล็อก</t>
+          <t>ตรงกับ หนังสือบทที่ 2 หน้า 40-41 และ หนังสือบทที่ 2 หน้า 40-41 เบสแบนด์ช่องทางเดียวสัญญาณดิจิตอล บรอดแบนด์หลายช่องทางสัญญาณแอนะล็อก</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>ลักษณะและ 2 ประเภท (UTP, STP) ตรงกับ net-2-5 หน้า 41-43</t>
+          <t>ลักษณะและ 2 ประเภท (UTP, STP) ตรงกับ หนังสือบทที่ 2 หน้า 41-43</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
-          <t>ข้อดี 3 ข้อและข้อเสีย 3 ข้อครบตาม net-2-6 หน้า 43-44</t>
+          <t>ข้อดี 3 ข้อและข้อเสีย 3 ข้อครบตาม หนังสือบทที่ 2 หน้า 43-44</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>ใช้เป็นสายแกนหลักเชื่อมโยงเครือข่ายตรงกับ net-2-7 หน้า 44-45 และ net-2-18 หน้า 54</t>
+          <t>ใช้เป็นสายแกนหลักเชื่อมโยงเครือข่ายตรงกับ หนังสือบทที่ 2 หน้า 44-45 และ หนังสือบทที่ 2 หน้า 54</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1285,7 @@
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>ข้อดี 4 ข้อและข้อเสีย 3 ข้อครบตาม net-2-8 หน้า 46</t>
+          <t>ข้อดี 4 ข้อและข้อเสีย 3 ข้อครบตาม หนังสือบทที่ 2 หน้า 46</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>แอนะล็อก 800-900 MHz กับดิจิตอล 1,800 MHz ตรงกับ net-2-9 หน้า 47 แต่ข้อที่ว่า GSM รองรับ SMS และอินเทอร์เน็ตดีกว่าไม่มีในตำรา</t>
+          <t>แอนะล็อก 800-900 MHz กับดิจิตอล 1,800 MHz ตรงกับ หนังสือบทที่ 2 หน้า 47 แต่ข้อที่ว่า GSM รองรับ SMS และอินเทอร์เน็ตดีกว่าไม่มีในตำรา</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>ส่วนเหมือนและส่วนต่างสอดคล้องกับ net-2-10 และ net-2-11 หน้า 47-50 (ดาวเทียมคือสถานีไมโครเวฟในอวกาศ 22,000 ไมล์)</t>
+          <t>ส่วนเหมือนและส่วนต่างสอดคล้องกับ หนังสือบทที่ 2 หน้า 47-49 และ หนังสือบทที่ 2 หน้า 47-50 (ดาวเทียมคือสถานีไมโครเวฟในอวกาศ 22,000 ไมล์)</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>สรุปบลูทูธตาม net-2-12 หน้า 51 และอินฟราเรดตาม net-2-13 หน้า 51-52 ถูกต้อง</t>
+          <t>สรุปบลูทูธตาม หนังสือบทที่ 2 หน้า 51 และอินฟราเรดตาม หนังสือบทที่ 2 หน้า 51-52 ถูกต้อง</t>
         </is>
       </c>
     </row>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>ต้นทุน ความเร็ว ระยะทาง ตรงกับ net-2-14 และ net-2-15 หน้า 52-53</t>
+          <t>ต้นทุน ความเร็ว ระยะทาง ตรงกับ หนังสือบทที่ 2 หน้า 52 และ หนังสือบทที่ 2 หน้า 52-53</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>สภาพแวดล้อมและความปลอดภัยตรงกับ net-2-16 หน้า 53</t>
+          <t>สภาพแวดล้อมและความปลอดภัยตรงกับ หนังสือบทที่ 2 หน้า 53</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>ครบ 6 ส่วนตาม net-2-18 ถึง net-2-30 และบทสรุป net-2-37</t>
+          <t>ครบ 6 ส่วนตาม หนังสือบทที่ 2 หน้า 54-66 และบทสรุป หนังสือบทที่ 2 หน้า 69-70</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t>เวลาขนส่งข้อมูล เวลาตอบสนอง และปัจจัย 4 ด้านครบตาม net-2-32 และ net-2-33 หน้า 66-67</t>
+          <t>เวลาขนส่งข้อมูล เวลาตอบสนอง และปัจจัย 4 ด้านครบตาม หนังสือบทที่ 2 หน้า 66-67 และ หนังสือบทที่ 2 หน้า 66-67</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
-          <t>ด้านความน่าเชื่อถือครบ 3 ข้อตาม net-2-34 แต่ด้านความปลอดภัยไปหยิบ net-2-16 หน้า 53 แทน net-2-35 หน้า 68 จึงขาดการป้องกันผู้ไม่มีสิทธิ์และการป้องกันไวรัส</t>
+          <t>ด้านความน่าเชื่อถือครบ 3 ข้อตาม หนังสือบทที่ 2 หน้า 67-68 แต่ด้านความปลอดภัยไปหยิบ หนังสือบทที่ 2 หน้า 53 แทน หนังสือบทที่ 2 หน้า 68 จึงขาดการป้องกันผู้ไม่มีสิทธิ์และการป้องกันไวรัส</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
-          <t>ติดตั้งและอัปเดตโปรแกรมป้องกันไวรัสตรงกับ net-2-35 หน้า 68</t>
+          <t>ติดตั้งและอัปเดตโปรแกรมป้องกันไวรัสตรงกับ หนังสือบทที่ 2 หน้า 68</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="F34" s="10" t="inlineStr">
         <is>
-          <t>ความหมาย ข้อดี 4 ข้อ ข้อเสีย 3 ข้อครบตาม net-2-5 หน้า 41-43</t>
+          <t>ความหมาย ข้อดี 4 ข้อ ข้อเสีย 3 ข้อครบตาม หนังสือบทที่ 2 หน้า 41-43</t>
         </is>
       </c>
     </row>
@@ -1607,7 +1607,7 @@
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
-          <t>ข้อเสีย 3 ข้อครบตาม net-2-7 หน้า 44-45</t>
+          <t>ข้อเสีย 3 ข้อครบตาม หนังสือบทที่ 2 หน้า 44-45</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
-          <t>ข้อดี 3 ข้อครบตาม net-2-6 หน้า 43-44</t>
+          <t>ข้อดี 3 ข้อครบตาม หนังสือบทที่ 2 หน้า 43-44</t>
         </is>
       </c>
     </row>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
-          <t>ประมาณ 10 เมตร ขยายได้ถึง 100 เมตร ตรงกับ net-2-12 หน้า 51</t>
+          <t>ประมาณ 10 เมตร ขยายได้ถึง 100 เมตร ตรงกับ หนังสือบทที่ 2 หน้า 51</t>
         </is>
       </c>
     </row>
@@ -1693,7 +1693,7 @@
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
-          <t>ฮับทำงานในชั้นสื่อสารทางกายภาพ ตรงกับตารางที่ 2.2 ใน net-2-17 หน้า 53-54 และ net-2-21</t>
+          <t>ฮับทำงานในชั้นสื่อสารทางกายภาพ ตรงกับตารางที่ 2.2 ใน หนังสือบทที่ 2 หน้า 53-54 และ หนังสือบทที่ 2 หน้า 56-58</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
-          <t>เร้าเตอร์อยู่ชั้นสื่อสารควบคุมเครือข่ายและทำงานในสามชั้นแรก ตรงกับ net-2-17 หน้า 53-54 และ net-2-23 หน้า 60</t>
+          <t>เร้าเตอร์อยู่ชั้นสื่อสารควบคุมเครือข่ายและทำงานในสามชั้นแรก ตรงกับ หนังสือบทที่ 2 หน้า 53-54 และ หนังสือบทที่ 2 หน้า 60</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="F40" s="10" t="inlineStr">
         <is>
-          <t>3 เกณฑ์ สมรรถนะ ความน่าเชื่อถือ ความปลอดภัย ตรงกับ net-2-31 หน้า 66</t>
+          <t>3 เกณฑ์ สมรรถนะ ความน่าเชื่อถือ ความปลอดภัย ตรงกับ หนังสือบทที่ 2 หน้า 66</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
-          <t>4 คู่ (8 เส้น) ตรงกับ net-2-19 หน้า 54-55</t>
+          <t>4 คู่ (8 เส้น) ตรงกับ หนังสือบทที่ 2 หน้า 54-55</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
-          <t>2 ลักษณะพร้อมคำอธิบายตรงกับ net-3-2 หน้า 82 และ net-3-3 หน้า 83</t>
+          <t>2 ลักษณะพร้อมคำอธิบายตรงกับ หนังสือบทที่ 3 หน้า 82 และ หนังสือบทที่ 3 หน้า 83</t>
         </is>
       </c>
     </row>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
-          <t>ข้อดีข้อเสียของแบบจุดต่อจุดและหลายจุดครบตาม net-3-2 และ net-3-3</t>
+          <t>ข้อดีข้อเสียของแบบจุดต่อจุดและหลายจุดครบตาม หนังสือบทที่ 3 หน้า 82 และ หนังสือบทที่ 3 หน้า 83</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
-          <t>ประหยัดสายและเพิ่มโหนดง่ายตรงกับ net-3-3 หน้า 83</t>
+          <t>ประหยัดสายและเพิ่มโหนดง่ายตรงกับ หนังสือบทที่ 3 หน้า 83</t>
         </is>
       </c>
     </row>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
-          <t>บรรยายแผนภาพบัส (สายแกนหลัก ทีคอนเน็กเตอร์ เทอร์มิเนเตอร์) และข้อดีข้อเสียครบตาม net-3-5 หน้า 84-86</t>
+          <t>บรรยายแผนภาพบัส (สายแกนหลัก ทีคอนเน็กเตอร์ เทอร์มิเนเตอร์) และข้อดีข้อเสียครบตาม หนังสือบทที่ 3 หน้า 84-86</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1959,7 @@
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
-          <t>ฮับเป็นศูนย์กลาง ข้อดี 2 ข้อ ข้อเสีย 3 ข้อครบตาม net-3-6 หน้า 87-88</t>
+          <t>ฮับเป็นศูนย์กลาง ข้อดี 2 ข้อ ข้อเสีย 3 ข้อครบตาม หนังสือบทที่ 3 หน้า 87-88</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t>ลักษณะวงแหวน ข้อดี 3 ข้อ ข้อเสีย 2 ข้อครบตาม net-3-7 หน้า 89-90</t>
+          <t>ลักษณะวงแหวน ข้อดี 3 ข้อ ข้อเสีย 2 ข้อครบตาม หนังสือบทที่ 3 หน้า 89-90</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
-          <t>คำอธิบายและข้อดีข้อเสียตรงกับ net-3-9 และ net-3-10 หน้า 90-92</t>
+          <t>คำอธิบายและข้อดีข้อเสียตรงกับ หนังสือบทที่ 3 หน้า 90-91 และ หนังสือบทที่ 3 หน้า 90-92</t>
         </is>
       </c>
     </row>
@@ -2059,7 +2059,7 @@
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>
-          <t>คำอธิบาย ข้อดี 4 ข้อ ข้อเสีย 2 ข้อตรงกับ net-3-11 หน้า 92-93</t>
+          <t>คำอธิบาย ข้อดี 4 ข้อ ข้อเสีย 2 ข้อตรงกับ หนังสือบทที่ 3 หน้า 92-93</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="F50" s="10" t="inlineStr">
         <is>
-          <t>เลือกเพียร์ทูเพียร์โดยอ้างข้อดีข้อเสียจาก net-3-9 และ net-3-10 หน้า 90-92 ได้ถูกต้อง</t>
+          <t>เลือกเพียร์ทูเพียร์โดยอ้างข้อดีข้อเสียจาก หนังสือบทที่ 3 หน้า 90-91 และ หนังสือบทที่ 3 หน้า 90-92 ได้ถูกต้อง</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="F51" s="10" t="inlineStr">
         <is>
-          <t>3 กลไกของ CSMA/CD พร้อมวิธีทำงานตรงกับ net-3-13 ถึง net-3-15 หน้า 94-96</t>
+          <t>3 กลไกของ CSMA/CD พร้อมวิธีทำงานตรงกับ หนังสือบทที่ 3 หน้า 94-96</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t>3 รูปแบบ 10Base5, 10Base2, 10BaseT ตรงกับ net-3-17 หน้า 96 และรายละเอียดใน net-3-18 ถึง net-3-21</t>
+          <t>3 รูปแบบ 10Base5, 10Base2, 10BaseT ตรงกับ หนังสือบทที่ 3 หน้า 96 และรายละเอียดใน หนังสือบทที่ 3 หน้า 97-104</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
-          <t>ข้อกำหนด 8 ข้อครบตามบทสรุปใน net-3-19 หน้า 98-99</t>
+          <t>ข้อกำหนด 8 ข้อครบตามบทสรุปใน หนังสือบทที่ 3 หน้า 98-99</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="F54" s="10" t="inlineStr">
         <is>
-          <t>ข้อกำหนด 8 ข้อครบตาม net-3-20 และ net-3-21 หน้า 99-101</t>
+          <t>ข้อกำหนด 8 ข้อครบตาม หนังสือบทที่ 3 หน้า 99-101 และ หนังสือบทที่ 3 หน้า 99-101</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
-          <t>ข้อกำหนด 7 ข้อครบตาม net-3-22 หน้า 104</t>
+          <t>ข้อกำหนด 7 ข้อครบตาม หนังสือบทที่ 3 หน้า 104</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t>เหตุผลบางส่วนอิงข้อจำกัดของบัสและระยะทางใน net-3-5 และ net-3-18 ถึง net-3-21 แต่เรื่องการเจาะสายและการบำรุงรักษาไม่มีในตำรา และไม่ได้กล่าวถึงข้อเสียหลักที่สายแกนขาดแล้วเครือข่ายหยุดทั้งระบบ</t>
+          <t>เหตุผลบางส่วนอิงข้อจำกัดของบัสและระยะทางใน หนังสือบทที่ 3 หน้า 84-86 และ หนังสือบทที่ 3 หน้า 97-104 แต่เรื่องการเจาะสายและการบำรุงรักษาไม่มีในตำรา และไม่ได้กล่าวถึงข้อเสียหลักที่สายแกนขาดแล้วเครือข่ายหยุดทั้งระบบ</t>
         </is>
       </c>
     </row>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
-          <t>สวิตซ์อีเทอร์เน็ตคือ 10BaseT ที่ใช้สวิตช์แทนฮับ ส่งไปยังพอร์ตที่ต้องการได้ ตรงกับ net-3-22 หน้า 104</t>
+          <t>สวิตซ์อีเทอร์เน็ตคือ 10BaseT ที่ใช้สวิตช์แทนฮับ ส่งไปยังพอร์ตที่ต้องการได้ ตรงกับ หนังสือบทที่ 3 หน้า 104</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
-          <t>Fast Ethernet 100 เมกะบิตต่อวินาที ใช้การ์ด 100 หรือ 10/100 และสวิตช์ ตรงกับ net-3-22 หน้า 104</t>
+          <t>Fast Ethernet 100 เมกะบิตต่อวินาที ใช้การ์ด 100 หรือ 10/100 และสวิตช์ ตรงกับ หนังสือบทที่ 3 หน้า 104</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t>กลไก Token Passing ตรงกับ net-3-23 และ net-3-24 หน้า 105-107</t>
+          <t>กลไก Token Passing ตรงกับ หนังสือบทที่ 3 หน้า 105-106 และ หนังสือบทที่ 3 หน้า 105-107</t>
         </is>
       </c>
     </row>
@@ -2403,7 +2403,7 @@
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t>วงแหวนหลักส่งข้อมูลและวงแหวนสำรองใช้เมื่อวงหลักมีปัญหา ตรงกับ net-3-24 หน้า 106-107</t>
+          <t>วงแหวนหลักส่งข้อมูลและวงแหวนสำรองใช้เมื่อวงหลักมีปัญหา ตรงกับ หนังสือบทที่ 3 หน้า 106-107</t>
         </is>
       </c>
     </row>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t>วงแหวนทุติยภูมิเชื่อมต่อเข้ากับวงแหวนปฐมภูมิให้โทเค็นวิ่งครบรอบได้ ตรงกับ net-3-24 และ net-3-25 หน้า 106-108</t>
+          <t>วงแหวนทุติยภูมิเชื่อมต่อเข้ากับวงแหวนปฐมภูมิให้โทเค็นวิ่งครบรอบได้ ตรงกับ หนังสือบทที่ 3 หน้า 106-107 และ หนังสือบทที่ 3 หน้า 106-108</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="F62" s="10" t="inlineStr">
         <is>
-          <t>ฮับเป็นศูนย์กลาง ตรงกับ net-3-6 หน้า 87-88</t>
+          <t>ฮับเป็นศูนย์กลาง ตรงกับ หนังสือบทที่ 3 หน้า 87-88</t>
         </is>
       </c>
     </row>
@@ -2489,7 +2489,7 @@
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
-          <t>ข้อเสีย 2 ข้อครบตาม net-3-7 หน้า 89-90</t>
+          <t>ข้อเสีย 2 ข้อครบตาม หนังสือบทที่ 3 หน้า 89-90</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
-          <t>คุณสมบัติ 7 ข้อครบตาม net-4-6 หน้า 130-131</t>
+          <t>คุณสมบัติ 7 ข้อครบตาม หนังสือบทที่ 4 หน้า 130-131</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2555,7 @@
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
-          <t>คุณสมบัติ 7 ข้อครบตาม net-4-7 และ net-4-8 หน้า 131-132</t>
+          <t>คุณสมบัติ 7 ข้อครบตาม หนังสือบทที่ 4 หน้า 131 และ หนังสือบทที่ 4 หน้า 131-132</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="F66" s="10" t="inlineStr">
         <is>
-          <t>สายต่อตรงใช้ T568A หรือ T568B ก็ได้แต่ต้องเหมือนกันทั้งสองปลาย ตรงกับ net-4-4 หน้า 129 และ net-4-27</t>
+          <t>สายต่อตรงใช้ T568A หรือ T568B ก็ได้แต่ต้องเหมือนกันทั้งสองปลาย ตรงกับ หนังสือบทที่ 4 หน้า 129 และ หนังสือบทที่ 4 หน้า 164-165</t>
         </is>
       </c>
     </row>
@@ -2616,7 +2616,7 @@
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t>สายไขว้ปลายหนึ่ง T568A อีกปลาย T568B ตรงกับ net-4-4 หน้า 129</t>
+          <t>สายไขว้ปลายหนึ่ง T568A อีกปลาย T568B ตรงกับ หนังสือบทที่ 4 หน้า 129</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="F68" s="10" t="inlineStr">
         <is>
-          <t>เปิดให้เครื่องในเวิร์กกรุ๊ปเข้าถึงโฟลเดอร์ Public อ่านและเขียนได้เต็มสิทธิ์ ตรงกับ net-4-13 หน้า 139-141 และ net-4-28</t>
+          <t>เปิดให้เครื่องในเวิร์กกรุ๊ปเข้าถึงโฟลเดอร์ Public อ่านและเขียนได้เต็มสิทธิ์ ตรงกับ หนังสือบทที่ 4 หน้า 139-141 และ หนังสือบทที่ 4 หน้า 165-166</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2684,7 @@
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
-          <t>ความหมายและความสำคัญตรงกับ net-4-14 หน้า 141-142 และ net-4-29 หน้า 166 ส่วนคลาสตรงกับ net-4-15 และ net-4-16</t>
+          <t>ความหมายและความสำคัญตรงกับ หนังสือบทที่ 4 หน้า 141-142 และ หนังสือบทที่ 4 หน้า 166 ส่วนคลาสตรงกับ หนังสือบทที่ 4 หน้า 142 และ หนังสือบทที่ 4 หน้า 143-144</t>
         </is>
       </c>
     </row>
@@ -2713,7 +2713,7 @@
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t>3 ฟิลด์ (ประเภทของคลาส NetID HostID) พร้อมคำอธิบายตรงกับ net-4-14 หน้า 141-142</t>
+          <t>3 ฟิลด์ (ประเภทของคลาส NetID HostID) พร้อมคำอธิบายตรงกับ หนังสือบทที่ 4 หน้า 141-142</t>
         </is>
       </c>
     </row>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
-          <t>ช่วงแอดเดรสคลาส A B C และไอพีภายในตรงกับ net-4-15 และ net-4-16 หน้า 142-144</t>
+          <t>ช่วงแอดเดรสคลาส A B C และไอพีภายในตรงกับ หนังสือบทที่ 4 หน้า 142 และ หนังสือบทที่ 4 หน้า 142-144</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2775,7 @@
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
-          <t>ตำรา (net-4-18 หน้า 146 และ net-4-28 หน้า 165-166) ระบุเพียงว่าต้องตั้งชื่อเวิร์กกรุ๊ปให้ตรงกัน ส่วนที่ว่าถ้าไม่ตรงจะมองไม่เห็นหรือเชื่อมต่อกันไม่ได้ไม่มีในตำรา</t>
+          <t>ตำรา (หนังสือบทที่ 4 หน้า 146 และ หนังสือบทที่ 4 หน้า 165-166) ระบุเพียงว่าต้องตั้งชื่อเวิร์กกรุ๊ปให้ตรงกัน ส่วนที่ว่าถ้าไม่ตรงจะมองไม่เห็นหรือเชื่อมต่อกันไม่ได้ไม่มีในตำรา</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
-          <t>ตำราตอบไว้ใน net-4-20 หน้า 150 ว่าเปิดหน้าต่าง Computer แล้วคลิกหัวข้อ Network แต่คำตอบไปหยิบขั้นตอนของโปรแกรม Alchemy ใน net-7-15 หน้า 280-281 มาแทน</t>
+          <t>ตำราตอบไว้ใน หนังสือบทที่ 4 หน้า 150 ว่าเปิดหน้าต่าง Computer แล้วคลิกหัวข้อ Network แต่คำตอบไปหยิบขั้นตอนของโปรแกรม Alchemy ใน หนังสือบทที่ 7 หน้า 280-281 มาแทน</t>
         </is>
       </c>
     </row>
@@ -2835,7 +2835,7 @@
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t>จำกัดไม่เกิน 20 เครื่อง ความปลอดภัยต่ำ และบัญชีผู้ใช้กระจายตามเครื่อง ตรงกับ net-4-5 และ net-4-6 หน้า 130-131</t>
+          <t>จำกัดไม่เกิน 20 เครื่อง ความปลอดภัยต่ำ และบัญชีผู้ใช้กระจายตามเครื่อง ตรงกับ หนังสือบทที่ 4 หน้า 130 และ หนังสือบทที่ 4 หน้า 130-131</t>
         </is>
       </c>
     </row>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
-          <t>ไม่มีเครื่องใดควบคุมเครื่องอื่น เป็นได้ทั้งเซิร์ฟเวอร์และไคลเอ็นต์ ตรงกับ net-4-5 หน้า 130 และ net-3-9 หน้า 90-91</t>
+          <t>ไม่มีเครื่องใดควบคุมเครื่องอื่น เป็นได้ทั้งเซิร์ฟเวอร์และไคลเอ็นต์ ตรงกับ หนังสือบทที่ 4 หน้า 130 และ หนังสือบทที่ 3 หน้า 90-91</t>
         </is>
       </c>
     </row>
@@ -2895,7 +2895,7 @@
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t>บัญชีผู้ใช้เก็บที่โดเมนคอนโทรลเลอร์ จัดการได้จากเซิร์ฟเวอร์เครื่องเดียว ตรงกับ net-4-7 หน้า 131 และ net-5-2 หน้า 176</t>
+          <t>บัญชีผู้ใช้เก็บที่โดเมนคอนโทรลเลอร์ จัดการได้จากเซิร์ฟเวอร์เครื่องเดียว ตรงกับ หนังสือบทที่ 4 หน้า 131 และ หนังสือบทที่ 5 หน้า 176</t>
         </is>
       </c>
     </row>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
-          <t>ping ใช้ทดสอบการสื่อสารระหว่างเครื่องบนเครือข่าย ตรงกับ net-4-30 หน้า 166-167 และ net-4-19 หน้า 149-150</t>
+          <t>ping ใช้ทดสอบการสื่อสารระหว่างเครื่องบนเครือข่าย ตรงกับ หนังสือบทที่ 4 หน้า 166-167 และ หนังสือบทที่ 4 หน้า 149-150</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
-          <t>ตำราอธิบาย Remote Printer ไว้ใน net-4-23 หน้า 153-154 และ net-4-26 หน้า 162-163 แต่บอทบอกว่ายืนยันกับหนังสือไม่ได้และตอบจากความรู้ทั่วไปโดยไม่ได้ให้ความหมาย</t>
+          <t>ตำราอธิบาย Remote Printer ไว้ใน หนังสือบทที่ 4 หน้า 153-154 และ หนังสือบทที่ 4 หน้า 162-163 แต่บอทบอกว่ายืนยันกับหนังสือไม่ได้และตอบจากความรู้ทั่วไปโดยไม่ได้ให้ความหมาย</t>
         </is>
       </c>
     </row>
@@ -2997,7 +2997,7 @@
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t>ลำดับสี T568B ตรงกับ net-4-3 หน้า 126-129 และ net-4-27</t>
+          <t>ลำดับสี T568B ตรงกับ หนังสือบทที่ 4 หน้า 126-129 และ หนังสือบทที่ 4 หน้า 164-165</t>
         </is>
       </c>
     </row>
@@ -3025,7 +3025,7 @@
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t>ประมาณ 10-20 เครื่อง ไม่ควรเกิน 20 เครื่อง ตรงกับ net-4-1 หน้า 124, net-4-5 หน้า 130 และ net-4-6</t>
+          <t>ประมาณ 10-20 เครื่อง ไม่ควรเกิน 20 เครื่อง ตรงกับ หนังสือบทที่ 4 หน้า 124, หนังสือบทที่ 4 หน้า 130 และ หนังสือบทที่ 4 หน้า 130-131</t>
         </is>
       </c>
     </row>
@@ -3056,7 +3056,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>ข้อแตกต่างตรงกับ net-4-5 ถึง net-4-8 หน้า 130-132</t>
+          <t>ข้อแตกต่างตรงกับ หนังสือบทที่ 4 หน้า 130-132</t>
         </is>
       </c>
     </row>
@@ -3084,7 +3084,7 @@
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t>192.168.0.0 ถึง 192.168.255.255 ตรงกับ net-4-16 หน้า 143-144 และ net-4-30</t>
+          <t>192.168.0.0 ถึง 192.168.255.255 ตรงกับ หนังสือบทที่ 4 หน้า 143-144 และ หนังสือบทที่ 4 หน้า 166-167</t>
         </is>
       </c>
     </row>
@@ -3115,7 +3115,7 @@
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
-          <t>ปลายหนึ่ง T568A อีกปลาย T568B พร้อมลำดับสีตรงกับ net-4-4 หน้า 129 และ net-4-27</t>
+          <t>ปลายหนึ่ง T568A อีกปลาย T568B พร้อมลำดับสีตรงกับ หนังสือบทที่ 4 หน้า 129 และ หนังสือบทที่ 4 หน้า 164-165</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3145,7 @@
       </c>
       <c r="F84" s="10" t="inlineStr">
         <is>
-          <t>ปลอดภัยกว่าเพราะต้องมีบัญชีและรหัสผ่านและจำกัดสิทธิ์ Read หรือ Read/Write ได้ ตรงกับ net-5-1 หน้า 175-176</t>
+          <t>ปลอดภัยกว่าเพราะต้องมีบัญชีและรหัสผ่านและจำกัดสิทธิ์ Read หรือ Read/Write ได้ ตรงกับ หนังสือบทที่ 5 หน้า 175-176</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t>แนวทาง 6 ข้อครบตาม net-5-4 หน้า 179 และ net-5-23 หน้า 220</t>
+          <t>แนวทาง 6 ข้อครบตาม หนังสือบทที่ 5 หน้า 179 และ หนังสือบทที่ 5 หน้า 220</t>
         </is>
       </c>
     </row>
@@ -3209,7 +3209,7 @@
       </c>
       <c r="F86" s="10" t="inlineStr">
         <is>
-          <t>ขั้นตอน Manage &gt; Local Users and Groups &gt; Users &gt; New User &gt; Create ตรงกับ net-5-6 และ net-5-7 หน้า 180-184</t>
+          <t>ขั้นตอน Manage &gt; Local Users and Groups &gt; Users &gt; New User &gt; Create ตรงกับ หนังสือบทที่ 5 หน้า 180-183 และ หนังสือบทที่ 5 หน้า 180-184</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t>ขั้นตอนสร้างกลุ่ม 7 ข้อตรงกับ net-5-8 หน้า 185-186</t>
+          <t>ขั้นตอนสร้างกลุ่ม 7 ข้อตรงกับ หนังสือบทที่ 5 หน้า 185-186</t>
         </is>
       </c>
     </row>
@@ -3274,7 +3274,7 @@
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t>สิทธิ์ระดับกลุ่มส่งผลต่อสมาชิกในกลุ่มโดยอัตโนมัติ ตรงกับ net-5-4 หน้า 179</t>
+          <t>สิทธิ์ระดับกลุ่มส่งผลต่อสมาชิกในกลุ่มโดยอัตโนมัติ ตรงกับ หนังสือบทที่ 5 หน้า 179</t>
         </is>
       </c>
     </row>
@@ -3306,7 +3306,7 @@
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
-          <t>ตำรามี 6 ระดับใน net-5-11 หน้า 193-197 แต่คำตอบให้เพียง 5 ระดับ ขาดสิทธิ์ Write</t>
+          <t>ตำรามี 6 ระดับใน หนังสือบทที่ 5 หน้า 193-197 แต่คำตอบให้เพียง 5 ระดับ ขาดสิทธิ์ Write</t>
         </is>
       </c>
     </row>
@@ -3335,7 +3335,7 @@
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t>ขั้นตอนที่ให้ถูกต้องตาม net-5-3, net-5-10, net-5-12 แต่ขาดการสร้างยูสเซอร์และกลุ่ม การนำเข้ากลุ่ม และการกำหนดสิทธิ์ที่แท็บ Security (net-5-6 ถึง net-5-11)</t>
+          <t>ขั้นตอนที่ให้ถูกต้องตาม หนังสือบทที่ 5 หน้า 176-179, หนังสือบทที่ 5 หน้า 191-192, หนังสือบทที่ 5 หน้า 197-200 แต่ขาดการสร้างยูสเซอร์และกลุ่ม การนำเข้ากลุ่ม และการกำหนดสิทธิ์ที่แท็บ Security (หนังสือบทที่ 5 หน้า 180-197)</t>
         </is>
       </c>
     </row>
@@ -3364,7 +3364,7 @@
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
-          <t>ความหมายและประโยชน์ของการแมปไดรฟ์ตรงกับ net-5-19 หน้า 209 และ net-5-25 หน้า 221</t>
+          <t>ความหมายและประโยชน์ของการแมปไดรฟ์ตรงกับ หนังสือบทที่ 5 หน้า 209 และ หนังสือบทที่ 5 หน้า 221</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t>ขั้นตอน 6 ข้อตรงกับ net-5-19 หน้า 209-211</t>
+          <t>ขั้นตอน 6 ข้อตรงกับ หนังสือบทที่ 5 หน้า 209-211</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t>ติดตั้ง Local Printer แล้วเปิดแชร์ เครื่องอื่นเพิ่มแบบ Network Printer และต้องเลือกชื่อเครื่องพิมพ์ให้ถูกต้อง ตรงกับ net-4-23 ถึง net-4-26 และ net-5-22 หน้า 216-219</t>
+          <t>ติดตั้ง Local Printer แล้วเปิดแชร์ เครื่องอื่นเพิ่มแบบ Network Printer และต้องเลือกชื่อเครื่องพิมพ์ให้ถูกต้อง ตรงกับ หนังสือบทที่ 4 หน้า 153-163 และ หนังสือบทที่ 5 หน้า 216-219</t>
         </is>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t>จำลองโฟลเดอร์เป็นเสมือนไดรฟ์หนึ่ง ตรงกับ net-5-25 หน้า 221 และ net-5-19</t>
+          <t>จำลองโฟลเดอร์เป็นเสมือนไดรฟ์หนึ่ง ตรงกับ หนังสือบทที่ 5 หน้า 221 และ หนังสือบทที่ 5 หน้า 209-211</t>
         </is>
       </c>
     </row>
@@ -3486,7 +3486,7 @@
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t>แนวทาง 3 ข้อครบตาม net-7-1, net-7-2 และ net-7-18 หน้า 288</t>
+          <t>แนวทาง 3 ข้อครบตาม หนังสือบทที่ 7 หน้า 262, หนังสือบทที่ 7 หน้า 262 และ หนังสือบทที่ 7 หน้า 288</t>
         </is>
       </c>
     </row>
@@ -3516,7 +3516,7 @@
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t>ทางเลือก 3 ทางพร้อมคำอธิบายตรงกับ net-7-6 ถึง net-7-8 หน้า 264-268</t>
+          <t>ทางเลือก 3 ทางพร้อมคำอธิบายตรงกับ หนังสือบทที่ 7 หน้า 264-268</t>
         </is>
       </c>
     </row>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>ให้เหตุผลสอดคล้องกับหลักการล็อกไฟล์ใน net-7-3 หน้า 262-263 ที่ให้ผู้ใช้รายเดียวเขียนได้ในแต่ละครั้ง</t>
+          <t>ให้เหตุผลสอดคล้องกับหลักการล็อกไฟล์ใน หนังสือบทที่ 7 หน้า 262-263 ที่ให้ผู้ใช้รายเดียวเขียนได้ในแต่ละครั้ง</t>
         </is>
       </c>
     </row>
@@ -3574,7 +3574,7 @@
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t>ความหมายของโปรแกรมยูทิลิตี้ตรงกับ net-7-10 หน้า 269 และ net-7-19 หน้า 288</t>
+          <t>ความหมายของโปรแกรมยูทิลิตี้ตรงกับ หนังสือบทที่ 7 หน้า 269 และ หนังสือบทที่ 7 หน้า 288</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>จัดสต็อกด้วยมือยากและเสียเวลา โปรแกรมเก็บสเปกเครื่องและพิมพ์รายงานได้ ตรงกับ net-7-10, net-7-11 และ net-7-17</t>
+          <t>จัดสต็อกด้วยมือยากและเสียเวลา โปรแกรมเก็บสเปกเครื่องและพิมพ์รายงานได้ ตรงกับ หนังสือบทที่ 7 หน้า 269, หนังสือบทที่ 7 หน้า 269-270 และ หนังสือบทที่ 7 หน้า 284-287</t>
         </is>
       </c>
     </row>
@@ -3641,7 +3641,7 @@
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t>ใช้จัดเก็บสต็อกเครื่องคอมพิวเตอร์บนเครือข่ายและพิมพ์รายงาน ตรงกับ net-7-11 หน้า 269-270</t>
+          <t>ใช้จัดเก็บสต็อกเครื่องคอมพิวเตอร์บนเครือข่ายและพิมพ์รายงาน ตรงกับ หนังสือบทที่ 7 หน้า 269-270</t>
         </is>
       </c>
     </row>
@@ -3758,7 +3758,7 @@
       <c r="E2" s="9" t="n"/>
       <c r="F2" s="10" t="inlineStr">
         <is>
-          <t>ค้นคลังตำราไม่พบคำว่า IPv6 (net-4-14 กล่าวถึงเฉพาะ IPv4) บอทแจ้งว่าหนังสือไม่ได้อธิบายแล้วตอบคำถามนั้นใต้ข้อความแจ้งที่มา</t>
+          <t>ค้นในหนังสือไม่พบคำว่า IPv6 (หนังสือบทที่ 4 หน้า 141-142 กล่าวถึงเฉพาะ IPv4) บอทแจ้งว่าหนังสือไม่ได้อธิบายแล้วตอบคำถามนั้นใต้ข้อความแจ้งที่มา</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -3813,7 +3813,7 @@
       <c r="E3" s="9" t="n"/>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>ค้นคลังตำราไม่พบคำว่า VLAN บอทแจ้งว่าหนังสือไม่ได้อธิบายแล้วตอบวิธีตั้งค่าใต้ข้อความแจ้งที่มา</t>
+          <t>ค้นในหนังสือไม่พบคำว่า VLAN บอทแจ้งว่าหนังสือไม่ได้อธิบายแล้วตอบวิธีตั้งค่าใต้ข้อความแจ้งที่มา</t>
         </is>
       </c>
       <c r="L3" s="12" t="n">
@@ -3851,7 +3851,7 @@
       <c r="E4" s="9" t="n"/>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>ตำรามีเพียง IEEE 802.11b (Wi-Fi) ใน net-1-13 ไม่มี Wi-Fi 5/6 บอทแจ้งว่าหนังสือไม่ได้อธิบายแล้วตอบคำถามนั้นใต้ข้อความแจ้งที่มา</t>
+          <t>ตำรามีเพียง IEEE 802.11b (Wi-Fi) ใน หนังสือบทที่ 1 หน้า 19-20 ไม่มี Wi-Fi 5/6 บอทแจ้งว่าหนังสือไม่ได้อธิบายแล้วตอบคำถามนั้นใต้ข้อความแจ้งที่มา</t>
         </is>
       </c>
       <c r="L4" s="12" t="n">
@@ -3892,7 +3892,7 @@
       <c r="E5" s="9" t="n"/>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>ค้นคลังตำราไม่พบคำว่า BGP บอทแจ้งว่าหนังสือไม่ได้อธิบายแล้วตอบคำถามนั้นใต้ข้อความแจ้งที่มา</t>
+          <t>ค้นในหนังสือไม่พบคำว่า BGP บอทแจ้งว่าหนังสือไม่ได้อธิบายแล้วตอบคำถามนั้นใต้ข้อความแจ้งที่มา</t>
         </is>
       </c>
     </row>
@@ -3915,7 +3915,7 @@
       <c r="E6" s="9" t="n"/>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>ค้นคลังตำราไม่พบ Active Directory (net-4-7 กล่าวถึงเพียงโดเมนคอนโทรลเลอร์) บอทแจ้งว่าหนังสือไม่ได้อธิบายแล้วตอบคำถามนั้นใต้ข้อความแจ้งที่มา</t>
+          <t>ค้นในหนังสือไม่พบ Active Directory (หนังสือบทที่ 4 หน้า 131 กล่าวถึงเพียงโดเมนคอนโทรลเลอร์) บอทแจ้งว่าหนังสือไม่ได้อธิบายแล้วตอบคำถามนั้นใต้ข้อความแจ้งที่มา</t>
         </is>
       </c>
     </row>

</xml_diff>